<commit_message>
[ADD] 261015 튜토리얼 추가
</commit_message>
<xml_diff>
--- a/Assets/DB/MMM_DB_Ver.05.xlsx
+++ b/Assets/DB/MMM_DB_Ver.05.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\MoreMustMush\Assets\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64BB3913-FD7D-4A02-AAD7-0D8E3308EAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EBF2F06-1097-4685-9A42-C0AC5C5204CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4500" yWindow="570" windowWidth="18900" windowHeight="13410" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5790" yWindow="1035" windowWidth="18660" windowHeight="13995" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9798" uniqueCount="7731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9846" uniqueCount="7755">
   <si>
     <t>Upgrade_Table</t>
   </si>
@@ -26579,6 +26579,94 @@
   </si>
   <si>
     <t>{0} готово! Поставь на Мировое древо в разделе "Украшение"</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>균사 트리 강화</t>
+  </si>
+  <si>
+    <t>날씨</t>
+  </si>
+  <si>
+    <t>보스 도전 버튼</t>
+  </si>
+  <si>
+    <t>새 기능이 열렸어요: {0}</t>
+  </si>
+  <si>
+    <t>수확기를 잡고 아래로 당겼다 놓으면 버섯을 향해 날아가요!</t>
+  </si>
+  <si>
+    <t>첫 강화를 사 보세요! 밝게 빛나는 노드를 누르세요</t>
+  </si>
+  <si>
+    <t>강해졌어요! 다시 수확하러 가 볼까요?</t>
+  </si>
+  <si>
+    <t>수확하러 가서 첫 스테이지를 마쳐 보세요!</t>
+  </si>
+  <si>
+    <t>Mycelium Tree Upgrades</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>菌糸ツリー強化</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Weather</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>天気</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Boss Challenge Button</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ボス挑戦ボタン</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>New feature unlocked: {0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>新しい機能が解放されました:{0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Grab the Harvester, pull it down, and let go to send it flying at the mushroom!</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>収穫機をつかんで下に引いて離すと、キノコに向かって飛んでいくよ!</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Buy your first upgrade! Tap the glowing node</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>はじめての強化を買ってみよう!光っているノードを押してね</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>You got stronger! Ready to go harvest again?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>強くなったね!もう一度収穫に行こうか?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Go harvest and clear the first stage!</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>収穫に行って、最初のステージをクリアしよう!</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -30704,7 +30792,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H1422"/>
+  <dimension ref="A1:H1430"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="2" max="2" width="12.75" style="2" bestFit="1" customWidth="1"/>
@@ -67396,6 +67484,214 @@
       </c>
       <c r="H1422" s="130" t="s">
         <v>7717</v>
+      </c>
+    </row>
+    <row r="1423" spans="1:8">
+      <c r="A1423">
+        <v>901196</v>
+      </c>
+      <c r="B1423" s="2">
+        <v>91196</v>
+      </c>
+      <c r="C1423" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1423" s="130" t="s">
+        <v>7731</v>
+      </c>
+      <c r="E1423" s="130" t="s">
+        <v>7739</v>
+      </c>
+      <c r="F1423" s="130" t="s">
+        <v>7740</v>
+      </c>
+      <c r="G1423" s="130" t="s">
+        <v>816</v>
+      </c>
+      <c r="H1423" s="130" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="1424" spans="1:8">
+      <c r="A1424">
+        <v>901197</v>
+      </c>
+      <c r="B1424" s="2">
+        <v>91197</v>
+      </c>
+      <c r="C1424" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1424" s="130" t="s">
+        <v>7732</v>
+      </c>
+      <c r="E1424" s="130" t="s">
+        <v>7741</v>
+      </c>
+      <c r="F1424" s="130" t="s">
+        <v>7742</v>
+      </c>
+      <c r="G1424" s="130" t="s">
+        <v>816</v>
+      </c>
+      <c r="H1424" s="130" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="1425" spans="1:8">
+      <c r="A1425">
+        <v>901198</v>
+      </c>
+      <c r="B1425" s="2">
+        <v>91198</v>
+      </c>
+      <c r="C1425" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1425" s="130" t="s">
+        <v>7733</v>
+      </c>
+      <c r="E1425" s="130" t="s">
+        <v>7743</v>
+      </c>
+      <c r="F1425" s="130" t="s">
+        <v>7744</v>
+      </c>
+      <c r="G1425" s="130" t="s">
+        <v>816</v>
+      </c>
+      <c r="H1425" s="130" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="1426" spans="1:8">
+      <c r="A1426">
+        <v>901199</v>
+      </c>
+      <c r="B1426" s="2">
+        <v>91199</v>
+      </c>
+      <c r="C1426" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1426" s="130" t="s">
+        <v>7734</v>
+      </c>
+      <c r="E1426" s="130" t="s">
+        <v>7745</v>
+      </c>
+      <c r="F1426" s="130" t="s">
+        <v>7746</v>
+      </c>
+      <c r="G1426" s="130" t="s">
+        <v>816</v>
+      </c>
+      <c r="H1426" s="130" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="1427" spans="1:8">
+      <c r="A1427">
+        <v>901200</v>
+      </c>
+      <c r="B1427" s="2">
+        <v>91200</v>
+      </c>
+      <c r="C1427" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1427" s="130" t="s">
+        <v>7735</v>
+      </c>
+      <c r="E1427" s="130" t="s">
+        <v>7747</v>
+      </c>
+      <c r="F1427" s="130" t="s">
+        <v>7748</v>
+      </c>
+      <c r="G1427" s="130" t="s">
+        <v>816</v>
+      </c>
+      <c r="H1427" s="130" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="1428" spans="1:8">
+      <c r="A1428">
+        <v>901201</v>
+      </c>
+      <c r="B1428" s="2">
+        <v>91201</v>
+      </c>
+      <c r="C1428" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1428" s="130" t="s">
+        <v>7736</v>
+      </c>
+      <c r="E1428" s="130" t="s">
+        <v>7749</v>
+      </c>
+      <c r="F1428" s="130" t="s">
+        <v>7750</v>
+      </c>
+      <c r="G1428" s="130" t="s">
+        <v>816</v>
+      </c>
+      <c r="H1428" s="130" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="1429" spans="1:8">
+      <c r="A1429">
+        <v>901202</v>
+      </c>
+      <c r="B1429" s="2">
+        <v>91202</v>
+      </c>
+      <c r="C1429" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1429" s="130" t="s">
+        <v>7737</v>
+      </c>
+      <c r="E1429" s="130" t="s">
+        <v>7751</v>
+      </c>
+      <c r="F1429" s="130" t="s">
+        <v>7752</v>
+      </c>
+      <c r="G1429" s="130" t="s">
+        <v>816</v>
+      </c>
+      <c r="H1429" s="130" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="1430" spans="1:8">
+      <c r="A1430">
+        <v>901203</v>
+      </c>
+      <c r="B1430" s="2">
+        <v>91203</v>
+      </c>
+      <c r="C1430" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1430" s="130" t="s">
+        <v>7738</v>
+      </c>
+      <c r="E1430" s="130" t="s">
+        <v>7753</v>
+      </c>
+      <c r="F1430" s="130" t="s">
+        <v>7754</v>
+      </c>
+      <c r="G1430" s="130" t="s">
+        <v>816</v>
+      </c>
+      <c r="H1430" s="130" t="s">
+        <v>816</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[MOD] 261015 보스 밸런싱
모든 보스 체력 대폭 조정
대왕송이 강화
</commit_message>
<xml_diff>
--- a/Assets/DB/MMM_DB_Ver.05.xlsx
+++ b/Assets/DB/MMM_DB_Ver.05.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\MoreMustMush\Assets\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EBF2F06-1097-4685-9A42-C0AC5C5204CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70A8BBAE-F033-478E-90D4-D4528F65E15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5790" yWindow="1035" windowWidth="18660" windowHeight="13995" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27552,46 +27552,46 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -27600,12 +27600,12 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -28073,29 +28073,29 @@
   <sheetData>
     <row r="1" spans="2:44" ht="12" customHeight="1"/>
     <row r="2" spans="2:44">
-      <c r="B2" s="154" t="s">
+      <c r="B2" s="156" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="155"/>
-      <c r="D2" s="155"/>
-      <c r="E2" s="155"/>
-      <c r="F2" s="155"/>
-      <c r="G2" s="155"/>
-      <c r="H2" s="155"/>
-      <c r="I2" s="155"/>
-      <c r="J2" s="155"/>
-      <c r="K2" s="155"/>
-      <c r="L2" s="155"/>
-      <c r="M2" s="155"/>
-      <c r="N2" s="155"/>
-      <c r="O2" s="155"/>
-      <c r="P2" s="155"/>
-      <c r="Q2" s="155"/>
-      <c r="R2" s="155"/>
-      <c r="S2" s="155"/>
-      <c r="T2" s="155"/>
-      <c r="U2" s="155"/>
-      <c r="V2" s="156"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="157"/>
+      <c r="E2" s="157"/>
+      <c r="F2" s="157"/>
+      <c r="G2" s="157"/>
+      <c r="H2" s="157"/>
+      <c r="I2" s="157"/>
+      <c r="J2" s="157"/>
+      <c r="K2" s="157"/>
+      <c r="L2" s="157"/>
+      <c r="M2" s="157"/>
+      <c r="N2" s="157"/>
+      <c r="O2" s="157"/>
+      <c r="P2" s="157"/>
+      <c r="Q2" s="157"/>
+      <c r="R2" s="157"/>
+      <c r="S2" s="157"/>
+      <c r="T2" s="157"/>
+      <c r="U2" s="157"/>
+      <c r="V2" s="158"/>
     </row>
     <row r="3" spans="2:44">
       <c r="B3" s="17"/>
@@ -28152,29 +28152,29 @@
       <c r="V4" s="14"/>
     </row>
     <row r="5" spans="2:44">
-      <c r="B5" s="154" t="s">
+      <c r="B5" s="156" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="155"/>
-      <c r="D5" s="155"/>
-      <c r="E5" s="155"/>
-      <c r="F5" s="155"/>
-      <c r="G5" s="155"/>
-      <c r="H5" s="155"/>
-      <c r="I5" s="155"/>
-      <c r="J5" s="155"/>
-      <c r="K5" s="155"/>
-      <c r="L5" s="155"/>
-      <c r="M5" s="155"/>
-      <c r="N5" s="155"/>
-      <c r="O5" s="155"/>
-      <c r="P5" s="155"/>
-      <c r="Q5" s="155"/>
-      <c r="R5" s="155"/>
-      <c r="S5" s="155"/>
-      <c r="T5" s="155"/>
-      <c r="U5" s="155"/>
-      <c r="V5" s="156"/>
+      <c r="C5" s="157"/>
+      <c r="D5" s="157"/>
+      <c r="E5" s="157"/>
+      <c r="F5" s="157"/>
+      <c r="G5" s="157"/>
+      <c r="H5" s="157"/>
+      <c r="I5" s="157"/>
+      <c r="J5" s="157"/>
+      <c r="K5" s="157"/>
+      <c r="L5" s="157"/>
+      <c r="M5" s="157"/>
+      <c r="N5" s="157"/>
+      <c r="O5" s="157"/>
+      <c r="P5" s="157"/>
+      <c r="Q5" s="157"/>
+      <c r="R5" s="157"/>
+      <c r="S5" s="157"/>
+      <c r="T5" s="157"/>
+      <c r="U5" s="157"/>
+      <c r="V5" s="158"/>
     </row>
     <row r="6" spans="2:44">
       <c r="B6" s="6"/>
@@ -28304,29 +28304,29 @@
     </row>
     <row r="10" spans="2:44" ht="8.1" customHeight="1"/>
     <row r="11" spans="2:44">
-      <c r="B11" s="154" t="s">
+      <c r="B11" s="156" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="155"/>
-      <c r="D11" s="155"/>
-      <c r="E11" s="155"/>
-      <c r="F11" s="155"/>
-      <c r="G11" s="155"/>
-      <c r="H11" s="155"/>
-      <c r="I11" s="155"/>
-      <c r="J11" s="155"/>
-      <c r="K11" s="155"/>
-      <c r="L11" s="155"/>
-      <c r="M11" s="155"/>
-      <c r="N11" s="155"/>
-      <c r="O11" s="155"/>
-      <c r="P11" s="155"/>
-      <c r="Q11" s="155"/>
-      <c r="R11" s="155"/>
-      <c r="S11" s="155"/>
-      <c r="T11" s="155"/>
-      <c r="U11" s="155"/>
-      <c r="V11" s="156"/>
+      <c r="C11" s="157"/>
+      <c r="D11" s="157"/>
+      <c r="E11" s="157"/>
+      <c r="F11" s="157"/>
+      <c r="G11" s="157"/>
+      <c r="H11" s="157"/>
+      <c r="I11" s="157"/>
+      <c r="J11" s="157"/>
+      <c r="K11" s="157"/>
+      <c r="L11" s="157"/>
+      <c r="M11" s="157"/>
+      <c r="N11" s="157"/>
+      <c r="O11" s="157"/>
+      <c r="P11" s="157"/>
+      <c r="Q11" s="157"/>
+      <c r="R11" s="157"/>
+      <c r="S11" s="157"/>
+      <c r="T11" s="157"/>
+      <c r="U11" s="157"/>
+      <c r="V11" s="158"/>
     </row>
     <row r="12" spans="2:44">
       <c r="B12" s="6"/>
@@ -28613,19 +28613,19 @@
       <c r="AF22" s="27"/>
     </row>
     <row r="23" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B23" s="157" t="s">
+      <c r="B23" s="159" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="144"/>
-      <c r="D23" s="144"/>
-      <c r="E23" s="144"/>
-      <c r="F23" s="144"/>
-      <c r="G23" s="144"/>
-      <c r="H23" s="143" t="s">
+      <c r="C23" s="146"/>
+      <c r="D23" s="146"/>
+      <c r="E23" s="146"/>
+      <c r="F23" s="146"/>
+      <c r="G23" s="146"/>
+      <c r="H23" s="161" t="s">
         <v>67</v>
       </c>
-      <c r="I23" s="144"/>
-      <c r="J23" s="144"/>
+      <c r="I23" s="146"/>
+      <c r="J23" s="146"/>
       <c r="K23" s="28" t="s">
         <v>68</v>
       </c>
@@ -28653,18 +28653,18 @@
     </row>
     <row r="24" spans="2:32" s="10" customFormat="1">
       <c r="B24" s="86"/>
-      <c r="C24" s="153" t="s">
+      <c r="C24" s="136" t="s">
         <v>3</v>
       </c>
-      <c r="D24" s="151"/>
-      <c r="E24" s="151"/>
-      <c r="F24" s="151"/>
-      <c r="G24" s="152"/>
-      <c r="H24" s="150" t="s">
+      <c r="D24" s="137"/>
+      <c r="E24" s="137"/>
+      <c r="F24" s="137"/>
+      <c r="G24" s="138"/>
+      <c r="H24" s="142" t="s">
         <v>69</v>
       </c>
-      <c r="I24" s="151"/>
-      <c r="J24" s="152"/>
+      <c r="I24" s="137"/>
+      <c r="J24" s="138"/>
       <c r="K24" s="34" t="s">
         <v>70</v>
       </c>
@@ -28692,14 +28692,14 @@
     </row>
     <row r="25" spans="2:32" s="10" customFormat="1">
       <c r="B25" s="22"/>
-      <c r="C25" s="140"/>
-      <c r="D25" s="140"/>
-      <c r="E25" s="140"/>
-      <c r="F25" s="140"/>
-      <c r="G25" s="141"/>
-      <c r="H25" s="158"/>
-      <c r="I25" s="140"/>
-      <c r="J25" s="141"/>
+      <c r="C25" s="139"/>
+      <c r="D25" s="139"/>
+      <c r="E25" s="139"/>
+      <c r="F25" s="139"/>
+      <c r="G25" s="140"/>
+      <c r="H25" s="143"/>
+      <c r="I25" s="139"/>
+      <c r="J25" s="140"/>
       <c r="K25" s="19" t="s">
         <v>49</v>
       </c>
@@ -28721,18 +28721,18 @@
     </row>
     <row r="26" spans="2:32" s="10" customFormat="1">
       <c r="B26" s="22"/>
-      <c r="C26" s="139" t="s">
+      <c r="C26" s="144" t="s">
         <v>72</v>
       </c>
-      <c r="D26" s="140"/>
-      <c r="E26" s="140"/>
-      <c r="F26" s="140"/>
-      <c r="G26" s="141"/>
-      <c r="H26" s="146" t="s">
+      <c r="D26" s="139"/>
+      <c r="E26" s="139"/>
+      <c r="F26" s="139"/>
+      <c r="G26" s="140"/>
+      <c r="H26" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I26" s="140"/>
-      <c r="J26" s="141"/>
+      <c r="I26" s="139"/>
+      <c r="J26" s="140"/>
       <c r="K26" s="19" t="s">
         <v>74</v>
       </c>
@@ -28752,18 +28752,18 @@
     </row>
     <row r="27" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B27" s="22"/>
-      <c r="C27" s="139" t="s">
+      <c r="C27" s="144" t="s">
         <v>9</v>
       </c>
-      <c r="D27" s="140"/>
-      <c r="E27" s="140"/>
-      <c r="F27" s="140"/>
-      <c r="G27" s="141"/>
-      <c r="H27" s="146" t="s">
+      <c r="D27" s="139"/>
+      <c r="E27" s="139"/>
+      <c r="F27" s="139"/>
+      <c r="G27" s="140"/>
+      <c r="H27" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I27" s="140"/>
-      <c r="J27" s="141"/>
+      <c r="I27" s="139"/>
+      <c r="J27" s="140"/>
       <c r="K27" s="19" t="s">
         <v>75</v>
       </c>
@@ -28783,18 +28783,18 @@
     </row>
     <row r="28" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B28" s="22"/>
-      <c r="C28" s="139" t="s">
+      <c r="C28" s="144" t="s">
         <v>76</v>
       </c>
-      <c r="D28" s="140"/>
-      <c r="E28" s="140"/>
-      <c r="F28" s="140"/>
-      <c r="G28" s="141"/>
-      <c r="H28" s="146" t="s">
+      <c r="D28" s="139"/>
+      <c r="E28" s="139"/>
+      <c r="F28" s="139"/>
+      <c r="G28" s="140"/>
+      <c r="H28" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I28" s="140"/>
-      <c r="J28" s="141"/>
+      <c r="I28" s="139"/>
+      <c r="J28" s="140"/>
       <c r="K28" s="19" t="s">
         <v>77</v>
       </c>
@@ -28814,18 +28814,18 @@
     </row>
     <row r="29" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B29" s="22"/>
-      <c r="C29" s="139" t="s">
+      <c r="C29" s="144" t="s">
         <v>67</v>
       </c>
-      <c r="D29" s="140"/>
-      <c r="E29" s="140"/>
-      <c r="F29" s="140"/>
-      <c r="G29" s="141"/>
-      <c r="H29" s="146" t="s">
+      <c r="D29" s="139"/>
+      <c r="E29" s="139"/>
+      <c r="F29" s="139"/>
+      <c r="G29" s="140"/>
+      <c r="H29" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I29" s="140"/>
-      <c r="J29" s="141"/>
+      <c r="I29" s="139"/>
+      <c r="J29" s="140"/>
       <c r="K29" s="19" t="s">
         <v>78</v>
       </c>
@@ -28845,18 +28845,18 @@
     </row>
     <row r="30" spans="2:32" s="10" customFormat="1">
       <c r="B30" s="22"/>
-      <c r="C30" s="139" t="s">
+      <c r="C30" s="144" t="s">
         <v>79</v>
       </c>
-      <c r="D30" s="140"/>
-      <c r="E30" s="140"/>
-      <c r="F30" s="140"/>
-      <c r="G30" s="141"/>
-      <c r="H30" s="146" t="s">
+      <c r="D30" s="139"/>
+      <c r="E30" s="139"/>
+      <c r="F30" s="139"/>
+      <c r="G30" s="140"/>
+      <c r="H30" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I30" s="140"/>
-      <c r="J30" s="141"/>
+      <c r="I30" s="139"/>
+      <c r="J30" s="140"/>
       <c r="K30" s="120" t="s">
         <v>421</v>
       </c>
@@ -28876,18 +28876,18 @@
     </row>
     <row r="31" spans="2:32" s="10" customFormat="1">
       <c r="B31" s="22"/>
-      <c r="C31" s="139" t="s">
+      <c r="C31" s="144" t="s">
         <v>7</v>
       </c>
-      <c r="D31" s="140"/>
-      <c r="E31" s="140"/>
-      <c r="F31" s="140"/>
-      <c r="G31" s="141"/>
-      <c r="H31" s="146" t="s">
+      <c r="D31" s="139"/>
+      <c r="E31" s="139"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="140"/>
+      <c r="H31" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I31" s="140"/>
-      <c r="J31" s="141"/>
+      <c r="I31" s="139"/>
+      <c r="J31" s="140"/>
       <c r="K31" s="19" t="s">
         <v>80</v>
       </c>
@@ -28907,18 +28907,18 @@
     </row>
     <row r="32" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B32" s="75"/>
-      <c r="C32" s="145" t="s">
+      <c r="C32" s="160" t="s">
         <v>422</v>
       </c>
-      <c r="D32" s="137"/>
-      <c r="E32" s="137"/>
-      <c r="F32" s="137"/>
-      <c r="G32" s="138"/>
-      <c r="H32" s="136" t="s">
+      <c r="D32" s="149"/>
+      <c r="E32" s="149"/>
+      <c r="F32" s="149"/>
+      <c r="G32" s="150"/>
+      <c r="H32" s="148" t="s">
         <v>81</v>
       </c>
-      <c r="I32" s="137"/>
-      <c r="J32" s="138"/>
+      <c r="I32" s="149"/>
+      <c r="J32" s="150"/>
       <c r="K32" s="81" t="s">
         <v>82</v>
       </c>
@@ -28980,19 +28980,19 @@
       <c r="AF33" s="27"/>
     </row>
     <row r="34" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B34" s="148" t="s">
+      <c r="B34" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C34" s="144"/>
-      <c r="D34" s="144"/>
-      <c r="E34" s="144"/>
-      <c r="F34" s="144"/>
-      <c r="G34" s="149"/>
-      <c r="H34" s="148" t="s">
+      <c r="C34" s="146"/>
+      <c r="D34" s="146"/>
+      <c r="E34" s="146"/>
+      <c r="F34" s="146"/>
+      <c r="G34" s="147"/>
+      <c r="H34" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I34" s="144"/>
-      <c r="J34" s="149"/>
+      <c r="I34" s="146"/>
+      <c r="J34" s="147"/>
       <c r="K34" s="28" t="s">
         <v>68</v>
       </c>
@@ -29020,18 +29020,18 @@
     </row>
     <row r="35" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B35" s="86"/>
-      <c r="C35" s="153" t="s">
+      <c r="C35" s="136" t="s">
         <v>7</v>
       </c>
-      <c r="D35" s="151"/>
-      <c r="E35" s="151"/>
-      <c r="F35" s="151"/>
-      <c r="G35" s="152"/>
-      <c r="H35" s="150" t="s">
+      <c r="D35" s="137"/>
+      <c r="E35" s="137"/>
+      <c r="F35" s="137"/>
+      <c r="G35" s="138"/>
+      <c r="H35" s="142" t="s">
         <v>69</v>
       </c>
-      <c r="I35" s="151"/>
-      <c r="J35" s="152"/>
+      <c r="I35" s="137"/>
+      <c r="J35" s="138"/>
       <c r="K35" s="34" t="s">
         <v>84</v>
       </c>
@@ -29059,18 +29059,18 @@
     </row>
     <row r="36" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B36" s="75"/>
-      <c r="C36" s="145" t="s">
+      <c r="C36" s="160" t="s">
         <v>423</v>
       </c>
-      <c r="D36" s="137"/>
-      <c r="E36" s="137"/>
-      <c r="F36" s="137"/>
-      <c r="G36" s="138"/>
-      <c r="H36" s="136" t="s">
+      <c r="D36" s="149"/>
+      <c r="E36" s="149"/>
+      <c r="F36" s="149"/>
+      <c r="G36" s="150"/>
+      <c r="H36" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="I36" s="137"/>
-      <c r="J36" s="138"/>
+      <c r="I36" s="149"/>
+      <c r="J36" s="150"/>
       <c r="K36" s="81" t="s">
         <v>85</v>
       </c>
@@ -29132,19 +29132,19 @@
       <c r="AF37" s="92"/>
     </row>
     <row r="38" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B38" s="148" t="s">
+      <c r="B38" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C38" s="144"/>
-      <c r="D38" s="144"/>
-      <c r="E38" s="144"/>
-      <c r="F38" s="144"/>
-      <c r="G38" s="149"/>
-      <c r="H38" s="148" t="s">
+      <c r="C38" s="146"/>
+      <c r="D38" s="146"/>
+      <c r="E38" s="146"/>
+      <c r="F38" s="146"/>
+      <c r="G38" s="147"/>
+      <c r="H38" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I38" s="144"/>
-      <c r="J38" s="149"/>
+      <c r="I38" s="146"/>
+      <c r="J38" s="147"/>
       <c r="K38" s="28" t="s">
         <v>68</v>
       </c>
@@ -29172,18 +29172,18 @@
     </row>
     <row r="39" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B39" s="21"/>
-      <c r="C39" s="139" t="s">
+      <c r="C39" s="144" t="s">
         <v>14</v>
       </c>
-      <c r="D39" s="140"/>
-      <c r="E39" s="140"/>
-      <c r="F39" s="140"/>
-      <c r="G39" s="141"/>
-      <c r="H39" s="146" t="s">
+      <c r="D39" s="139"/>
+      <c r="E39" s="139"/>
+      <c r="F39" s="139"/>
+      <c r="G39" s="140"/>
+      <c r="H39" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I39" s="140"/>
-      <c r="J39" s="141"/>
+      <c r="I39" s="139"/>
+      <c r="J39" s="140"/>
       <c r="K39" s="19" t="s">
         <v>86</v>
       </c>
@@ -29203,18 +29203,18 @@
     </row>
     <row r="40" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B40" s="22"/>
-      <c r="C40" s="139" t="s">
+      <c r="C40" s="144" t="s">
         <v>87</v>
       </c>
-      <c r="D40" s="140"/>
-      <c r="E40" s="140"/>
-      <c r="F40" s="140"/>
-      <c r="G40" s="141"/>
-      <c r="H40" s="146" t="s">
+      <c r="D40" s="139"/>
+      <c r="E40" s="139"/>
+      <c r="F40" s="139"/>
+      <c r="G40" s="140"/>
+      <c r="H40" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I40" s="140"/>
-      <c r="J40" s="141"/>
+      <c r="I40" s="139"/>
+      <c r="J40" s="140"/>
       <c r="K40" s="19" t="s">
         <v>88</v>
       </c>
@@ -29234,18 +29234,18 @@
     </row>
     <row r="41" spans="2:32" s="10" customFormat="1">
       <c r="B41" s="22"/>
-      <c r="C41" s="139" t="s">
+      <c r="C41" s="144" t="s">
         <v>16</v>
       </c>
-      <c r="D41" s="140"/>
-      <c r="E41" s="140"/>
-      <c r="F41" s="140"/>
-      <c r="G41" s="141"/>
-      <c r="H41" s="146" t="s">
+      <c r="D41" s="139"/>
+      <c r="E41" s="139"/>
+      <c r="F41" s="139"/>
+      <c r="G41" s="140"/>
+      <c r="H41" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I41" s="140"/>
-      <c r="J41" s="141"/>
+      <c r="I41" s="139"/>
+      <c r="J41" s="140"/>
       <c r="K41" s="19" t="s">
         <v>89</v>
       </c>
@@ -29265,18 +29265,18 @@
     </row>
     <row r="42" spans="2:32" s="10" customFormat="1">
       <c r="B42" s="22"/>
-      <c r="C42" s="139" t="s">
+      <c r="C42" s="144" t="s">
         <v>90</v>
       </c>
-      <c r="D42" s="140"/>
-      <c r="E42" s="140"/>
-      <c r="F42" s="140"/>
-      <c r="G42" s="141"/>
-      <c r="H42" s="146" t="s">
+      <c r="D42" s="139"/>
+      <c r="E42" s="139"/>
+      <c r="F42" s="139"/>
+      <c r="G42" s="140"/>
+      <c r="H42" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I42" s="140"/>
-      <c r="J42" s="141"/>
+      <c r="I42" s="139"/>
+      <c r="J42" s="140"/>
       <c r="K42" s="19" t="s">
         <v>91</v>
       </c>
@@ -29296,18 +29296,18 @@
     </row>
     <row r="43" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B43" s="75"/>
-      <c r="C43" s="142" t="s">
+      <c r="C43" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="D43" s="137"/>
-      <c r="E43" s="137"/>
-      <c r="F43" s="137"/>
-      <c r="G43" s="138"/>
-      <c r="H43" s="136" t="s">
+      <c r="D43" s="149"/>
+      <c r="E43" s="149"/>
+      <c r="F43" s="149"/>
+      <c r="G43" s="150"/>
+      <c r="H43" s="148" t="s">
         <v>73</v>
       </c>
-      <c r="I43" s="137"/>
-      <c r="J43" s="138"/>
+      <c r="I43" s="149"/>
+      <c r="J43" s="150"/>
       <c r="K43" s="81" t="s">
         <v>92</v>
       </c>
@@ -29369,19 +29369,19 @@
       <c r="AF44" s="27"/>
     </row>
     <row r="45" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B45" s="148" t="s">
+      <c r="B45" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C45" s="144"/>
-      <c r="D45" s="144"/>
-      <c r="E45" s="144"/>
-      <c r="F45" s="144"/>
-      <c r="G45" s="149"/>
-      <c r="H45" s="159" t="s">
+      <c r="C45" s="146"/>
+      <c r="D45" s="146"/>
+      <c r="E45" s="146"/>
+      <c r="F45" s="146"/>
+      <c r="G45" s="147"/>
+      <c r="H45" s="153" t="s">
         <v>67</v>
       </c>
-      <c r="I45" s="160"/>
-      <c r="J45" s="161"/>
+      <c r="I45" s="154"/>
+      <c r="J45" s="155"/>
       <c r="K45" s="83" t="s">
         <v>68</v>
       </c>
@@ -29409,18 +29409,18 @@
     </row>
     <row r="46" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B46" s="21"/>
-      <c r="C46" s="139" t="s">
+      <c r="C46" s="144" t="s">
         <v>15</v>
       </c>
-      <c r="D46" s="140"/>
-      <c r="E46" s="140"/>
-      <c r="F46" s="140"/>
-      <c r="G46" s="141"/>
-      <c r="H46" s="150" t="s">
+      <c r="D46" s="139"/>
+      <c r="E46" s="139"/>
+      <c r="F46" s="139"/>
+      <c r="G46" s="140"/>
+      <c r="H46" s="142" t="s">
         <v>73</v>
       </c>
-      <c r="I46" s="151"/>
-      <c r="J46" s="152"/>
+      <c r="I46" s="137"/>
+      <c r="J46" s="138"/>
       <c r="K46" s="19" t="s">
         <v>93</v>
       </c>
@@ -29440,18 +29440,18 @@
     </row>
     <row r="47" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B47" s="22"/>
-      <c r="C47" s="139" t="s">
+      <c r="C47" s="144" t="s">
         <v>94</v>
       </c>
-      <c r="D47" s="140"/>
-      <c r="E47" s="140"/>
-      <c r="F47" s="140"/>
-      <c r="G47" s="141"/>
-      <c r="H47" s="146" t="s">
+      <c r="D47" s="139"/>
+      <c r="E47" s="139"/>
+      <c r="F47" s="139"/>
+      <c r="G47" s="140"/>
+      <c r="H47" s="141" t="s">
         <v>81</v>
       </c>
-      <c r="I47" s="140"/>
-      <c r="J47" s="141"/>
+      <c r="I47" s="139"/>
+      <c r="J47" s="140"/>
       <c r="K47" s="19" t="s">
         <v>95</v>
       </c>
@@ -29471,14 +29471,14 @@
     </row>
     <row r="48" spans="2:32" s="10" customFormat="1">
       <c r="B48" s="22"/>
-      <c r="C48" s="140"/>
-      <c r="D48" s="140"/>
-      <c r="E48" s="140"/>
-      <c r="F48" s="140"/>
-      <c r="G48" s="141"/>
-      <c r="H48" s="158"/>
-      <c r="I48" s="140"/>
-      <c r="J48" s="141"/>
+      <c r="C48" s="139"/>
+      <c r="D48" s="139"/>
+      <c r="E48" s="139"/>
+      <c r="F48" s="139"/>
+      <c r="G48" s="140"/>
+      <c r="H48" s="143"/>
+      <c r="I48" s="139"/>
+      <c r="J48" s="140"/>
       <c r="K48" s="19" t="s">
         <v>49</v>
       </c>
@@ -29500,14 +29500,14 @@
     </row>
     <row r="49" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B49" s="22"/>
-      <c r="C49" s="140"/>
-      <c r="D49" s="140"/>
-      <c r="E49" s="140"/>
-      <c r="F49" s="140"/>
-      <c r="G49" s="141"/>
-      <c r="H49" s="158"/>
-      <c r="I49" s="140"/>
-      <c r="J49" s="141"/>
+      <c r="C49" s="139"/>
+      <c r="D49" s="139"/>
+      <c r="E49" s="139"/>
+      <c r="F49" s="139"/>
+      <c r="G49" s="140"/>
+      <c r="H49" s="143"/>
+      <c r="I49" s="139"/>
+      <c r="J49" s="140"/>
       <c r="K49" s="19" t="s">
         <v>49</v>
       </c>
@@ -29564,19 +29564,19 @@
       <c r="AG50" s="92"/>
     </row>
     <row r="51" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B51" s="148" t="s">
+      <c r="B51" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C51" s="144"/>
-      <c r="D51" s="144"/>
-      <c r="E51" s="144"/>
-      <c r="F51" s="144"/>
-      <c r="G51" s="149"/>
-      <c r="H51" s="148" t="s">
+      <c r="C51" s="146"/>
+      <c r="D51" s="146"/>
+      <c r="E51" s="146"/>
+      <c r="F51" s="146"/>
+      <c r="G51" s="147"/>
+      <c r="H51" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I51" s="144"/>
-      <c r="J51" s="149"/>
+      <c r="I51" s="146"/>
+      <c r="J51" s="147"/>
       <c r="K51" s="28" t="s">
         <v>68</v>
       </c>
@@ -29605,18 +29605,18 @@
     </row>
     <row r="52" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B52" s="21"/>
-      <c r="C52" s="139" t="s">
+      <c r="C52" s="144" t="s">
         <v>23</v>
       </c>
-      <c r="D52" s="140"/>
-      <c r="E52" s="140"/>
-      <c r="F52" s="140"/>
-      <c r="G52" s="141"/>
-      <c r="H52" s="146" t="s">
+      <c r="D52" s="139"/>
+      <c r="E52" s="139"/>
+      <c r="F52" s="139"/>
+      <c r="G52" s="140"/>
+      <c r="H52" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I52" s="140"/>
-      <c r="J52" s="141"/>
+      <c r="I52" s="139"/>
+      <c r="J52" s="140"/>
       <c r="K52" s="19" t="s">
         <v>99</v>
       </c>
@@ -29636,18 +29636,18 @@
     </row>
     <row r="53" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B53" s="22"/>
-      <c r="C53" s="139" t="s">
+      <c r="C53" s="144" t="s">
         <v>100</v>
       </c>
-      <c r="D53" s="140"/>
-      <c r="E53" s="140"/>
-      <c r="F53" s="140"/>
-      <c r="G53" s="141"/>
-      <c r="H53" s="146" t="s">
+      <c r="D53" s="139"/>
+      <c r="E53" s="139"/>
+      <c r="F53" s="139"/>
+      <c r="G53" s="140"/>
+      <c r="H53" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I53" s="140"/>
-      <c r="J53" s="141"/>
+      <c r="I53" s="139"/>
+      <c r="J53" s="140"/>
       <c r="K53" s="19" t="s">
         <v>101</v>
       </c>
@@ -29667,18 +29667,18 @@
     </row>
     <row r="54" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B54" s="75"/>
-      <c r="C54" s="142" t="s">
+      <c r="C54" s="152" t="s">
         <v>102</v>
       </c>
-      <c r="D54" s="137"/>
-      <c r="E54" s="137"/>
-      <c r="F54" s="137"/>
-      <c r="G54" s="138"/>
-      <c r="H54" s="136" t="s">
+      <c r="D54" s="149"/>
+      <c r="E54" s="149"/>
+      <c r="F54" s="149"/>
+      <c r="G54" s="150"/>
+      <c r="H54" s="148" t="s">
         <v>73</v>
       </c>
-      <c r="I54" s="137"/>
-      <c r="J54" s="138"/>
+      <c r="I54" s="149"/>
+      <c r="J54" s="150"/>
       <c r="K54" s="81" t="s">
         <v>103</v>
       </c>
@@ -29742,19 +29742,19 @@
       <c r="AG55" s="92"/>
     </row>
     <row r="56" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B56" s="148" t="s">
+      <c r="B56" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C56" s="144"/>
-      <c r="D56" s="144"/>
-      <c r="E56" s="144"/>
-      <c r="F56" s="144"/>
-      <c r="G56" s="149"/>
-      <c r="H56" s="148" t="s">
+      <c r="C56" s="146"/>
+      <c r="D56" s="146"/>
+      <c r="E56" s="146"/>
+      <c r="F56" s="146"/>
+      <c r="G56" s="147"/>
+      <c r="H56" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I56" s="144"/>
-      <c r="J56" s="149"/>
+      <c r="I56" s="146"/>
+      <c r="J56" s="147"/>
       <c r="K56" s="28" t="s">
         <v>68</v>
       </c>
@@ -29783,18 +29783,18 @@
     </row>
     <row r="57" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B57" s="21"/>
-      <c r="C57" s="139" t="s">
+      <c r="C57" s="144" t="s">
         <v>6</v>
       </c>
-      <c r="D57" s="140"/>
-      <c r="E57" s="140"/>
-      <c r="F57" s="140"/>
-      <c r="G57" s="141"/>
-      <c r="H57" s="146" t="s">
+      <c r="D57" s="139"/>
+      <c r="E57" s="139"/>
+      <c r="F57" s="139"/>
+      <c r="G57" s="140"/>
+      <c r="H57" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I57" s="140"/>
-      <c r="J57" s="141"/>
+      <c r="I57" s="139"/>
+      <c r="J57" s="140"/>
       <c r="K57" s="19" t="s">
         <v>104</v>
       </c>
@@ -29814,18 +29814,18 @@
     </row>
     <row r="58" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B58" s="22"/>
-      <c r="C58" s="139" t="s">
+      <c r="C58" s="144" t="s">
         <v>105</v>
       </c>
-      <c r="D58" s="140"/>
-      <c r="E58" s="140"/>
-      <c r="F58" s="140"/>
-      <c r="G58" s="141"/>
-      <c r="H58" s="146" t="s">
+      <c r="D58" s="139"/>
+      <c r="E58" s="139"/>
+      <c r="F58" s="139"/>
+      <c r="G58" s="140"/>
+      <c r="H58" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I58" s="140"/>
-      <c r="J58" s="141"/>
+      <c r="I58" s="139"/>
+      <c r="J58" s="140"/>
       <c r="K58" s="19" t="s">
         <v>106</v>
       </c>
@@ -29845,18 +29845,18 @@
     </row>
     <row r="59" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B59" s="22"/>
-      <c r="C59" s="139" t="s">
+      <c r="C59" s="144" t="s">
         <v>9</v>
       </c>
-      <c r="D59" s="140"/>
-      <c r="E59" s="140"/>
-      <c r="F59" s="140"/>
-      <c r="G59" s="141"/>
-      <c r="H59" s="146" t="s">
+      <c r="D59" s="139"/>
+      <c r="E59" s="139"/>
+      <c r="F59" s="139"/>
+      <c r="G59" s="140"/>
+      <c r="H59" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I59" s="140"/>
-      <c r="J59" s="141"/>
+      <c r="I59" s="139"/>
+      <c r="J59" s="140"/>
       <c r="K59" s="19" t="s">
         <v>107</v>
       </c>
@@ -29876,18 +29876,18 @@
     </row>
     <row r="60" spans="2:33" s="10" customFormat="1">
       <c r="B60" s="22"/>
-      <c r="C60" s="139" t="s">
+      <c r="C60" s="144" t="s">
         <v>108</v>
       </c>
-      <c r="D60" s="140"/>
-      <c r="E60" s="140"/>
-      <c r="F60" s="140"/>
-      <c r="G60" s="141"/>
-      <c r="H60" s="146" t="s">
+      <c r="D60" s="139"/>
+      <c r="E60" s="139"/>
+      <c r="F60" s="139"/>
+      <c r="G60" s="140"/>
+      <c r="H60" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I60" s="140"/>
-      <c r="J60" s="141"/>
+      <c r="I60" s="139"/>
+      <c r="J60" s="140"/>
       <c r="K60" s="19" t="s">
         <v>109</v>
       </c>
@@ -29907,18 +29907,18 @@
     </row>
     <row r="61" spans="2:33" s="10" customFormat="1">
       <c r="B61" s="22"/>
-      <c r="C61" s="139" t="s">
+      <c r="C61" s="144" t="s">
         <v>110</v>
       </c>
-      <c r="D61" s="140"/>
-      <c r="E61" s="140"/>
-      <c r="F61" s="140"/>
-      <c r="G61" s="141"/>
-      <c r="H61" s="146" t="s">
+      <c r="D61" s="139"/>
+      <c r="E61" s="139"/>
+      <c r="F61" s="139"/>
+      <c r="G61" s="140"/>
+      <c r="H61" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I61" s="140"/>
-      <c r="J61" s="141"/>
+      <c r="I61" s="139"/>
+      <c r="J61" s="140"/>
       <c r="K61" s="19" t="s">
         <v>111</v>
       </c>
@@ -29938,18 +29938,18 @@
     </row>
     <row r="62" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B62" s="75"/>
-      <c r="C62" s="142" t="s">
+      <c r="C62" s="152" t="s">
         <v>112</v>
       </c>
-      <c r="D62" s="137"/>
-      <c r="E62" s="137"/>
-      <c r="F62" s="137"/>
-      <c r="G62" s="138"/>
-      <c r="H62" s="136" t="s">
+      <c r="D62" s="149"/>
+      <c r="E62" s="149"/>
+      <c r="F62" s="149"/>
+      <c r="G62" s="150"/>
+      <c r="H62" s="148" t="s">
         <v>81</v>
       </c>
-      <c r="I62" s="137"/>
-      <c r="J62" s="138"/>
+      <c r="I62" s="149"/>
+      <c r="J62" s="150"/>
       <c r="K62" s="81" t="s">
         <v>113</v>
       </c>
@@ -30013,19 +30013,19 @@
       <c r="AG63" s="92"/>
     </row>
     <row r="64" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B64" s="148" t="s">
+      <c r="B64" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C64" s="144"/>
-      <c r="D64" s="144"/>
-      <c r="E64" s="144"/>
-      <c r="F64" s="144"/>
-      <c r="G64" s="149"/>
-      <c r="H64" s="148" t="s">
+      <c r="C64" s="146"/>
+      <c r="D64" s="146"/>
+      <c r="E64" s="146"/>
+      <c r="F64" s="146"/>
+      <c r="G64" s="147"/>
+      <c r="H64" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I64" s="144"/>
-      <c r="J64" s="149"/>
+      <c r="I64" s="146"/>
+      <c r="J64" s="147"/>
       <c r="K64" s="83" t="s">
         <v>68</v>
       </c>
@@ -30054,18 +30054,18 @@
     </row>
     <row r="65" spans="2:33">
       <c r="B65" s="21"/>
-      <c r="C65" s="139" t="s">
+      <c r="C65" s="144" t="s">
         <v>114</v>
       </c>
-      <c r="D65" s="147"/>
-      <c r="E65" s="147"/>
-      <c r="F65" s="147"/>
-      <c r="G65" s="141"/>
-      <c r="H65" s="150" t="s">
+      <c r="D65" s="151"/>
+      <c r="E65" s="151"/>
+      <c r="F65" s="151"/>
+      <c r="G65" s="140"/>
+      <c r="H65" s="142" t="s">
         <v>69</v>
       </c>
-      <c r="I65" s="151"/>
-      <c r="J65" s="152"/>
+      <c r="I65" s="137"/>
+      <c r="J65" s="138"/>
       <c r="K65" s="19" t="s">
         <v>115</v>
       </c>
@@ -30085,18 +30085,18 @@
     </row>
     <row r="66" spans="2:33">
       <c r="B66" s="22"/>
-      <c r="C66" s="139" t="s">
+      <c r="C66" s="144" t="s">
         <v>116</v>
       </c>
-      <c r="D66" s="147"/>
-      <c r="E66" s="147"/>
-      <c r="F66" s="147"/>
-      <c r="G66" s="141"/>
-      <c r="H66" s="146" t="s">
+      <c r="D66" s="151"/>
+      <c r="E66" s="151"/>
+      <c r="F66" s="151"/>
+      <c r="G66" s="140"/>
+      <c r="H66" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I66" s="147"/>
-      <c r="J66" s="141"/>
+      <c r="I66" s="151"/>
+      <c r="J66" s="140"/>
       <c r="K66" s="19" t="s">
         <v>117</v>
       </c>
@@ -30116,18 +30116,18 @@
     </row>
     <row r="67" spans="2:33">
       <c r="B67" s="22"/>
-      <c r="C67" s="139" t="s">
+      <c r="C67" s="144" t="s">
         <v>9</v>
       </c>
-      <c r="D67" s="147"/>
-      <c r="E67" s="147"/>
-      <c r="F67" s="147"/>
-      <c r="G67" s="141"/>
-      <c r="H67" s="146" t="s">
+      <c r="D67" s="151"/>
+      <c r="E67" s="151"/>
+      <c r="F67" s="151"/>
+      <c r="G67" s="140"/>
+      <c r="H67" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I67" s="147"/>
-      <c r="J67" s="141"/>
+      <c r="I67" s="151"/>
+      <c r="J67" s="140"/>
       <c r="K67" s="19" t="s">
         <v>118</v>
       </c>
@@ -30147,18 +30147,18 @@
     </row>
     <row r="68" spans="2:33">
       <c r="B68" s="22"/>
-      <c r="C68" s="139" t="s">
+      <c r="C68" s="144" t="s">
         <v>119</v>
       </c>
-      <c r="D68" s="147"/>
-      <c r="E68" s="147"/>
-      <c r="F68" s="147"/>
-      <c r="G68" s="141"/>
-      <c r="H68" s="146" t="s">
+      <c r="D68" s="151"/>
+      <c r="E68" s="151"/>
+      <c r="F68" s="151"/>
+      <c r="G68" s="140"/>
+      <c r="H68" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I68" s="147"/>
-      <c r="J68" s="141"/>
+      <c r="I68" s="151"/>
+      <c r="J68" s="140"/>
       <c r="K68" s="19" t="s">
         <v>120</v>
       </c>
@@ -30178,18 +30178,18 @@
     </row>
     <row r="69" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
       <c r="B69" s="75"/>
-      <c r="C69" s="142" t="s">
+      <c r="C69" s="152" t="s">
         <v>121</v>
       </c>
-      <c r="D69" s="137"/>
-      <c r="E69" s="137"/>
-      <c r="F69" s="137"/>
-      <c r="G69" s="138"/>
-      <c r="H69" s="136" t="s">
+      <c r="D69" s="149"/>
+      <c r="E69" s="149"/>
+      <c r="F69" s="149"/>
+      <c r="G69" s="150"/>
+      <c r="H69" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="I69" s="137"/>
-      <c r="J69" s="138"/>
+      <c r="I69" s="149"/>
+      <c r="J69" s="150"/>
       <c r="K69" s="81" t="s">
         <v>122</v>
       </c>
@@ -30253,19 +30253,19 @@
       <c r="AG70" s="94"/>
     </row>
     <row r="71" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B71" s="148" t="s">
+      <c r="B71" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C71" s="144"/>
-      <c r="D71" s="144"/>
-      <c r="E71" s="144"/>
-      <c r="F71" s="144"/>
-      <c r="G71" s="149"/>
-      <c r="H71" s="148" t="s">
+      <c r="C71" s="146"/>
+      <c r="D71" s="146"/>
+      <c r="E71" s="146"/>
+      <c r="F71" s="146"/>
+      <c r="G71" s="147"/>
+      <c r="H71" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I71" s="144"/>
-      <c r="J71" s="149"/>
+      <c r="I71" s="146"/>
+      <c r="J71" s="147"/>
       <c r="K71" s="83" t="s">
         <v>68</v>
       </c>
@@ -30294,18 +30294,18 @@
     </row>
     <row r="72" spans="2:33">
       <c r="B72" s="21"/>
-      <c r="C72" s="139" t="s">
+      <c r="C72" s="144" t="s">
         <v>21</v>
       </c>
-      <c r="D72" s="147"/>
-      <c r="E72" s="147"/>
-      <c r="F72" s="147"/>
-      <c r="G72" s="141"/>
-      <c r="H72" s="150" t="s">
+      <c r="D72" s="151"/>
+      <c r="E72" s="151"/>
+      <c r="F72" s="151"/>
+      <c r="G72" s="140"/>
+      <c r="H72" s="142" t="s">
         <v>69</v>
       </c>
-      <c r="I72" s="151"/>
-      <c r="J72" s="152"/>
+      <c r="I72" s="137"/>
+      <c r="J72" s="138"/>
       <c r="K72" s="19" t="s">
         <v>123</v>
       </c>
@@ -30325,18 +30325,18 @@
     </row>
     <row r="73" spans="2:33">
       <c r="B73" s="22"/>
-      <c r="C73" s="139" t="s">
+      <c r="C73" s="144" t="s">
         <v>9</v>
       </c>
-      <c r="D73" s="147"/>
-      <c r="E73" s="147"/>
-      <c r="F73" s="147"/>
-      <c r="G73" s="141"/>
-      <c r="H73" s="146" t="s">
+      <c r="D73" s="151"/>
+      <c r="E73" s="151"/>
+      <c r="F73" s="151"/>
+      <c r="G73" s="140"/>
+      <c r="H73" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I73" s="147"/>
-      <c r="J73" s="141"/>
+      <c r="I73" s="151"/>
+      <c r="J73" s="140"/>
       <c r="K73" s="19" t="s">
         <v>124</v>
       </c>
@@ -30356,18 +30356,18 @@
     </row>
     <row r="74" spans="2:33">
       <c r="B74" s="22"/>
-      <c r="C74" s="139" t="s">
+      <c r="C74" s="144" t="s">
         <v>125</v>
       </c>
-      <c r="D74" s="147"/>
-      <c r="E74" s="147"/>
-      <c r="F74" s="147"/>
-      <c r="G74" s="141"/>
-      <c r="H74" s="146" t="s">
+      <c r="D74" s="151"/>
+      <c r="E74" s="151"/>
+      <c r="F74" s="151"/>
+      <c r="G74" s="140"/>
+      <c r="H74" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I74" s="147"/>
-      <c r="J74" s="141"/>
+      <c r="I74" s="151"/>
+      <c r="J74" s="140"/>
       <c r="K74" s="19" t="s">
         <v>126</v>
       </c>
@@ -30387,18 +30387,18 @@
     </row>
     <row r="75" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
       <c r="B75" s="75"/>
-      <c r="C75" s="142" t="s">
+      <c r="C75" s="152" t="s">
         <v>127</v>
       </c>
-      <c r="D75" s="137"/>
-      <c r="E75" s="137"/>
-      <c r="F75" s="137"/>
-      <c r="G75" s="138"/>
-      <c r="H75" s="136" t="s">
+      <c r="D75" s="149"/>
+      <c r="E75" s="149"/>
+      <c r="F75" s="149"/>
+      <c r="G75" s="150"/>
+      <c r="H75" s="148" t="s">
         <v>73</v>
       </c>
-      <c r="I75" s="137"/>
-      <c r="J75" s="138"/>
+      <c r="I75" s="149"/>
+      <c r="J75" s="150"/>
       <c r="K75" s="81" t="s">
         <v>128</v>
       </c>
@@ -30462,19 +30462,19 @@
       <c r="AG76" s="94"/>
     </row>
     <row r="77" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B77" s="148" t="s">
+      <c r="B77" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C77" s="144"/>
-      <c r="D77" s="144"/>
-      <c r="E77" s="144"/>
-      <c r="F77" s="144"/>
-      <c r="G77" s="149"/>
-      <c r="H77" s="148" t="s">
+      <c r="C77" s="146"/>
+      <c r="D77" s="146"/>
+      <c r="E77" s="146"/>
+      <c r="F77" s="146"/>
+      <c r="G77" s="147"/>
+      <c r="H77" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I77" s="144"/>
-      <c r="J77" s="149"/>
+      <c r="I77" s="146"/>
+      <c r="J77" s="147"/>
       <c r="K77" s="83" t="s">
         <v>68</v>
       </c>
@@ -30503,18 +30503,18 @@
     </row>
     <row r="78" spans="2:33">
       <c r="B78" s="21"/>
-      <c r="C78" s="139" t="s">
+      <c r="C78" s="144" t="s">
         <v>19</v>
       </c>
-      <c r="D78" s="147"/>
-      <c r="E78" s="147"/>
-      <c r="F78" s="147"/>
-      <c r="G78" s="141"/>
-      <c r="H78" s="150" t="s">
+      <c r="D78" s="151"/>
+      <c r="E78" s="151"/>
+      <c r="F78" s="151"/>
+      <c r="G78" s="140"/>
+      <c r="H78" s="142" t="s">
         <v>73</v>
       </c>
-      <c r="I78" s="151"/>
-      <c r="J78" s="152"/>
+      <c r="I78" s="137"/>
+      <c r="J78" s="138"/>
       <c r="K78" s="19" t="s">
         <v>129</v>
       </c>
@@ -30534,18 +30534,18 @@
     </row>
     <row r="79" spans="2:33">
       <c r="B79" s="22"/>
-      <c r="C79" s="139" t="s">
+      <c r="C79" s="144" t="s">
         <v>130</v>
       </c>
-      <c r="D79" s="147"/>
-      <c r="E79" s="147"/>
-      <c r="F79" s="147"/>
-      <c r="G79" s="141"/>
-      <c r="H79" s="146" t="s">
+      <c r="D79" s="151"/>
+      <c r="E79" s="151"/>
+      <c r="F79" s="151"/>
+      <c r="G79" s="140"/>
+      <c r="H79" s="141" t="s">
         <v>131</v>
       </c>
-      <c r="I79" s="147"/>
-      <c r="J79" s="141"/>
+      <c r="I79" s="151"/>
+      <c r="J79" s="140"/>
       <c r="K79" s="19" t="s">
         <v>132</v>
       </c>
@@ -30565,18 +30565,18 @@
     </row>
     <row r="80" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
       <c r="B80" s="75"/>
-      <c r="C80" s="142" t="s">
+      <c r="C80" s="152" t="s">
         <v>133</v>
       </c>
-      <c r="D80" s="137"/>
-      <c r="E80" s="137"/>
-      <c r="F80" s="137"/>
-      <c r="G80" s="138"/>
-      <c r="H80" s="136" t="s">
+      <c r="D80" s="149"/>
+      <c r="E80" s="149"/>
+      <c r="F80" s="149"/>
+      <c r="G80" s="150"/>
+      <c r="H80" s="148" t="s">
         <v>73</v>
       </c>
-      <c r="I80" s="137"/>
-      <c r="J80" s="138"/>
+      <c r="I80" s="149"/>
+      <c r="J80" s="150"/>
       <c r="K80" s="81" t="s">
         <v>134</v>
       </c>
@@ -30687,12 +30687,81 @@
     </row>
   </sheetData>
   <mergeCells count="97">
-    <mergeCell ref="C24:G25"/>
-    <mergeCell ref="H30:J30"/>
-    <mergeCell ref="H24:J25"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="H80:J80"/>
+    <mergeCell ref="C41:G41"/>
+    <mergeCell ref="H62:J62"/>
+    <mergeCell ref="C43:G43"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="H43:J43"/>
+    <mergeCell ref="H54:J54"/>
+    <mergeCell ref="H41:J41"/>
+    <mergeCell ref="C66:G66"/>
+    <mergeCell ref="C53:G53"/>
+    <mergeCell ref="B56:G56"/>
+    <mergeCell ref="H74:J74"/>
+    <mergeCell ref="H56:J56"/>
+    <mergeCell ref="H68:J68"/>
+    <mergeCell ref="H35:J35"/>
+    <mergeCell ref="C78:G78"/>
+    <mergeCell ref="H79:J79"/>
+    <mergeCell ref="H61:J61"/>
+    <mergeCell ref="C74:G74"/>
+    <mergeCell ref="C67:G67"/>
+    <mergeCell ref="C72:G72"/>
+    <mergeCell ref="H78:J78"/>
+    <mergeCell ref="H73:J73"/>
+    <mergeCell ref="H65:J65"/>
+    <mergeCell ref="H71:J71"/>
+    <mergeCell ref="H75:J75"/>
+    <mergeCell ref="C75:G75"/>
+    <mergeCell ref="B64:G64"/>
+    <mergeCell ref="H53:J53"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="C80:G80"/>
+    <mergeCell ref="H77:J77"/>
+    <mergeCell ref="B51:G51"/>
+    <mergeCell ref="C59:G59"/>
+    <mergeCell ref="H42:J42"/>
+    <mergeCell ref="C46:G46"/>
+    <mergeCell ref="C61:G61"/>
+    <mergeCell ref="H67:J67"/>
+    <mergeCell ref="H59:J59"/>
+    <mergeCell ref="B77:G77"/>
+    <mergeCell ref="H46:J46"/>
+    <mergeCell ref="H52:J52"/>
+    <mergeCell ref="C79:G79"/>
+    <mergeCell ref="C73:G73"/>
+    <mergeCell ref="H72:J72"/>
+    <mergeCell ref="C54:G54"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="C47:G49"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="C60:G60"/>
+    <mergeCell ref="C57:G57"/>
+    <mergeCell ref="C42:G42"/>
+    <mergeCell ref="C39:G39"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="B71:G71"/>
+    <mergeCell ref="B2:V2"/>
+    <mergeCell ref="B11:V11"/>
+    <mergeCell ref="C58:G58"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B5:V5"/>
+    <mergeCell ref="H47:J49"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="H34:J34"/>
+    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="H28:J28"/>
+    <mergeCell ref="H29:J29"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="H31:J31"/>
+    <mergeCell ref="H58:J58"/>
+    <mergeCell ref="H40:J40"/>
     <mergeCell ref="H51:J51"/>
     <mergeCell ref="H69:J69"/>
     <mergeCell ref="C29:G29"/>
@@ -30709,81 +30778,12 @@
     <mergeCell ref="C62:G62"/>
     <mergeCell ref="H32:J32"/>
     <mergeCell ref="B34:G34"/>
-    <mergeCell ref="B71:G71"/>
-    <mergeCell ref="B2:V2"/>
-    <mergeCell ref="B11:V11"/>
-    <mergeCell ref="C58:G58"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="B5:V5"/>
-    <mergeCell ref="H47:J49"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="H34:J34"/>
-    <mergeCell ref="H39:J39"/>
-    <mergeCell ref="H28:J28"/>
-    <mergeCell ref="H29:J29"/>
-    <mergeCell ref="H38:J38"/>
-    <mergeCell ref="H31:J31"/>
-    <mergeCell ref="H58:J58"/>
-    <mergeCell ref="H40:J40"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="C40:G40"/>
-    <mergeCell ref="C47:G49"/>
-    <mergeCell ref="B45:G45"/>
-    <mergeCell ref="C60:G60"/>
-    <mergeCell ref="C57:G57"/>
-    <mergeCell ref="C42:G42"/>
-    <mergeCell ref="C39:G39"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="C80:G80"/>
-    <mergeCell ref="H77:J77"/>
-    <mergeCell ref="B51:G51"/>
-    <mergeCell ref="C59:G59"/>
-    <mergeCell ref="H42:J42"/>
-    <mergeCell ref="C46:G46"/>
-    <mergeCell ref="C61:G61"/>
-    <mergeCell ref="H67:J67"/>
-    <mergeCell ref="H59:J59"/>
-    <mergeCell ref="B77:G77"/>
-    <mergeCell ref="H46:J46"/>
-    <mergeCell ref="H52:J52"/>
-    <mergeCell ref="C79:G79"/>
-    <mergeCell ref="C73:G73"/>
-    <mergeCell ref="H72:J72"/>
-    <mergeCell ref="C54:G54"/>
-    <mergeCell ref="H35:J35"/>
-    <mergeCell ref="C78:G78"/>
-    <mergeCell ref="H79:J79"/>
-    <mergeCell ref="H61:J61"/>
-    <mergeCell ref="C74:G74"/>
-    <mergeCell ref="C67:G67"/>
-    <mergeCell ref="C72:G72"/>
-    <mergeCell ref="H78:J78"/>
-    <mergeCell ref="H73:J73"/>
-    <mergeCell ref="H65:J65"/>
-    <mergeCell ref="H71:J71"/>
-    <mergeCell ref="H75:J75"/>
-    <mergeCell ref="C75:G75"/>
-    <mergeCell ref="B64:G64"/>
-    <mergeCell ref="H53:J53"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="H80:J80"/>
-    <mergeCell ref="C41:G41"/>
-    <mergeCell ref="H62:J62"/>
-    <mergeCell ref="C43:G43"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="H43:J43"/>
-    <mergeCell ref="H54:J54"/>
-    <mergeCell ref="H41:J41"/>
-    <mergeCell ref="C66:G66"/>
-    <mergeCell ref="C53:G53"/>
-    <mergeCell ref="B56:G56"/>
-    <mergeCell ref="H74:J74"/>
-    <mergeCell ref="H56:J56"/>
-    <mergeCell ref="H68:J68"/>
+    <mergeCell ref="C24:G25"/>
+    <mergeCell ref="H30:J30"/>
+    <mergeCell ref="H24:J25"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="H26:J26"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -69615,10 +69615,10 @@
       <c r="B2" s="162" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="151"/>
-      <c r="D2" s="151"/>
-      <c r="E2" s="151"/>
-      <c r="F2" s="151"/>
+      <c r="C2" s="137"/>
+      <c r="D2" s="137"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="137"/>
       <c r="G2" s="163"/>
       <c r="H2" s="11"/>
       <c r="I2" s="11"/>
@@ -69628,10 +69628,10 @@
       <c r="M2" s="165" t="s">
         <v>1</v>
       </c>
-      <c r="N2" s="144"/>
-      <c r="O2" s="144"/>
-      <c r="P2" s="144"/>
-      <c r="Q2" s="149"/>
+      <c r="N2" s="146"/>
+      <c r="O2" s="146"/>
+      <c r="P2" s="146"/>
+      <c r="Q2" s="147"/>
       <c r="R2" s="11"/>
       <c r="S2" s="11"/>
       <c r="T2" s="11"/>
@@ -69639,10 +69639,10 @@
       <c r="V2" s="165" t="s">
         <v>2</v>
       </c>
-      <c r="W2" s="144"/>
-      <c r="X2" s="144"/>
-      <c r="Y2" s="144"/>
-      <c r="Z2" s="149"/>
+      <c r="W2" s="146"/>
+      <c r="X2" s="146"/>
+      <c r="Y2" s="146"/>
+      <c r="Z2" s="147"/>
       <c r="AA2" s="11"/>
       <c r="AB2" s="11"/>
       <c r="AC2" s="10"/>
@@ -69761,10 +69761,10 @@
       <c r="V5" s="165" t="s">
         <v>10</v>
       </c>
-      <c r="W5" s="144"/>
-      <c r="X5" s="144"/>
-      <c r="Y5" s="144"/>
-      <c r="Z5" s="149"/>
+      <c r="W5" s="146"/>
+      <c r="X5" s="146"/>
+      <c r="Y5" s="146"/>
+      <c r="Z5" s="147"/>
       <c r="AA5" s="11"/>
       <c r="AB5" s="11"/>
       <c r="AC5" s="10"/>
@@ -69810,10 +69810,10 @@
       <c r="B7" s="165" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="144"/>
-      <c r="D7" s="144"/>
-      <c r="E7" s="144"/>
-      <c r="F7" s="149"/>
+      <c r="C7" s="146"/>
+      <c r="D7" s="146"/>
+      <c r="E7" s="146"/>
+      <c r="F7" s="147"/>
       <c r="G7" s="33"/>
       <c r="H7" s="33"/>
       <c r="I7" s="33"/>
@@ -69822,10 +69822,10 @@
       <c r="L7" s="165" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="144"/>
-      <c r="N7" s="144"/>
-      <c r="O7" s="144"/>
-      <c r="P7" s="149"/>
+      <c r="M7" s="146"/>
+      <c r="N7" s="146"/>
+      <c r="O7" s="146"/>
+      <c r="P7" s="147"/>
       <c r="Q7" s="11"/>
       <c r="R7" s="11"/>
       <c r="S7" s="11"/>
@@ -70034,10 +70034,10 @@
       <c r="AB14" s="164" t="s">
         <v>18</v>
       </c>
-      <c r="AC14" s="144"/>
-      <c r="AD14" s="144"/>
-      <c r="AE14" s="144"/>
-      <c r="AF14" s="149"/>
+      <c r="AC14" s="146"/>
+      <c r="AD14" s="146"/>
+      <c r="AE14" s="146"/>
+      <c r="AF14" s="147"/>
       <c r="AG14" s="100"/>
       <c r="AH14" s="45"/>
       <c r="AI14" s="12"/>
@@ -70111,10 +70111,10 @@
       <c r="AB17" s="164" t="s">
         <v>20</v>
       </c>
-      <c r="AC17" s="144"/>
-      <c r="AD17" s="144"/>
-      <c r="AE17" s="144"/>
-      <c r="AF17" s="149"/>
+      <c r="AC17" s="146"/>
+      <c r="AD17" s="146"/>
+      <c r="AE17" s="146"/>
+      <c r="AF17" s="147"/>
       <c r="AG17" s="102"/>
       <c r="AH17" s="38"/>
       <c r="AI17" s="10"/>
@@ -70232,10 +70232,10 @@
       <c r="AB21" s="164" t="s">
         <v>22</v>
       </c>
-      <c r="AC21" s="144"/>
-      <c r="AD21" s="144"/>
-      <c r="AE21" s="144"/>
-      <c r="AF21" s="149"/>
+      <c r="AC21" s="146"/>
+      <c r="AD21" s="146"/>
+      <c r="AE21" s="146"/>
+      <c r="AF21" s="147"/>
       <c r="AG21" s="116"/>
       <c r="AH21" s="117"/>
     </row>
@@ -71048,7 +71048,7 @@
         <v>781</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C7" t="s">
         <v>782</v>
@@ -71363,7 +71363,7 @@
         <v>754</v>
       </c>
       <c r="H4">
-        <v>0.21</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="5" spans="1:8">

</xml_diff>

<commit_message>
[MOD] 261016 BOSS_HP_K 5.0 → 1.0 (실측용, 사용자 결정)
</commit_message>
<xml_diff>
--- a/Assets/DB/MMM_DB_Ver.05.xlsx
+++ b/Assets/DB/MMM_DB_Ver.05.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\MoreMustMush-r3\Assets\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F6CACE-7DB9-4689-A4D7-1D0045D82701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A588FA7-6C26-41C5-B6D1-94C71F224D88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4500" yWindow="570" windowWidth="18900" windowHeight="13410" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27568,46 +27568,46 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -27616,12 +27616,12 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -28089,29 +28089,29 @@
   <sheetData>
     <row r="1" spans="2:44" ht="12" customHeight="1"/>
     <row r="2" spans="2:44">
-      <c r="B2" s="156" t="s">
+      <c r="B2" s="154" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="157"/>
-      <c r="D2" s="157"/>
-      <c r="E2" s="157"/>
-      <c r="F2" s="157"/>
-      <c r="G2" s="157"/>
-      <c r="H2" s="157"/>
-      <c r="I2" s="157"/>
-      <c r="J2" s="157"/>
-      <c r="K2" s="157"/>
-      <c r="L2" s="157"/>
-      <c r="M2" s="157"/>
-      <c r="N2" s="157"/>
-      <c r="O2" s="157"/>
-      <c r="P2" s="157"/>
-      <c r="Q2" s="157"/>
-      <c r="R2" s="157"/>
-      <c r="S2" s="157"/>
-      <c r="T2" s="157"/>
-      <c r="U2" s="157"/>
-      <c r="V2" s="158"/>
+      <c r="C2" s="155"/>
+      <c r="D2" s="155"/>
+      <c r="E2" s="155"/>
+      <c r="F2" s="155"/>
+      <c r="G2" s="155"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="155"/>
+      <c r="J2" s="155"/>
+      <c r="K2" s="155"/>
+      <c r="L2" s="155"/>
+      <c r="M2" s="155"/>
+      <c r="N2" s="155"/>
+      <c r="O2" s="155"/>
+      <c r="P2" s="155"/>
+      <c r="Q2" s="155"/>
+      <c r="R2" s="155"/>
+      <c r="S2" s="155"/>
+      <c r="T2" s="155"/>
+      <c r="U2" s="155"/>
+      <c r="V2" s="156"/>
     </row>
     <row r="3" spans="2:44">
       <c r="B3" s="17"/>
@@ -28168,29 +28168,29 @@
       <c r="V4" s="14"/>
     </row>
     <row r="5" spans="2:44">
-      <c r="B5" s="156" t="s">
+      <c r="B5" s="154" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="157"/>
-      <c r="D5" s="157"/>
-      <c r="E5" s="157"/>
-      <c r="F5" s="157"/>
-      <c r="G5" s="157"/>
-      <c r="H5" s="157"/>
-      <c r="I5" s="157"/>
-      <c r="J5" s="157"/>
-      <c r="K5" s="157"/>
-      <c r="L5" s="157"/>
-      <c r="M5" s="157"/>
-      <c r="N5" s="157"/>
-      <c r="O5" s="157"/>
-      <c r="P5" s="157"/>
-      <c r="Q5" s="157"/>
-      <c r="R5" s="157"/>
-      <c r="S5" s="157"/>
-      <c r="T5" s="157"/>
-      <c r="U5" s="157"/>
-      <c r="V5" s="158"/>
+      <c r="C5" s="155"/>
+      <c r="D5" s="155"/>
+      <c r="E5" s="155"/>
+      <c r="F5" s="155"/>
+      <c r="G5" s="155"/>
+      <c r="H5" s="155"/>
+      <c r="I5" s="155"/>
+      <c r="J5" s="155"/>
+      <c r="K5" s="155"/>
+      <c r="L5" s="155"/>
+      <c r="M5" s="155"/>
+      <c r="N5" s="155"/>
+      <c r="O5" s="155"/>
+      <c r="P5" s="155"/>
+      <c r="Q5" s="155"/>
+      <c r="R5" s="155"/>
+      <c r="S5" s="155"/>
+      <c r="T5" s="155"/>
+      <c r="U5" s="155"/>
+      <c r="V5" s="156"/>
     </row>
     <row r="6" spans="2:44">
       <c r="B6" s="6"/>
@@ -28320,29 +28320,29 @@
     </row>
     <row r="10" spans="2:44" ht="8.1" customHeight="1"/>
     <row r="11" spans="2:44">
-      <c r="B11" s="156" t="s">
+      <c r="B11" s="154" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="157"/>
-      <c r="D11" s="157"/>
-      <c r="E11" s="157"/>
-      <c r="F11" s="157"/>
-      <c r="G11" s="157"/>
-      <c r="H11" s="157"/>
-      <c r="I11" s="157"/>
-      <c r="J11" s="157"/>
-      <c r="K11" s="157"/>
-      <c r="L11" s="157"/>
-      <c r="M11" s="157"/>
-      <c r="N11" s="157"/>
-      <c r="O11" s="157"/>
-      <c r="P11" s="157"/>
-      <c r="Q11" s="157"/>
-      <c r="R11" s="157"/>
-      <c r="S11" s="157"/>
-      <c r="T11" s="157"/>
-      <c r="U11" s="157"/>
-      <c r="V11" s="158"/>
+      <c r="C11" s="155"/>
+      <c r="D11" s="155"/>
+      <c r="E11" s="155"/>
+      <c r="F11" s="155"/>
+      <c r="G11" s="155"/>
+      <c r="H11" s="155"/>
+      <c r="I11" s="155"/>
+      <c r="J11" s="155"/>
+      <c r="K11" s="155"/>
+      <c r="L11" s="155"/>
+      <c r="M11" s="155"/>
+      <c r="N11" s="155"/>
+      <c r="O11" s="155"/>
+      <c r="P11" s="155"/>
+      <c r="Q11" s="155"/>
+      <c r="R11" s="155"/>
+      <c r="S11" s="155"/>
+      <c r="T11" s="155"/>
+      <c r="U11" s="155"/>
+      <c r="V11" s="156"/>
     </row>
     <row r="12" spans="2:44">
       <c r="B12" s="6"/>
@@ -28629,19 +28629,19 @@
       <c r="AF22" s="27"/>
     </row>
     <row r="23" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B23" s="159" t="s">
+      <c r="B23" s="157" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="146"/>
-      <c r="D23" s="146"/>
-      <c r="E23" s="146"/>
-      <c r="F23" s="146"/>
-      <c r="G23" s="146"/>
-      <c r="H23" s="161" t="s">
+      <c r="C23" s="144"/>
+      <c r="D23" s="144"/>
+      <c r="E23" s="144"/>
+      <c r="F23" s="144"/>
+      <c r="G23" s="144"/>
+      <c r="H23" s="143" t="s">
         <v>67</v>
       </c>
-      <c r="I23" s="146"/>
-      <c r="J23" s="146"/>
+      <c r="I23" s="144"/>
+      <c r="J23" s="144"/>
       <c r="K23" s="28" t="s">
         <v>68</v>
       </c>
@@ -28669,18 +28669,18 @@
     </row>
     <row r="24" spans="2:32" s="10" customFormat="1">
       <c r="B24" s="86"/>
-      <c r="C24" s="136" t="s">
+      <c r="C24" s="153" t="s">
         <v>3</v>
       </c>
-      <c r="D24" s="137"/>
-      <c r="E24" s="137"/>
-      <c r="F24" s="137"/>
-      <c r="G24" s="138"/>
-      <c r="H24" s="142" t="s">
+      <c r="D24" s="151"/>
+      <c r="E24" s="151"/>
+      <c r="F24" s="151"/>
+      <c r="G24" s="152"/>
+      <c r="H24" s="150" t="s">
         <v>69</v>
       </c>
-      <c r="I24" s="137"/>
-      <c r="J24" s="138"/>
+      <c r="I24" s="151"/>
+      <c r="J24" s="152"/>
       <c r="K24" s="34" t="s">
         <v>70</v>
       </c>
@@ -28708,14 +28708,14 @@
     </row>
     <row r="25" spans="2:32" s="10" customFormat="1">
       <c r="B25" s="22"/>
-      <c r="C25" s="139"/>
-      <c r="D25" s="139"/>
-      <c r="E25" s="139"/>
-      <c r="F25" s="139"/>
-      <c r="G25" s="140"/>
-      <c r="H25" s="143"/>
-      <c r="I25" s="139"/>
-      <c r="J25" s="140"/>
+      <c r="C25" s="140"/>
+      <c r="D25" s="140"/>
+      <c r="E25" s="140"/>
+      <c r="F25" s="140"/>
+      <c r="G25" s="141"/>
+      <c r="H25" s="158"/>
+      <c r="I25" s="140"/>
+      <c r="J25" s="141"/>
       <c r="K25" s="19" t="s">
         <v>49</v>
       </c>
@@ -28737,18 +28737,18 @@
     </row>
     <row r="26" spans="2:32" s="10" customFormat="1">
       <c r="B26" s="22"/>
-      <c r="C26" s="144" t="s">
+      <c r="C26" s="139" t="s">
         <v>72</v>
       </c>
-      <c r="D26" s="139"/>
-      <c r="E26" s="139"/>
-      <c r="F26" s="139"/>
-      <c r="G26" s="140"/>
-      <c r="H26" s="141" t="s">
+      <c r="D26" s="140"/>
+      <c r="E26" s="140"/>
+      <c r="F26" s="140"/>
+      <c r="G26" s="141"/>
+      <c r="H26" s="146" t="s">
         <v>73</v>
       </c>
-      <c r="I26" s="139"/>
-      <c r="J26" s="140"/>
+      <c r="I26" s="140"/>
+      <c r="J26" s="141"/>
       <c r="K26" s="19" t="s">
         <v>74</v>
       </c>
@@ -28768,18 +28768,18 @@
     </row>
     <row r="27" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B27" s="22"/>
-      <c r="C27" s="144" t="s">
+      <c r="C27" s="139" t="s">
         <v>9</v>
       </c>
-      <c r="D27" s="139"/>
-      <c r="E27" s="139"/>
-      <c r="F27" s="139"/>
-      <c r="G27" s="140"/>
-      <c r="H27" s="141" t="s">
+      <c r="D27" s="140"/>
+      <c r="E27" s="140"/>
+      <c r="F27" s="140"/>
+      <c r="G27" s="141"/>
+      <c r="H27" s="146" t="s">
         <v>73</v>
       </c>
-      <c r="I27" s="139"/>
-      <c r="J27" s="140"/>
+      <c r="I27" s="140"/>
+      <c r="J27" s="141"/>
       <c r="K27" s="19" t="s">
         <v>75</v>
       </c>
@@ -28799,18 +28799,18 @@
     </row>
     <row r="28" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B28" s="22"/>
-      <c r="C28" s="144" t="s">
+      <c r="C28" s="139" t="s">
         <v>76</v>
       </c>
-      <c r="D28" s="139"/>
-      <c r="E28" s="139"/>
-      <c r="F28" s="139"/>
-      <c r="G28" s="140"/>
-      <c r="H28" s="141" t="s">
+      <c r="D28" s="140"/>
+      <c r="E28" s="140"/>
+      <c r="F28" s="140"/>
+      <c r="G28" s="141"/>
+      <c r="H28" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="I28" s="139"/>
-      <c r="J28" s="140"/>
+      <c r="I28" s="140"/>
+      <c r="J28" s="141"/>
       <c r="K28" s="19" t="s">
         <v>77</v>
       </c>
@@ -28830,18 +28830,18 @@
     </row>
     <row r="29" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B29" s="22"/>
-      <c r="C29" s="144" t="s">
+      <c r="C29" s="139" t="s">
         <v>67</v>
       </c>
-      <c r="D29" s="139"/>
-      <c r="E29" s="139"/>
-      <c r="F29" s="139"/>
-      <c r="G29" s="140"/>
-      <c r="H29" s="141" t="s">
+      <c r="D29" s="140"/>
+      <c r="E29" s="140"/>
+      <c r="F29" s="140"/>
+      <c r="G29" s="141"/>
+      <c r="H29" s="146" t="s">
         <v>73</v>
       </c>
-      <c r="I29" s="139"/>
-      <c r="J29" s="140"/>
+      <c r="I29" s="140"/>
+      <c r="J29" s="141"/>
       <c r="K29" s="19" t="s">
         <v>78</v>
       </c>
@@ -28861,18 +28861,18 @@
     </row>
     <row r="30" spans="2:32" s="10" customFormat="1">
       <c r="B30" s="22"/>
-      <c r="C30" s="144" t="s">
+      <c r="C30" s="139" t="s">
         <v>79</v>
       </c>
-      <c r="D30" s="139"/>
-      <c r="E30" s="139"/>
-      <c r="F30" s="139"/>
-      <c r="G30" s="140"/>
-      <c r="H30" s="141" t="s">
+      <c r="D30" s="140"/>
+      <c r="E30" s="140"/>
+      <c r="F30" s="140"/>
+      <c r="G30" s="141"/>
+      <c r="H30" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="I30" s="139"/>
-      <c r="J30" s="140"/>
+      <c r="I30" s="140"/>
+      <c r="J30" s="141"/>
       <c r="K30" s="120" t="s">
         <v>421</v>
       </c>
@@ -28892,18 +28892,18 @@
     </row>
     <row r="31" spans="2:32" s="10" customFormat="1">
       <c r="B31" s="22"/>
-      <c r="C31" s="144" t="s">
+      <c r="C31" s="139" t="s">
         <v>7</v>
       </c>
-      <c r="D31" s="139"/>
-      <c r="E31" s="139"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="140"/>
-      <c r="H31" s="141" t="s">
+      <c r="D31" s="140"/>
+      <c r="E31" s="140"/>
+      <c r="F31" s="140"/>
+      <c r="G31" s="141"/>
+      <c r="H31" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="I31" s="139"/>
-      <c r="J31" s="140"/>
+      <c r="I31" s="140"/>
+      <c r="J31" s="141"/>
       <c r="K31" s="19" t="s">
         <v>80</v>
       </c>
@@ -28923,18 +28923,18 @@
     </row>
     <row r="32" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B32" s="75"/>
-      <c r="C32" s="160" t="s">
+      <c r="C32" s="145" t="s">
         <v>422</v>
       </c>
-      <c r="D32" s="149"/>
-      <c r="E32" s="149"/>
-      <c r="F32" s="149"/>
-      <c r="G32" s="150"/>
-      <c r="H32" s="148" t="s">
+      <c r="D32" s="137"/>
+      <c r="E32" s="137"/>
+      <c r="F32" s="137"/>
+      <c r="G32" s="138"/>
+      <c r="H32" s="136" t="s">
         <v>81</v>
       </c>
-      <c r="I32" s="149"/>
-      <c r="J32" s="150"/>
+      <c r="I32" s="137"/>
+      <c r="J32" s="138"/>
       <c r="K32" s="81" t="s">
         <v>82</v>
       </c>
@@ -28996,19 +28996,19 @@
       <c r="AF33" s="27"/>
     </row>
     <row r="34" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B34" s="145" t="s">
+      <c r="B34" s="148" t="s">
         <v>66</v>
       </c>
-      <c r="C34" s="146"/>
-      <c r="D34" s="146"/>
-      <c r="E34" s="146"/>
-      <c r="F34" s="146"/>
-      <c r="G34" s="147"/>
-      <c r="H34" s="145" t="s">
+      <c r="C34" s="144"/>
+      <c r="D34" s="144"/>
+      <c r="E34" s="144"/>
+      <c r="F34" s="144"/>
+      <c r="G34" s="149"/>
+      <c r="H34" s="148" t="s">
         <v>67</v>
       </c>
-      <c r="I34" s="146"/>
-      <c r="J34" s="147"/>
+      <c r="I34" s="144"/>
+      <c r="J34" s="149"/>
       <c r="K34" s="28" t="s">
         <v>68</v>
       </c>
@@ -29036,18 +29036,18 @@
     </row>
     <row r="35" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B35" s="86"/>
-      <c r="C35" s="136" t="s">
+      <c r="C35" s="153" t="s">
         <v>7</v>
       </c>
-      <c r="D35" s="137"/>
-      <c r="E35" s="137"/>
-      <c r="F35" s="137"/>
-      <c r="G35" s="138"/>
-      <c r="H35" s="142" t="s">
+      <c r="D35" s="151"/>
+      <c r="E35" s="151"/>
+      <c r="F35" s="151"/>
+      <c r="G35" s="152"/>
+      <c r="H35" s="150" t="s">
         <v>69</v>
       </c>
-      <c r="I35" s="137"/>
-      <c r="J35" s="138"/>
+      <c r="I35" s="151"/>
+      <c r="J35" s="152"/>
       <c r="K35" s="34" t="s">
         <v>84</v>
       </c>
@@ -29075,18 +29075,18 @@
     </row>
     <row r="36" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B36" s="75"/>
-      <c r="C36" s="160" t="s">
+      <c r="C36" s="145" t="s">
         <v>423</v>
       </c>
-      <c r="D36" s="149"/>
-      <c r="E36" s="149"/>
-      <c r="F36" s="149"/>
-      <c r="G36" s="150"/>
-      <c r="H36" s="148" t="s">
+      <c r="D36" s="137"/>
+      <c r="E36" s="137"/>
+      <c r="F36" s="137"/>
+      <c r="G36" s="138"/>
+      <c r="H36" s="136" t="s">
         <v>69</v>
       </c>
-      <c r="I36" s="149"/>
-      <c r="J36" s="150"/>
+      <c r="I36" s="137"/>
+      <c r="J36" s="138"/>
       <c r="K36" s="81" t="s">
         <v>85</v>
       </c>
@@ -29148,19 +29148,19 @@
       <c r="AF37" s="92"/>
     </row>
     <row r="38" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B38" s="145" t="s">
+      <c r="B38" s="148" t="s">
         <v>66</v>
       </c>
-      <c r="C38" s="146"/>
-      <c r="D38" s="146"/>
-      <c r="E38" s="146"/>
-      <c r="F38" s="146"/>
-      <c r="G38" s="147"/>
-      <c r="H38" s="145" t="s">
+      <c r="C38" s="144"/>
+      <c r="D38" s="144"/>
+      <c r="E38" s="144"/>
+      <c r="F38" s="144"/>
+      <c r="G38" s="149"/>
+      <c r="H38" s="148" t="s">
         <v>67</v>
       </c>
-      <c r="I38" s="146"/>
-      <c r="J38" s="147"/>
+      <c r="I38" s="144"/>
+      <c r="J38" s="149"/>
       <c r="K38" s="28" t="s">
         <v>68</v>
       </c>
@@ -29188,18 +29188,18 @@
     </row>
     <row r="39" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B39" s="21"/>
-      <c r="C39" s="144" t="s">
+      <c r="C39" s="139" t="s">
         <v>14</v>
       </c>
-      <c r="D39" s="139"/>
-      <c r="E39" s="139"/>
-      <c r="F39" s="139"/>
-      <c r="G39" s="140"/>
-      <c r="H39" s="141" t="s">
+      <c r="D39" s="140"/>
+      <c r="E39" s="140"/>
+      <c r="F39" s="140"/>
+      <c r="G39" s="141"/>
+      <c r="H39" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="I39" s="139"/>
-      <c r="J39" s="140"/>
+      <c r="I39" s="140"/>
+      <c r="J39" s="141"/>
       <c r="K39" s="19" t="s">
         <v>86</v>
       </c>
@@ -29219,18 +29219,18 @@
     </row>
     <row r="40" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B40" s="22"/>
-      <c r="C40" s="144" t="s">
+      <c r="C40" s="139" t="s">
         <v>87</v>
       </c>
-      <c r="D40" s="139"/>
-      <c r="E40" s="139"/>
-      <c r="F40" s="139"/>
-      <c r="G40" s="140"/>
-      <c r="H40" s="141" t="s">
+      <c r="D40" s="140"/>
+      <c r="E40" s="140"/>
+      <c r="F40" s="140"/>
+      <c r="G40" s="141"/>
+      <c r="H40" s="146" t="s">
         <v>73</v>
       </c>
-      <c r="I40" s="139"/>
-      <c r="J40" s="140"/>
+      <c r="I40" s="140"/>
+      <c r="J40" s="141"/>
       <c r="K40" s="19" t="s">
         <v>88</v>
       </c>
@@ -29250,18 +29250,18 @@
     </row>
     <row r="41" spans="2:32" s="10" customFormat="1">
       <c r="B41" s="22"/>
-      <c r="C41" s="144" t="s">
+      <c r="C41" s="139" t="s">
         <v>16</v>
       </c>
-      <c r="D41" s="139"/>
-      <c r="E41" s="139"/>
-      <c r="F41" s="139"/>
-      <c r="G41" s="140"/>
-      <c r="H41" s="141" t="s">
+      <c r="D41" s="140"/>
+      <c r="E41" s="140"/>
+      <c r="F41" s="140"/>
+      <c r="G41" s="141"/>
+      <c r="H41" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="I41" s="139"/>
-      <c r="J41" s="140"/>
+      <c r="I41" s="140"/>
+      <c r="J41" s="141"/>
       <c r="K41" s="19" t="s">
         <v>89</v>
       </c>
@@ -29281,18 +29281,18 @@
     </row>
     <row r="42" spans="2:32" s="10" customFormat="1">
       <c r="B42" s="22"/>
-      <c r="C42" s="144" t="s">
+      <c r="C42" s="139" t="s">
         <v>90</v>
       </c>
-      <c r="D42" s="139"/>
-      <c r="E42" s="139"/>
-      <c r="F42" s="139"/>
-      <c r="G42" s="140"/>
-      <c r="H42" s="141" t="s">
+      <c r="D42" s="140"/>
+      <c r="E42" s="140"/>
+      <c r="F42" s="140"/>
+      <c r="G42" s="141"/>
+      <c r="H42" s="146" t="s">
         <v>73</v>
       </c>
-      <c r="I42" s="139"/>
-      <c r="J42" s="140"/>
+      <c r="I42" s="140"/>
+      <c r="J42" s="141"/>
       <c r="K42" s="19" t="s">
         <v>91</v>
       </c>
@@ -29312,18 +29312,18 @@
     </row>
     <row r="43" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B43" s="75"/>
-      <c r="C43" s="152" t="s">
+      <c r="C43" s="142" t="s">
         <v>15</v>
       </c>
-      <c r="D43" s="149"/>
-      <c r="E43" s="149"/>
-      <c r="F43" s="149"/>
-      <c r="G43" s="150"/>
-      <c r="H43" s="148" t="s">
+      <c r="D43" s="137"/>
+      <c r="E43" s="137"/>
+      <c r="F43" s="137"/>
+      <c r="G43" s="138"/>
+      <c r="H43" s="136" t="s">
         <v>73</v>
       </c>
-      <c r="I43" s="149"/>
-      <c r="J43" s="150"/>
+      <c r="I43" s="137"/>
+      <c r="J43" s="138"/>
       <c r="K43" s="81" t="s">
         <v>92</v>
       </c>
@@ -29385,19 +29385,19 @@
       <c r="AF44" s="27"/>
     </row>
     <row r="45" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B45" s="145" t="s">
+      <c r="B45" s="148" t="s">
         <v>66</v>
       </c>
-      <c r="C45" s="146"/>
-      <c r="D45" s="146"/>
-      <c r="E45" s="146"/>
-      <c r="F45" s="146"/>
-      <c r="G45" s="147"/>
-      <c r="H45" s="153" t="s">
+      <c r="C45" s="144"/>
+      <c r="D45" s="144"/>
+      <c r="E45" s="144"/>
+      <c r="F45" s="144"/>
+      <c r="G45" s="149"/>
+      <c r="H45" s="159" t="s">
         <v>67</v>
       </c>
-      <c r="I45" s="154"/>
-      <c r="J45" s="155"/>
+      <c r="I45" s="160"/>
+      <c r="J45" s="161"/>
       <c r="K45" s="83" t="s">
         <v>68</v>
       </c>
@@ -29425,18 +29425,18 @@
     </row>
     <row r="46" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B46" s="21"/>
-      <c r="C46" s="144" t="s">
+      <c r="C46" s="139" t="s">
         <v>15</v>
       </c>
-      <c r="D46" s="139"/>
-      <c r="E46" s="139"/>
-      <c r="F46" s="139"/>
-      <c r="G46" s="140"/>
-      <c r="H46" s="142" t="s">
+      <c r="D46" s="140"/>
+      <c r="E46" s="140"/>
+      <c r="F46" s="140"/>
+      <c r="G46" s="141"/>
+      <c r="H46" s="150" t="s">
         <v>73</v>
       </c>
-      <c r="I46" s="137"/>
-      <c r="J46" s="138"/>
+      <c r="I46" s="151"/>
+      <c r="J46" s="152"/>
       <c r="K46" s="19" t="s">
         <v>93</v>
       </c>
@@ -29456,18 +29456,18 @@
     </row>
     <row r="47" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B47" s="22"/>
-      <c r="C47" s="144" t="s">
+      <c r="C47" s="139" t="s">
         <v>94</v>
       </c>
-      <c r="D47" s="139"/>
-      <c r="E47" s="139"/>
-      <c r="F47" s="139"/>
-      <c r="G47" s="140"/>
-      <c r="H47" s="141" t="s">
+      <c r="D47" s="140"/>
+      <c r="E47" s="140"/>
+      <c r="F47" s="140"/>
+      <c r="G47" s="141"/>
+      <c r="H47" s="146" t="s">
         <v>81</v>
       </c>
-      <c r="I47" s="139"/>
-      <c r="J47" s="140"/>
+      <c r="I47" s="140"/>
+      <c r="J47" s="141"/>
       <c r="K47" s="19" t="s">
         <v>95</v>
       </c>
@@ -29487,14 +29487,14 @@
     </row>
     <row r="48" spans="2:32" s="10" customFormat="1">
       <c r="B48" s="22"/>
-      <c r="C48" s="139"/>
-      <c r="D48" s="139"/>
-      <c r="E48" s="139"/>
-      <c r="F48" s="139"/>
-      <c r="G48" s="140"/>
-      <c r="H48" s="143"/>
-      <c r="I48" s="139"/>
-      <c r="J48" s="140"/>
+      <c r="C48" s="140"/>
+      <c r="D48" s="140"/>
+      <c r="E48" s="140"/>
+      <c r="F48" s="140"/>
+      <c r="G48" s="141"/>
+      <c r="H48" s="158"/>
+      <c r="I48" s="140"/>
+      <c r="J48" s="141"/>
       <c r="K48" s="19" t="s">
         <v>49</v>
       </c>
@@ -29516,14 +29516,14 @@
     </row>
     <row r="49" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B49" s="22"/>
-      <c r="C49" s="139"/>
-      <c r="D49" s="139"/>
-      <c r="E49" s="139"/>
-      <c r="F49" s="139"/>
-      <c r="G49" s="140"/>
-      <c r="H49" s="143"/>
-      <c r="I49" s="139"/>
-      <c r="J49" s="140"/>
+      <c r="C49" s="140"/>
+      <c r="D49" s="140"/>
+      <c r="E49" s="140"/>
+      <c r="F49" s="140"/>
+      <c r="G49" s="141"/>
+      <c r="H49" s="158"/>
+      <c r="I49" s="140"/>
+      <c r="J49" s="141"/>
       <c r="K49" s="19" t="s">
         <v>49</v>
       </c>
@@ -29580,19 +29580,19 @@
       <c r="AG50" s="92"/>
     </row>
     <row r="51" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B51" s="145" t="s">
+      <c r="B51" s="148" t="s">
         <v>66</v>
       </c>
-      <c r="C51" s="146"/>
-      <c r="D51" s="146"/>
-      <c r="E51" s="146"/>
-      <c r="F51" s="146"/>
-      <c r="G51" s="147"/>
-      <c r="H51" s="145" t="s">
+      <c r="C51" s="144"/>
+      <c r="D51" s="144"/>
+      <c r="E51" s="144"/>
+      <c r="F51" s="144"/>
+      <c r="G51" s="149"/>
+      <c r="H51" s="148" t="s">
         <v>67</v>
       </c>
-      <c r="I51" s="146"/>
-      <c r="J51" s="147"/>
+      <c r="I51" s="144"/>
+      <c r="J51" s="149"/>
       <c r="K51" s="28" t="s">
         <v>68</v>
       </c>
@@ -29621,18 +29621,18 @@
     </row>
     <row r="52" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B52" s="21"/>
-      <c r="C52" s="144" t="s">
+      <c r="C52" s="139" t="s">
         <v>23</v>
       </c>
-      <c r="D52" s="139"/>
-      <c r="E52" s="139"/>
-      <c r="F52" s="139"/>
-      <c r="G52" s="140"/>
-      <c r="H52" s="141" t="s">
+      <c r="D52" s="140"/>
+      <c r="E52" s="140"/>
+      <c r="F52" s="140"/>
+      <c r="G52" s="141"/>
+      <c r="H52" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="I52" s="139"/>
-      <c r="J52" s="140"/>
+      <c r="I52" s="140"/>
+      <c r="J52" s="141"/>
       <c r="K52" s="19" t="s">
         <v>99</v>
       </c>
@@ -29652,18 +29652,18 @@
     </row>
     <row r="53" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B53" s="22"/>
-      <c r="C53" s="144" t="s">
+      <c r="C53" s="139" t="s">
         <v>100</v>
       </c>
-      <c r="D53" s="139"/>
-      <c r="E53" s="139"/>
-      <c r="F53" s="139"/>
-      <c r="G53" s="140"/>
-      <c r="H53" s="141" t="s">
+      <c r="D53" s="140"/>
+      <c r="E53" s="140"/>
+      <c r="F53" s="140"/>
+      <c r="G53" s="141"/>
+      <c r="H53" s="146" t="s">
         <v>73</v>
       </c>
-      <c r="I53" s="139"/>
-      <c r="J53" s="140"/>
+      <c r="I53" s="140"/>
+      <c r="J53" s="141"/>
       <c r="K53" s="19" t="s">
         <v>101</v>
       </c>
@@ -29683,18 +29683,18 @@
     </row>
     <row r="54" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B54" s="75"/>
-      <c r="C54" s="152" t="s">
+      <c r="C54" s="142" t="s">
         <v>102</v>
       </c>
-      <c r="D54" s="149"/>
-      <c r="E54" s="149"/>
-      <c r="F54" s="149"/>
-      <c r="G54" s="150"/>
-      <c r="H54" s="148" t="s">
+      <c r="D54" s="137"/>
+      <c r="E54" s="137"/>
+      <c r="F54" s="137"/>
+      <c r="G54" s="138"/>
+      <c r="H54" s="136" t="s">
         <v>73</v>
       </c>
-      <c r="I54" s="149"/>
-      <c r="J54" s="150"/>
+      <c r="I54" s="137"/>
+      <c r="J54" s="138"/>
       <c r="K54" s="81" t="s">
         <v>103</v>
       </c>
@@ -29758,19 +29758,19 @@
       <c r="AG55" s="92"/>
     </row>
     <row r="56" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B56" s="145" t="s">
+      <c r="B56" s="148" t="s">
         <v>66</v>
       </c>
-      <c r="C56" s="146"/>
-      <c r="D56" s="146"/>
-      <c r="E56" s="146"/>
-      <c r="F56" s="146"/>
-      <c r="G56" s="147"/>
-      <c r="H56" s="145" t="s">
+      <c r="C56" s="144"/>
+      <c r="D56" s="144"/>
+      <c r="E56" s="144"/>
+      <c r="F56" s="144"/>
+      <c r="G56" s="149"/>
+      <c r="H56" s="148" t="s">
         <v>67</v>
       </c>
-      <c r="I56" s="146"/>
-      <c r="J56" s="147"/>
+      <c r="I56" s="144"/>
+      <c r="J56" s="149"/>
       <c r="K56" s="28" t="s">
         <v>68</v>
       </c>
@@ -29799,18 +29799,18 @@
     </row>
     <row r="57" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B57" s="21"/>
-      <c r="C57" s="144" t="s">
+      <c r="C57" s="139" t="s">
         <v>6</v>
       </c>
-      <c r="D57" s="139"/>
-      <c r="E57" s="139"/>
-      <c r="F57" s="139"/>
-      <c r="G57" s="140"/>
-      <c r="H57" s="141" t="s">
+      <c r="D57" s="140"/>
+      <c r="E57" s="140"/>
+      <c r="F57" s="140"/>
+      <c r="G57" s="141"/>
+      <c r="H57" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="I57" s="139"/>
-      <c r="J57" s="140"/>
+      <c r="I57" s="140"/>
+      <c r="J57" s="141"/>
       <c r="K57" s="19" t="s">
         <v>104</v>
       </c>
@@ -29830,18 +29830,18 @@
     </row>
     <row r="58" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B58" s="22"/>
-      <c r="C58" s="144" t="s">
+      <c r="C58" s="139" t="s">
         <v>105</v>
       </c>
-      <c r="D58" s="139"/>
-      <c r="E58" s="139"/>
-      <c r="F58" s="139"/>
-      <c r="G58" s="140"/>
-      <c r="H58" s="141" t="s">
+      <c r="D58" s="140"/>
+      <c r="E58" s="140"/>
+      <c r="F58" s="140"/>
+      <c r="G58" s="141"/>
+      <c r="H58" s="146" t="s">
         <v>73</v>
       </c>
-      <c r="I58" s="139"/>
-      <c r="J58" s="140"/>
+      <c r="I58" s="140"/>
+      <c r="J58" s="141"/>
       <c r="K58" s="19" t="s">
         <v>106</v>
       </c>
@@ -29861,18 +29861,18 @@
     </row>
     <row r="59" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B59" s="22"/>
-      <c r="C59" s="144" t="s">
+      <c r="C59" s="139" t="s">
         <v>9</v>
       </c>
-      <c r="D59" s="139"/>
-      <c r="E59" s="139"/>
-      <c r="F59" s="139"/>
-      <c r="G59" s="140"/>
-      <c r="H59" s="141" t="s">
+      <c r="D59" s="140"/>
+      <c r="E59" s="140"/>
+      <c r="F59" s="140"/>
+      <c r="G59" s="141"/>
+      <c r="H59" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="I59" s="139"/>
-      <c r="J59" s="140"/>
+      <c r="I59" s="140"/>
+      <c r="J59" s="141"/>
       <c r="K59" s="19" t="s">
         <v>107</v>
       </c>
@@ -29892,18 +29892,18 @@
     </row>
     <row r="60" spans="2:33" s="10" customFormat="1">
       <c r="B60" s="22"/>
-      <c r="C60" s="144" t="s">
+      <c r="C60" s="139" t="s">
         <v>108</v>
       </c>
-      <c r="D60" s="139"/>
-      <c r="E60" s="139"/>
-      <c r="F60" s="139"/>
-      <c r="G60" s="140"/>
-      <c r="H60" s="141" t="s">
+      <c r="D60" s="140"/>
+      <c r="E60" s="140"/>
+      <c r="F60" s="140"/>
+      <c r="G60" s="141"/>
+      <c r="H60" s="146" t="s">
         <v>73</v>
       </c>
-      <c r="I60" s="139"/>
-      <c r="J60" s="140"/>
+      <c r="I60" s="140"/>
+      <c r="J60" s="141"/>
       <c r="K60" s="19" t="s">
         <v>109</v>
       </c>
@@ -29923,18 +29923,18 @@
     </row>
     <row r="61" spans="2:33" s="10" customFormat="1">
       <c r="B61" s="22"/>
-      <c r="C61" s="144" t="s">
+      <c r="C61" s="139" t="s">
         <v>110</v>
       </c>
-      <c r="D61" s="139"/>
-      <c r="E61" s="139"/>
-      <c r="F61" s="139"/>
-      <c r="G61" s="140"/>
-      <c r="H61" s="141" t="s">
+      <c r="D61" s="140"/>
+      <c r="E61" s="140"/>
+      <c r="F61" s="140"/>
+      <c r="G61" s="141"/>
+      <c r="H61" s="146" t="s">
         <v>73</v>
       </c>
-      <c r="I61" s="139"/>
-      <c r="J61" s="140"/>
+      <c r="I61" s="140"/>
+      <c r="J61" s="141"/>
       <c r="K61" s="19" t="s">
         <v>111</v>
       </c>
@@ -29954,18 +29954,18 @@
     </row>
     <row r="62" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B62" s="75"/>
-      <c r="C62" s="152" t="s">
+      <c r="C62" s="142" t="s">
         <v>112</v>
       </c>
-      <c r="D62" s="149"/>
-      <c r="E62" s="149"/>
-      <c r="F62" s="149"/>
-      <c r="G62" s="150"/>
-      <c r="H62" s="148" t="s">
+      <c r="D62" s="137"/>
+      <c r="E62" s="137"/>
+      <c r="F62" s="137"/>
+      <c r="G62" s="138"/>
+      <c r="H62" s="136" t="s">
         <v>81</v>
       </c>
-      <c r="I62" s="149"/>
-      <c r="J62" s="150"/>
+      <c r="I62" s="137"/>
+      <c r="J62" s="138"/>
       <c r="K62" s="81" t="s">
         <v>113</v>
       </c>
@@ -30029,19 +30029,19 @@
       <c r="AG63" s="92"/>
     </row>
     <row r="64" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B64" s="145" t="s">
+      <c r="B64" s="148" t="s">
         <v>66</v>
       </c>
-      <c r="C64" s="146"/>
-      <c r="D64" s="146"/>
-      <c r="E64" s="146"/>
-      <c r="F64" s="146"/>
-      <c r="G64" s="147"/>
-      <c r="H64" s="145" t="s">
+      <c r="C64" s="144"/>
+      <c r="D64" s="144"/>
+      <c r="E64" s="144"/>
+      <c r="F64" s="144"/>
+      <c r="G64" s="149"/>
+      <c r="H64" s="148" t="s">
         <v>67</v>
       </c>
-      <c r="I64" s="146"/>
-      <c r="J64" s="147"/>
+      <c r="I64" s="144"/>
+      <c r="J64" s="149"/>
       <c r="K64" s="83" t="s">
         <v>68</v>
       </c>
@@ -30070,18 +30070,18 @@
     </row>
     <row r="65" spans="2:33">
       <c r="B65" s="21"/>
-      <c r="C65" s="144" t="s">
+      <c r="C65" s="139" t="s">
         <v>114</v>
       </c>
-      <c r="D65" s="151"/>
-      <c r="E65" s="151"/>
-      <c r="F65" s="151"/>
-      <c r="G65" s="140"/>
-      <c r="H65" s="142" t="s">
+      <c r="D65" s="147"/>
+      <c r="E65" s="147"/>
+      <c r="F65" s="147"/>
+      <c r="G65" s="141"/>
+      <c r="H65" s="150" t="s">
         <v>69</v>
       </c>
-      <c r="I65" s="137"/>
-      <c r="J65" s="138"/>
+      <c r="I65" s="151"/>
+      <c r="J65" s="152"/>
       <c r="K65" s="19" t="s">
         <v>115</v>
       </c>
@@ -30101,18 +30101,18 @@
     </row>
     <row r="66" spans="2:33">
       <c r="B66" s="22"/>
-      <c r="C66" s="144" t="s">
+      <c r="C66" s="139" t="s">
         <v>116</v>
       </c>
-      <c r="D66" s="151"/>
-      <c r="E66" s="151"/>
-      <c r="F66" s="151"/>
-      <c r="G66" s="140"/>
-      <c r="H66" s="141" t="s">
+      <c r="D66" s="147"/>
+      <c r="E66" s="147"/>
+      <c r="F66" s="147"/>
+      <c r="G66" s="141"/>
+      <c r="H66" s="146" t="s">
         <v>73</v>
       </c>
-      <c r="I66" s="151"/>
-      <c r="J66" s="140"/>
+      <c r="I66" s="147"/>
+      <c r="J66" s="141"/>
       <c r="K66" s="19" t="s">
         <v>117</v>
       </c>
@@ -30132,18 +30132,18 @@
     </row>
     <row r="67" spans="2:33">
       <c r="B67" s="22"/>
-      <c r="C67" s="144" t="s">
+      <c r="C67" s="139" t="s">
         <v>9</v>
       </c>
-      <c r="D67" s="151"/>
-      <c r="E67" s="151"/>
-      <c r="F67" s="151"/>
-      <c r="G67" s="140"/>
-      <c r="H67" s="141" t="s">
+      <c r="D67" s="147"/>
+      <c r="E67" s="147"/>
+      <c r="F67" s="147"/>
+      <c r="G67" s="141"/>
+      <c r="H67" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="I67" s="151"/>
-      <c r="J67" s="140"/>
+      <c r="I67" s="147"/>
+      <c r="J67" s="141"/>
       <c r="K67" s="19" t="s">
         <v>118</v>
       </c>
@@ -30163,18 +30163,18 @@
     </row>
     <row r="68" spans="2:33">
       <c r="B68" s="22"/>
-      <c r="C68" s="144" t="s">
+      <c r="C68" s="139" t="s">
         <v>119</v>
       </c>
-      <c r="D68" s="151"/>
-      <c r="E68" s="151"/>
-      <c r="F68" s="151"/>
-      <c r="G68" s="140"/>
-      <c r="H68" s="141" t="s">
+      <c r="D68" s="147"/>
+      <c r="E68" s="147"/>
+      <c r="F68" s="147"/>
+      <c r="G68" s="141"/>
+      <c r="H68" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="I68" s="151"/>
-      <c r="J68" s="140"/>
+      <c r="I68" s="147"/>
+      <c r="J68" s="141"/>
       <c r="K68" s="19" t="s">
         <v>120</v>
       </c>
@@ -30194,18 +30194,18 @@
     </row>
     <row r="69" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
       <c r="B69" s="75"/>
-      <c r="C69" s="152" t="s">
+      <c r="C69" s="142" t="s">
         <v>121</v>
       </c>
-      <c r="D69" s="149"/>
-      <c r="E69" s="149"/>
-      <c r="F69" s="149"/>
-      <c r="G69" s="150"/>
-      <c r="H69" s="148" t="s">
+      <c r="D69" s="137"/>
+      <c r="E69" s="137"/>
+      <c r="F69" s="137"/>
+      <c r="G69" s="138"/>
+      <c r="H69" s="136" t="s">
         <v>69</v>
       </c>
-      <c r="I69" s="149"/>
-      <c r="J69" s="150"/>
+      <c r="I69" s="137"/>
+      <c r="J69" s="138"/>
       <c r="K69" s="81" t="s">
         <v>122</v>
       </c>
@@ -30269,19 +30269,19 @@
       <c r="AG70" s="94"/>
     </row>
     <row r="71" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B71" s="145" t="s">
+      <c r="B71" s="148" t="s">
         <v>66</v>
       </c>
-      <c r="C71" s="146"/>
-      <c r="D71" s="146"/>
-      <c r="E71" s="146"/>
-      <c r="F71" s="146"/>
-      <c r="G71" s="147"/>
-      <c r="H71" s="145" t="s">
+      <c r="C71" s="144"/>
+      <c r="D71" s="144"/>
+      <c r="E71" s="144"/>
+      <c r="F71" s="144"/>
+      <c r="G71" s="149"/>
+      <c r="H71" s="148" t="s">
         <v>67</v>
       </c>
-      <c r="I71" s="146"/>
-      <c r="J71" s="147"/>
+      <c r="I71" s="144"/>
+      <c r="J71" s="149"/>
       <c r="K71" s="83" t="s">
         <v>68</v>
       </c>
@@ -30310,18 +30310,18 @@
     </row>
     <row r="72" spans="2:33">
       <c r="B72" s="21"/>
-      <c r="C72" s="144" t="s">
+      <c r="C72" s="139" t="s">
         <v>21</v>
       </c>
-      <c r="D72" s="151"/>
-      <c r="E72" s="151"/>
-      <c r="F72" s="151"/>
-      <c r="G72" s="140"/>
-      <c r="H72" s="142" t="s">
+      <c r="D72" s="147"/>
+      <c r="E72" s="147"/>
+      <c r="F72" s="147"/>
+      <c r="G72" s="141"/>
+      <c r="H72" s="150" t="s">
         <v>69</v>
       </c>
-      <c r="I72" s="137"/>
-      <c r="J72" s="138"/>
+      <c r="I72" s="151"/>
+      <c r="J72" s="152"/>
       <c r="K72" s="19" t="s">
         <v>123</v>
       </c>
@@ -30341,18 +30341,18 @@
     </row>
     <row r="73" spans="2:33">
       <c r="B73" s="22"/>
-      <c r="C73" s="144" t="s">
+      <c r="C73" s="139" t="s">
         <v>9</v>
       </c>
-      <c r="D73" s="151"/>
-      <c r="E73" s="151"/>
-      <c r="F73" s="151"/>
-      <c r="G73" s="140"/>
-      <c r="H73" s="141" t="s">
+      <c r="D73" s="147"/>
+      <c r="E73" s="147"/>
+      <c r="F73" s="147"/>
+      <c r="G73" s="141"/>
+      <c r="H73" s="146" t="s">
         <v>69</v>
       </c>
-      <c r="I73" s="151"/>
-      <c r="J73" s="140"/>
+      <c r="I73" s="147"/>
+      <c r="J73" s="141"/>
       <c r="K73" s="19" t="s">
         <v>124</v>
       </c>
@@ -30372,18 +30372,18 @@
     </row>
     <row r="74" spans="2:33">
       <c r="B74" s="22"/>
-      <c r="C74" s="144" t="s">
+      <c r="C74" s="139" t="s">
         <v>125</v>
       </c>
-      <c r="D74" s="151"/>
-      <c r="E74" s="151"/>
-      <c r="F74" s="151"/>
-      <c r="G74" s="140"/>
-      <c r="H74" s="141" t="s">
+      <c r="D74" s="147"/>
+      <c r="E74" s="147"/>
+      <c r="F74" s="147"/>
+      <c r="G74" s="141"/>
+      <c r="H74" s="146" t="s">
         <v>73</v>
       </c>
-      <c r="I74" s="151"/>
-      <c r="J74" s="140"/>
+      <c r="I74" s="147"/>
+      <c r="J74" s="141"/>
       <c r="K74" s="19" t="s">
         <v>126</v>
       </c>
@@ -30403,18 +30403,18 @@
     </row>
     <row r="75" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
       <c r="B75" s="75"/>
-      <c r="C75" s="152" t="s">
+      <c r="C75" s="142" t="s">
         <v>127</v>
       </c>
-      <c r="D75" s="149"/>
-      <c r="E75" s="149"/>
-      <c r="F75" s="149"/>
-      <c r="G75" s="150"/>
-      <c r="H75" s="148" t="s">
+      <c r="D75" s="137"/>
+      <c r="E75" s="137"/>
+      <c r="F75" s="137"/>
+      <c r="G75" s="138"/>
+      <c r="H75" s="136" t="s">
         <v>73</v>
       </c>
-      <c r="I75" s="149"/>
-      <c r="J75" s="150"/>
+      <c r="I75" s="137"/>
+      <c r="J75" s="138"/>
       <c r="K75" s="81" t="s">
         <v>128</v>
       </c>
@@ -30478,19 +30478,19 @@
       <c r="AG76" s="94"/>
     </row>
     <row r="77" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B77" s="145" t="s">
+      <c r="B77" s="148" t="s">
         <v>66</v>
       </c>
-      <c r="C77" s="146"/>
-      <c r="D77" s="146"/>
-      <c r="E77" s="146"/>
-      <c r="F77" s="146"/>
-      <c r="G77" s="147"/>
-      <c r="H77" s="145" t="s">
+      <c r="C77" s="144"/>
+      <c r="D77" s="144"/>
+      <c r="E77" s="144"/>
+      <c r="F77" s="144"/>
+      <c r="G77" s="149"/>
+      <c r="H77" s="148" t="s">
         <v>67</v>
       </c>
-      <c r="I77" s="146"/>
-      <c r="J77" s="147"/>
+      <c r="I77" s="144"/>
+      <c r="J77" s="149"/>
       <c r="K77" s="83" t="s">
         <v>68</v>
       </c>
@@ -30519,18 +30519,18 @@
     </row>
     <row r="78" spans="2:33">
       <c r="B78" s="21"/>
-      <c r="C78" s="144" t="s">
+      <c r="C78" s="139" t="s">
         <v>19</v>
       </c>
-      <c r="D78" s="151"/>
-      <c r="E78" s="151"/>
-      <c r="F78" s="151"/>
-      <c r="G78" s="140"/>
-      <c r="H78" s="142" t="s">
+      <c r="D78" s="147"/>
+      <c r="E78" s="147"/>
+      <c r="F78" s="147"/>
+      <c r="G78" s="141"/>
+      <c r="H78" s="150" t="s">
         <v>73</v>
       </c>
-      <c r="I78" s="137"/>
-      <c r="J78" s="138"/>
+      <c r="I78" s="151"/>
+      <c r="J78" s="152"/>
       <c r="K78" s="19" t="s">
         <v>129</v>
       </c>
@@ -30550,18 +30550,18 @@
     </row>
     <row r="79" spans="2:33">
       <c r="B79" s="22"/>
-      <c r="C79" s="144" t="s">
+      <c r="C79" s="139" t="s">
         <v>130</v>
       </c>
-      <c r="D79" s="151"/>
-      <c r="E79" s="151"/>
-      <c r="F79" s="151"/>
-      <c r="G79" s="140"/>
-      <c r="H79" s="141" t="s">
+      <c r="D79" s="147"/>
+      <c r="E79" s="147"/>
+      <c r="F79" s="147"/>
+      <c r="G79" s="141"/>
+      <c r="H79" s="146" t="s">
         <v>131</v>
       </c>
-      <c r="I79" s="151"/>
-      <c r="J79" s="140"/>
+      <c r="I79" s="147"/>
+      <c r="J79" s="141"/>
       <c r="K79" s="19" t="s">
         <v>132</v>
       </c>
@@ -30581,18 +30581,18 @@
     </row>
     <row r="80" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
       <c r="B80" s="75"/>
-      <c r="C80" s="152" t="s">
+      <c r="C80" s="142" t="s">
         <v>133</v>
       </c>
-      <c r="D80" s="149"/>
-      <c r="E80" s="149"/>
-      <c r="F80" s="149"/>
-      <c r="G80" s="150"/>
-      <c r="H80" s="148" t="s">
+      <c r="D80" s="137"/>
+      <c r="E80" s="137"/>
+      <c r="F80" s="137"/>
+      <c r="G80" s="138"/>
+      <c r="H80" s="136" t="s">
         <v>73</v>
       </c>
-      <c r="I80" s="149"/>
-      <c r="J80" s="150"/>
+      <c r="I80" s="137"/>
+      <c r="J80" s="138"/>
       <c r="K80" s="81" t="s">
         <v>134</v>
       </c>
@@ -30703,6 +30703,87 @@
     </row>
   </sheetData>
   <mergeCells count="97">
+    <mergeCell ref="C24:G25"/>
+    <mergeCell ref="H30:J30"/>
+    <mergeCell ref="H24:J25"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="H51:J51"/>
+    <mergeCell ref="H69:J69"/>
+    <mergeCell ref="C29:G29"/>
+    <mergeCell ref="C65:G65"/>
+    <mergeCell ref="H66:J66"/>
+    <mergeCell ref="C52:G52"/>
+    <mergeCell ref="C68:G68"/>
+    <mergeCell ref="C69:G69"/>
+    <mergeCell ref="H64:J64"/>
+    <mergeCell ref="H60:J60"/>
+    <mergeCell ref="H57:J57"/>
+    <mergeCell ref="H45:J45"/>
+    <mergeCell ref="C30:G30"/>
+    <mergeCell ref="C62:G62"/>
+    <mergeCell ref="H32:J32"/>
+    <mergeCell ref="B34:G34"/>
+    <mergeCell ref="B71:G71"/>
+    <mergeCell ref="B2:V2"/>
+    <mergeCell ref="B11:V11"/>
+    <mergeCell ref="C58:G58"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B5:V5"/>
+    <mergeCell ref="H47:J49"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="H34:J34"/>
+    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="H28:J28"/>
+    <mergeCell ref="H29:J29"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="H31:J31"/>
+    <mergeCell ref="H58:J58"/>
+    <mergeCell ref="H40:J40"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="C47:G49"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="C60:G60"/>
+    <mergeCell ref="C57:G57"/>
+    <mergeCell ref="C42:G42"/>
+    <mergeCell ref="C39:G39"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="C80:G80"/>
+    <mergeCell ref="H77:J77"/>
+    <mergeCell ref="B51:G51"/>
+    <mergeCell ref="C59:G59"/>
+    <mergeCell ref="H42:J42"/>
+    <mergeCell ref="C46:G46"/>
+    <mergeCell ref="C61:G61"/>
+    <mergeCell ref="H67:J67"/>
+    <mergeCell ref="H59:J59"/>
+    <mergeCell ref="B77:G77"/>
+    <mergeCell ref="H46:J46"/>
+    <mergeCell ref="H52:J52"/>
+    <mergeCell ref="C79:G79"/>
+    <mergeCell ref="C73:G73"/>
+    <mergeCell ref="H72:J72"/>
+    <mergeCell ref="C54:G54"/>
+    <mergeCell ref="H35:J35"/>
+    <mergeCell ref="C78:G78"/>
+    <mergeCell ref="H79:J79"/>
+    <mergeCell ref="H61:J61"/>
+    <mergeCell ref="C74:G74"/>
+    <mergeCell ref="C67:G67"/>
+    <mergeCell ref="C72:G72"/>
+    <mergeCell ref="H78:J78"/>
+    <mergeCell ref="H73:J73"/>
+    <mergeCell ref="H65:J65"/>
+    <mergeCell ref="H71:J71"/>
+    <mergeCell ref="H75:J75"/>
+    <mergeCell ref="C75:G75"/>
+    <mergeCell ref="B64:G64"/>
+    <mergeCell ref="H53:J53"/>
+    <mergeCell ref="H36:J36"/>
     <mergeCell ref="H80:J80"/>
     <mergeCell ref="C41:G41"/>
     <mergeCell ref="H62:J62"/>
@@ -30719,87 +30800,6 @@
     <mergeCell ref="H74:J74"/>
     <mergeCell ref="H56:J56"/>
     <mergeCell ref="H68:J68"/>
-    <mergeCell ref="H35:J35"/>
-    <mergeCell ref="C78:G78"/>
-    <mergeCell ref="H79:J79"/>
-    <mergeCell ref="H61:J61"/>
-    <mergeCell ref="C74:G74"/>
-    <mergeCell ref="C67:G67"/>
-    <mergeCell ref="C72:G72"/>
-    <mergeCell ref="H78:J78"/>
-    <mergeCell ref="H73:J73"/>
-    <mergeCell ref="H65:J65"/>
-    <mergeCell ref="H71:J71"/>
-    <mergeCell ref="H75:J75"/>
-    <mergeCell ref="C75:G75"/>
-    <mergeCell ref="B64:G64"/>
-    <mergeCell ref="H53:J53"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="C80:G80"/>
-    <mergeCell ref="H77:J77"/>
-    <mergeCell ref="B51:G51"/>
-    <mergeCell ref="C59:G59"/>
-    <mergeCell ref="H42:J42"/>
-    <mergeCell ref="C46:G46"/>
-    <mergeCell ref="C61:G61"/>
-    <mergeCell ref="H67:J67"/>
-    <mergeCell ref="H59:J59"/>
-    <mergeCell ref="B77:G77"/>
-    <mergeCell ref="H46:J46"/>
-    <mergeCell ref="H52:J52"/>
-    <mergeCell ref="C79:G79"/>
-    <mergeCell ref="C73:G73"/>
-    <mergeCell ref="H72:J72"/>
-    <mergeCell ref="C54:G54"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="C40:G40"/>
-    <mergeCell ref="C47:G49"/>
-    <mergeCell ref="B45:G45"/>
-    <mergeCell ref="C60:G60"/>
-    <mergeCell ref="C57:G57"/>
-    <mergeCell ref="C42:G42"/>
-    <mergeCell ref="C39:G39"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="B71:G71"/>
-    <mergeCell ref="B2:V2"/>
-    <mergeCell ref="B11:V11"/>
-    <mergeCell ref="C58:G58"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="B5:V5"/>
-    <mergeCell ref="H47:J49"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="H34:J34"/>
-    <mergeCell ref="H39:J39"/>
-    <mergeCell ref="H28:J28"/>
-    <mergeCell ref="H29:J29"/>
-    <mergeCell ref="H38:J38"/>
-    <mergeCell ref="H31:J31"/>
-    <mergeCell ref="H58:J58"/>
-    <mergeCell ref="H40:J40"/>
-    <mergeCell ref="H51:J51"/>
-    <mergeCell ref="H69:J69"/>
-    <mergeCell ref="C29:G29"/>
-    <mergeCell ref="C65:G65"/>
-    <mergeCell ref="H66:J66"/>
-    <mergeCell ref="C52:G52"/>
-    <mergeCell ref="C68:G68"/>
-    <mergeCell ref="C69:G69"/>
-    <mergeCell ref="H64:J64"/>
-    <mergeCell ref="H60:J60"/>
-    <mergeCell ref="H57:J57"/>
-    <mergeCell ref="H45:J45"/>
-    <mergeCell ref="C30:G30"/>
-    <mergeCell ref="C62:G62"/>
-    <mergeCell ref="H32:J32"/>
-    <mergeCell ref="B34:G34"/>
-    <mergeCell ref="C24:G25"/>
-    <mergeCell ref="H30:J30"/>
-    <mergeCell ref="H24:J25"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="H26:J26"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -69671,10 +69671,10 @@
       <c r="B2" s="162" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="137"/>
-      <c r="D2" s="137"/>
-      <c r="E2" s="137"/>
-      <c r="F2" s="137"/>
+      <c r="C2" s="151"/>
+      <c r="D2" s="151"/>
+      <c r="E2" s="151"/>
+      <c r="F2" s="151"/>
       <c r="G2" s="163"/>
       <c r="H2" s="11"/>
       <c r="I2" s="11"/>
@@ -69684,10 +69684,10 @@
       <c r="M2" s="165" t="s">
         <v>1</v>
       </c>
-      <c r="N2" s="146"/>
-      <c r="O2" s="146"/>
-      <c r="P2" s="146"/>
-      <c r="Q2" s="147"/>
+      <c r="N2" s="144"/>
+      <c r="O2" s="144"/>
+      <c r="P2" s="144"/>
+      <c r="Q2" s="149"/>
       <c r="R2" s="11"/>
       <c r="S2" s="11"/>
       <c r="T2" s="11"/>
@@ -69695,10 +69695,10 @@
       <c r="V2" s="165" t="s">
         <v>2</v>
       </c>
-      <c r="W2" s="146"/>
-      <c r="X2" s="146"/>
-      <c r="Y2" s="146"/>
-      <c r="Z2" s="147"/>
+      <c r="W2" s="144"/>
+      <c r="X2" s="144"/>
+      <c r="Y2" s="144"/>
+      <c r="Z2" s="149"/>
       <c r="AA2" s="11"/>
       <c r="AB2" s="11"/>
       <c r="AC2" s="10"/>
@@ -69817,10 +69817,10 @@
       <c r="V5" s="165" t="s">
         <v>10</v>
       </c>
-      <c r="W5" s="146"/>
-      <c r="X5" s="146"/>
-      <c r="Y5" s="146"/>
-      <c r="Z5" s="147"/>
+      <c r="W5" s="144"/>
+      <c r="X5" s="144"/>
+      <c r="Y5" s="144"/>
+      <c r="Z5" s="149"/>
       <c r="AA5" s="11"/>
       <c r="AB5" s="11"/>
       <c r="AC5" s="10"/>
@@ -69866,10 +69866,10 @@
       <c r="B7" s="165" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="146"/>
-      <c r="D7" s="146"/>
-      <c r="E7" s="146"/>
-      <c r="F7" s="147"/>
+      <c r="C7" s="144"/>
+      <c r="D7" s="144"/>
+      <c r="E7" s="144"/>
+      <c r="F7" s="149"/>
       <c r="G7" s="33"/>
       <c r="H7" s="33"/>
       <c r="I7" s="33"/>
@@ -69878,10 +69878,10 @@
       <c r="L7" s="165" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="146"/>
-      <c r="N7" s="146"/>
-      <c r="O7" s="146"/>
-      <c r="P7" s="147"/>
+      <c r="M7" s="144"/>
+      <c r="N7" s="144"/>
+      <c r="O7" s="144"/>
+      <c r="P7" s="149"/>
       <c r="Q7" s="11"/>
       <c r="R7" s="11"/>
       <c r="S7" s="11"/>
@@ -70090,10 +70090,10 @@
       <c r="AB14" s="164" t="s">
         <v>18</v>
       </c>
-      <c r="AC14" s="146"/>
-      <c r="AD14" s="146"/>
-      <c r="AE14" s="146"/>
-      <c r="AF14" s="147"/>
+      <c r="AC14" s="144"/>
+      <c r="AD14" s="144"/>
+      <c r="AE14" s="144"/>
+      <c r="AF14" s="149"/>
       <c r="AG14" s="100"/>
       <c r="AH14" s="45"/>
       <c r="AI14" s="12"/>
@@ -70167,10 +70167,10 @@
       <c r="AB17" s="164" t="s">
         <v>20</v>
       </c>
-      <c r="AC17" s="146"/>
-      <c r="AD17" s="146"/>
-      <c r="AE17" s="146"/>
-      <c r="AF17" s="147"/>
+      <c r="AC17" s="144"/>
+      <c r="AD17" s="144"/>
+      <c r="AE17" s="144"/>
+      <c r="AF17" s="149"/>
       <c r="AG17" s="102"/>
       <c r="AH17" s="38"/>
       <c r="AI17" s="10"/>
@@ -70288,10 +70288,10 @@
       <c r="AB21" s="164" t="s">
         <v>22</v>
       </c>
-      <c r="AC21" s="146"/>
-      <c r="AD21" s="146"/>
-      <c r="AE21" s="146"/>
-      <c r="AF21" s="147"/>
+      <c r="AC21" s="144"/>
+      <c r="AD21" s="144"/>
+      <c r="AE21" s="144"/>
+      <c r="AF21" s="149"/>
       <c r="AG21" s="116"/>
       <c r="AH21" s="117"/>
     </row>
@@ -71104,7 +71104,7 @@
         <v>781</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C7" t="s">
         <v>782</v>

</xml_diff>

<commit_message>
[ADD|MOD] 261016 Stage 점수 번역 · 옛 그림 Resources 밖으로(WebGL 용량) · itch 몽환 수채화 페이지 자료
- StageHUD: Cur_Score 옆 "점수" 라벨을 Loc.T로 번역 (String 901322 EN/JA/RU/UK)
- 옛 그림 세트(Doodle·Generated·Soft)를 Assets/ArtArchive·ArtSource로 옮겨 WebGL 160MB로
- itch 페이지 자료(Marketing/itch_dream, Tools/itch) · GIF·스크린샷 합성 스크립트
- 인계: itch 페이지 1·2, Stage 번역·웹빌드

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assets/DB/MMM_DB_Ver.05.xlsx
+++ b/Assets/DB/MMM_DB_Ver.05.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\MoreMustMush\Assets\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{529870C9-7E70-4ACB-982F-C2B8467411F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0722B07-0035-4E49-A6B2-50ABC1F7F5C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10554" uniqueCount="8347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10566" uniqueCount="8352">
   <si>
     <t>Upgrade_Table</t>
   </si>
@@ -28917,6 +28917,24 @@
   </si>
   <si>
     <t>Вирушай по врожай і пройди перший етап!</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>점수</t>
+  </si>
+  <si>
+    <t>세트 밖이지만 배치한 UI가 쓰는 한·영 전용 폰트 (ONEMobilePOP 등). 한국어·영어에서는 그대로 두고, 그 밖의 언어에서는 그 언어 본문 폰트로 바꾼다 (TextLangFont)</t>
+  </si>
+  <si>
+    <t>Score</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>スコア</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Очки</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -33042,7 +33060,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H1548"/>
+  <dimension ref="A1:H1550"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="2" max="2" width="12.75" style="2" bestFit="1" customWidth="1"/>
@@ -73010,6 +73028,58 @@
       </c>
       <c r="H1548" s="130" t="s">
         <v>8313</v>
+      </c>
+    </row>
+    <row r="1549" spans="1:8">
+      <c r="A1549">
+        <v>901322</v>
+      </c>
+      <c r="B1549" s="2">
+        <v>91322</v>
+      </c>
+      <c r="C1549" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1549" s="130" t="s">
+        <v>8347</v>
+      </c>
+      <c r="E1549" s="130" t="s">
+        <v>8349</v>
+      </c>
+      <c r="F1549" s="130" t="s">
+        <v>8350</v>
+      </c>
+      <c r="G1549" s="130" t="s">
+        <v>8351</v>
+      </c>
+      <c r="H1549" s="130" t="s">
+        <v>8351</v>
+      </c>
+    </row>
+    <row r="1550" spans="1:8">
+      <c r="A1550">
+        <v>901323</v>
+      </c>
+      <c r="B1550" s="2">
+        <v>91323</v>
+      </c>
+      <c r="C1550" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1550" s="130" t="s">
+        <v>8348</v>
+      </c>
+      <c r="E1550" s="130" t="s">
+        <v>816</v>
+      </c>
+      <c r="F1550" s="130" t="s">
+        <v>816</v>
+      </c>
+      <c r="G1550" s="130" t="s">
+        <v>816</v>
+      </c>
+      <c r="H1550" s="130" t="s">
+        <v>816</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[MOD] 261019 번역 누락 보완: Combo·NEW·Lv·MAX·LVL
- Stage 씬 ComboText에 LocText(key 콤보)
- 정산 NEW 태그, 트리 노드 Lv/MAX, 툴팁 LVL을 Loc.T/F로
- 번역표 13줄 추가 (Str_ID 901343~901355, EN·JA·RU·UK)
- 인계 2026-10-19_번역누락_보완.md (머지 충돌 해결·조사 결과·pt-BR 미반영)
</commit_message>
<xml_diff>
--- a/Assets/DB/MMM_DB_Ver.05.xlsx
+++ b/Assets/DB/MMM_DB_Ver.05.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\MoreMustMush\Assets\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A7D5E0-2018-44FE-87B5-AC21C6C2DA8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7004AC3-463F-4F71-A084-F38FC1B090FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4500" yWindow="570" windowWidth="18900" windowHeight="13410" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10699" uniqueCount="8463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10777" uniqueCount="8502">
   <si>
     <t>Upgrade_Table</t>
   </si>
@@ -29643,6 +29643,123 @@
   <si>
     <t>Висота смуги {0}, шкода: атака ×{1}</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>콤보</t>
+  </si>
+  <si>
+    <t>Combo</t>
+  </si>
+  <si>
+    <t>コンボ</t>
+  </si>
+  <si>
+    <t>Комбо</t>
+  </si>
+  <si>
+    <t>NEW</t>
+  </si>
+  <si>
+    <t>НОВОЕ</t>
+  </si>
+  <si>
+    <t>НОВЕ</t>
+  </si>
+  <si>
+    <t>Lv {0}</t>
+  </si>
+  <si>
+    <t>Ур. {0}</t>
+  </si>
+  <si>
+    <t>Рів. {0}</t>
+  </si>
+  <si>
+    <t>Lv {0}/{1}</t>
+  </si>
+  <si>
+    <t>Ур. {0}/{1}</t>
+  </si>
+  <si>
+    <t>Рів. {0}/{1}</t>
+  </si>
+  <si>
+    <t>MAX</t>
+  </si>
+  <si>
+    <t>МАКС</t>
+  </si>
+  <si>
+    <t>MAX {0}</t>
+  </si>
+  <si>
+    <t>МАКС {0}</t>
+  </si>
+  <si>
+    <t>MAX {0}/{1}</t>
+  </si>
+  <si>
+    <t>МАКС {0}/{1}</t>
+  </si>
+  <si>
+    <t>LVL {0} / {1}</t>
+  </si>
+  <si>
+    <t>Lv {0} / {1}</t>
+  </si>
+  <si>
+    <t>УР. {0} / {1}</t>
+  </si>
+  <si>
+    <t>РІВ. {0} / {1}</t>
+  </si>
+  <si>
+    <t>LVL {0} / ∞</t>
+  </si>
+  <si>
+    <t>Lv {0} / ∞</t>
+  </si>
+  <si>
+    <t>УР. {0} / ∞</t>
+  </si>
+  <si>
+    <t>РІВ. {0} / ∞</t>
+  </si>
+  <si>
+    <t>{0} Lv.{1}</t>
+  </si>
+  <si>
+    <t>{0} ур.{1}</t>
+  </si>
+  <si>
+    <t>{0} рів.{1}</t>
+  </si>
+  <si>
+    <t>{0} {1} Lv.{2}</t>
+  </si>
+  <si>
+    <t>{0} {1} ур.{2}</t>
+  </si>
+  <si>
+    <t>{0} {1} рів.{2}</t>
+  </si>
+  <si>
+    <t>★{0} · Lv.{1}</t>
+  </si>
+  <si>
+    <t>★{0} · ур.{1}</t>
+  </si>
+  <si>
+    <t>★{0} · рів.{1}</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;{0}&lt;/b&gt; &lt;color=#e8a900&gt;{1}&lt;/color&gt;  Lv.{2}/{3}</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;{0}&lt;/b&gt; &lt;color=#e8a900&gt;{1}&lt;/color&gt;  ур.{2}/{3}</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;{0}&lt;/b&gt; &lt;color=#e8a900&gt;{1}&lt;/color&gt;  рів.{2}/{3}</t>
   </si>
 </sst>
 </file>
@@ -30527,46 +30644,46 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -30575,12 +30692,12 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -31048,29 +31165,29 @@
   <sheetData>
     <row r="1" spans="2:44" ht="12" customHeight="1"/>
     <row r="2" spans="2:44">
-      <c r="B2" s="154" t="s">
+      <c r="B2" s="156" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="155"/>
-      <c r="D2" s="155"/>
-      <c r="E2" s="155"/>
-      <c r="F2" s="155"/>
-      <c r="G2" s="155"/>
-      <c r="H2" s="155"/>
-      <c r="I2" s="155"/>
-      <c r="J2" s="155"/>
-      <c r="K2" s="155"/>
-      <c r="L2" s="155"/>
-      <c r="M2" s="155"/>
-      <c r="N2" s="155"/>
-      <c r="O2" s="155"/>
-      <c r="P2" s="155"/>
-      <c r="Q2" s="155"/>
-      <c r="R2" s="155"/>
-      <c r="S2" s="155"/>
-      <c r="T2" s="155"/>
-      <c r="U2" s="155"/>
-      <c r="V2" s="156"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="157"/>
+      <c r="E2" s="157"/>
+      <c r="F2" s="157"/>
+      <c r="G2" s="157"/>
+      <c r="H2" s="157"/>
+      <c r="I2" s="157"/>
+      <c r="J2" s="157"/>
+      <c r="K2" s="157"/>
+      <c r="L2" s="157"/>
+      <c r="M2" s="157"/>
+      <c r="N2" s="157"/>
+      <c r="O2" s="157"/>
+      <c r="P2" s="157"/>
+      <c r="Q2" s="157"/>
+      <c r="R2" s="157"/>
+      <c r="S2" s="157"/>
+      <c r="T2" s="157"/>
+      <c r="U2" s="157"/>
+      <c r="V2" s="158"/>
     </row>
     <row r="3" spans="2:44">
       <c r="B3" s="17"/>
@@ -31127,29 +31244,29 @@
       <c r="V4" s="14"/>
     </row>
     <row r="5" spans="2:44">
-      <c r="B5" s="154" t="s">
+      <c r="B5" s="156" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="155"/>
-      <c r="D5" s="155"/>
-      <c r="E5" s="155"/>
-      <c r="F5" s="155"/>
-      <c r="G5" s="155"/>
-      <c r="H5" s="155"/>
-      <c r="I5" s="155"/>
-      <c r="J5" s="155"/>
-      <c r="K5" s="155"/>
-      <c r="L5" s="155"/>
-      <c r="M5" s="155"/>
-      <c r="N5" s="155"/>
-      <c r="O5" s="155"/>
-      <c r="P5" s="155"/>
-      <c r="Q5" s="155"/>
-      <c r="R5" s="155"/>
-      <c r="S5" s="155"/>
-      <c r="T5" s="155"/>
-      <c r="U5" s="155"/>
-      <c r="V5" s="156"/>
+      <c r="C5" s="157"/>
+      <c r="D5" s="157"/>
+      <c r="E5" s="157"/>
+      <c r="F5" s="157"/>
+      <c r="G5" s="157"/>
+      <c r="H5" s="157"/>
+      <c r="I5" s="157"/>
+      <c r="J5" s="157"/>
+      <c r="K5" s="157"/>
+      <c r="L5" s="157"/>
+      <c r="M5" s="157"/>
+      <c r="N5" s="157"/>
+      <c r="O5" s="157"/>
+      <c r="P5" s="157"/>
+      <c r="Q5" s="157"/>
+      <c r="R5" s="157"/>
+      <c r="S5" s="157"/>
+      <c r="T5" s="157"/>
+      <c r="U5" s="157"/>
+      <c r="V5" s="158"/>
     </row>
     <row r="6" spans="2:44">
       <c r="B6" s="6"/>
@@ -31279,29 +31396,29 @@
     </row>
     <row r="10" spans="2:44" ht="8.1" customHeight="1"/>
     <row r="11" spans="2:44">
-      <c r="B11" s="154" t="s">
+      <c r="B11" s="156" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="155"/>
-      <c r="D11" s="155"/>
-      <c r="E11" s="155"/>
-      <c r="F11" s="155"/>
-      <c r="G11" s="155"/>
-      <c r="H11" s="155"/>
-      <c r="I11" s="155"/>
-      <c r="J11" s="155"/>
-      <c r="K11" s="155"/>
-      <c r="L11" s="155"/>
-      <c r="M11" s="155"/>
-      <c r="N11" s="155"/>
-      <c r="O11" s="155"/>
-      <c r="P11" s="155"/>
-      <c r="Q11" s="155"/>
-      <c r="R11" s="155"/>
-      <c r="S11" s="155"/>
-      <c r="T11" s="155"/>
-      <c r="U11" s="155"/>
-      <c r="V11" s="156"/>
+      <c r="C11" s="157"/>
+      <c r="D11" s="157"/>
+      <c r="E11" s="157"/>
+      <c r="F11" s="157"/>
+      <c r="G11" s="157"/>
+      <c r="H11" s="157"/>
+      <c r="I11" s="157"/>
+      <c r="J11" s="157"/>
+      <c r="K11" s="157"/>
+      <c r="L11" s="157"/>
+      <c r="M11" s="157"/>
+      <c r="N11" s="157"/>
+      <c r="O11" s="157"/>
+      <c r="P11" s="157"/>
+      <c r="Q11" s="157"/>
+      <c r="R11" s="157"/>
+      <c r="S11" s="157"/>
+      <c r="T11" s="157"/>
+      <c r="U11" s="157"/>
+      <c r="V11" s="158"/>
     </row>
     <row r="12" spans="2:44">
       <c r="B12" s="6"/>
@@ -31588,19 +31705,19 @@
       <c r="AF22" s="27"/>
     </row>
     <row r="23" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B23" s="157" t="s">
+      <c r="B23" s="159" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="144"/>
-      <c r="D23" s="144"/>
-      <c r="E23" s="144"/>
-      <c r="F23" s="144"/>
-      <c r="G23" s="144"/>
-      <c r="H23" s="143" t="s">
+      <c r="C23" s="146"/>
+      <c r="D23" s="146"/>
+      <c r="E23" s="146"/>
+      <c r="F23" s="146"/>
+      <c r="G23" s="146"/>
+      <c r="H23" s="161" t="s">
         <v>67</v>
       </c>
-      <c r="I23" s="144"/>
-      <c r="J23" s="144"/>
+      <c r="I23" s="146"/>
+      <c r="J23" s="146"/>
       <c r="K23" s="28" t="s">
         <v>68</v>
       </c>
@@ -31628,18 +31745,18 @@
     </row>
     <row r="24" spans="2:32" s="10" customFormat="1">
       <c r="B24" s="86"/>
-      <c r="C24" s="153" t="s">
+      <c r="C24" s="136" t="s">
         <v>3</v>
       </c>
-      <c r="D24" s="151"/>
-      <c r="E24" s="151"/>
-      <c r="F24" s="151"/>
-      <c r="G24" s="152"/>
-      <c r="H24" s="150" t="s">
+      <c r="D24" s="137"/>
+      <c r="E24" s="137"/>
+      <c r="F24" s="137"/>
+      <c r="G24" s="138"/>
+      <c r="H24" s="142" t="s">
         <v>69</v>
       </c>
-      <c r="I24" s="151"/>
-      <c r="J24" s="152"/>
+      <c r="I24" s="137"/>
+      <c r="J24" s="138"/>
       <c r="K24" s="34" t="s">
         <v>70</v>
       </c>
@@ -31667,14 +31784,14 @@
     </row>
     <row r="25" spans="2:32" s="10" customFormat="1">
       <c r="B25" s="22"/>
-      <c r="C25" s="140"/>
-      <c r="D25" s="140"/>
-      <c r="E25" s="140"/>
-      <c r="F25" s="140"/>
-      <c r="G25" s="141"/>
-      <c r="H25" s="158"/>
-      <c r="I25" s="140"/>
-      <c r="J25" s="141"/>
+      <c r="C25" s="139"/>
+      <c r="D25" s="139"/>
+      <c r="E25" s="139"/>
+      <c r="F25" s="139"/>
+      <c r="G25" s="140"/>
+      <c r="H25" s="143"/>
+      <c r="I25" s="139"/>
+      <c r="J25" s="140"/>
       <c r="K25" s="19" t="s">
         <v>49</v>
       </c>
@@ -31696,18 +31813,18 @@
     </row>
     <row r="26" spans="2:32" s="10" customFormat="1">
       <c r="B26" s="22"/>
-      <c r="C26" s="139" t="s">
+      <c r="C26" s="144" t="s">
         <v>72</v>
       </c>
-      <c r="D26" s="140"/>
-      <c r="E26" s="140"/>
-      <c r="F26" s="140"/>
-      <c r="G26" s="141"/>
-      <c r="H26" s="146" t="s">
+      <c r="D26" s="139"/>
+      <c r="E26" s="139"/>
+      <c r="F26" s="139"/>
+      <c r="G26" s="140"/>
+      <c r="H26" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I26" s="140"/>
-      <c r="J26" s="141"/>
+      <c r="I26" s="139"/>
+      <c r="J26" s="140"/>
       <c r="K26" s="19" t="s">
         <v>74</v>
       </c>
@@ -31727,18 +31844,18 @@
     </row>
     <row r="27" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B27" s="22"/>
-      <c r="C27" s="139" t="s">
+      <c r="C27" s="144" t="s">
         <v>9</v>
       </c>
-      <c r="D27" s="140"/>
-      <c r="E27" s="140"/>
-      <c r="F27" s="140"/>
-      <c r="G27" s="141"/>
-      <c r="H27" s="146" t="s">
+      <c r="D27" s="139"/>
+      <c r="E27" s="139"/>
+      <c r="F27" s="139"/>
+      <c r="G27" s="140"/>
+      <c r="H27" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I27" s="140"/>
-      <c r="J27" s="141"/>
+      <c r="I27" s="139"/>
+      <c r="J27" s="140"/>
       <c r="K27" s="19" t="s">
         <v>75</v>
       </c>
@@ -31758,18 +31875,18 @@
     </row>
     <row r="28" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B28" s="22"/>
-      <c r="C28" s="139" t="s">
+      <c r="C28" s="144" t="s">
         <v>76</v>
       </c>
-      <c r="D28" s="140"/>
-      <c r="E28" s="140"/>
-      <c r="F28" s="140"/>
-      <c r="G28" s="141"/>
-      <c r="H28" s="146" t="s">
+      <c r="D28" s="139"/>
+      <c r="E28" s="139"/>
+      <c r="F28" s="139"/>
+      <c r="G28" s="140"/>
+      <c r="H28" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I28" s="140"/>
-      <c r="J28" s="141"/>
+      <c r="I28" s="139"/>
+      <c r="J28" s="140"/>
       <c r="K28" s="19" t="s">
         <v>77</v>
       </c>
@@ -31789,18 +31906,18 @@
     </row>
     <row r="29" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B29" s="22"/>
-      <c r="C29" s="139" t="s">
+      <c r="C29" s="144" t="s">
         <v>67</v>
       </c>
-      <c r="D29" s="140"/>
-      <c r="E29" s="140"/>
-      <c r="F29" s="140"/>
-      <c r="G29" s="141"/>
-      <c r="H29" s="146" t="s">
+      <c r="D29" s="139"/>
+      <c r="E29" s="139"/>
+      <c r="F29" s="139"/>
+      <c r="G29" s="140"/>
+      <c r="H29" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I29" s="140"/>
-      <c r="J29" s="141"/>
+      <c r="I29" s="139"/>
+      <c r="J29" s="140"/>
       <c r="K29" s="19" t="s">
         <v>78</v>
       </c>
@@ -31820,18 +31937,18 @@
     </row>
     <row r="30" spans="2:32" s="10" customFormat="1">
       <c r="B30" s="22"/>
-      <c r="C30" s="139" t="s">
+      <c r="C30" s="144" t="s">
         <v>79</v>
       </c>
-      <c r="D30" s="140"/>
-      <c r="E30" s="140"/>
-      <c r="F30" s="140"/>
-      <c r="G30" s="141"/>
-      <c r="H30" s="146" t="s">
+      <c r="D30" s="139"/>
+      <c r="E30" s="139"/>
+      <c r="F30" s="139"/>
+      <c r="G30" s="140"/>
+      <c r="H30" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I30" s="140"/>
-      <c r="J30" s="141"/>
+      <c r="I30" s="139"/>
+      <c r="J30" s="140"/>
       <c r="K30" s="120" t="s">
         <v>421</v>
       </c>
@@ -31851,18 +31968,18 @@
     </row>
     <row r="31" spans="2:32" s="10" customFormat="1">
       <c r="B31" s="22"/>
-      <c r="C31" s="139" t="s">
+      <c r="C31" s="144" t="s">
         <v>7</v>
       </c>
-      <c r="D31" s="140"/>
-      <c r="E31" s="140"/>
-      <c r="F31" s="140"/>
-      <c r="G31" s="141"/>
-      <c r="H31" s="146" t="s">
+      <c r="D31" s="139"/>
+      <c r="E31" s="139"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="140"/>
+      <c r="H31" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I31" s="140"/>
-      <c r="J31" s="141"/>
+      <c r="I31" s="139"/>
+      <c r="J31" s="140"/>
       <c r="K31" s="19" t="s">
         <v>80</v>
       </c>
@@ -31882,18 +31999,18 @@
     </row>
     <row r="32" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B32" s="75"/>
-      <c r="C32" s="145" t="s">
+      <c r="C32" s="160" t="s">
         <v>422</v>
       </c>
-      <c r="D32" s="137"/>
-      <c r="E32" s="137"/>
-      <c r="F32" s="137"/>
-      <c r="G32" s="138"/>
-      <c r="H32" s="136" t="s">
+      <c r="D32" s="149"/>
+      <c r="E32" s="149"/>
+      <c r="F32" s="149"/>
+      <c r="G32" s="150"/>
+      <c r="H32" s="148" t="s">
         <v>81</v>
       </c>
-      <c r="I32" s="137"/>
-      <c r="J32" s="138"/>
+      <c r="I32" s="149"/>
+      <c r="J32" s="150"/>
       <c r="K32" s="81" t="s">
         <v>82</v>
       </c>
@@ -31955,19 +32072,19 @@
       <c r="AF33" s="27"/>
     </row>
     <row r="34" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B34" s="148" t="s">
+      <c r="B34" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C34" s="144"/>
-      <c r="D34" s="144"/>
-      <c r="E34" s="144"/>
-      <c r="F34" s="144"/>
-      <c r="G34" s="149"/>
-      <c r="H34" s="148" t="s">
+      <c r="C34" s="146"/>
+      <c r="D34" s="146"/>
+      <c r="E34" s="146"/>
+      <c r="F34" s="146"/>
+      <c r="G34" s="147"/>
+      <c r="H34" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I34" s="144"/>
-      <c r="J34" s="149"/>
+      <c r="I34" s="146"/>
+      <c r="J34" s="147"/>
       <c r="K34" s="28" t="s">
         <v>68</v>
       </c>
@@ -31995,18 +32112,18 @@
     </row>
     <row r="35" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B35" s="86"/>
-      <c r="C35" s="153" t="s">
+      <c r="C35" s="136" t="s">
         <v>7</v>
       </c>
-      <c r="D35" s="151"/>
-      <c r="E35" s="151"/>
-      <c r="F35" s="151"/>
-      <c r="G35" s="152"/>
-      <c r="H35" s="150" t="s">
+      <c r="D35" s="137"/>
+      <c r="E35" s="137"/>
+      <c r="F35" s="137"/>
+      <c r="G35" s="138"/>
+      <c r="H35" s="142" t="s">
         <v>69</v>
       </c>
-      <c r="I35" s="151"/>
-      <c r="J35" s="152"/>
+      <c r="I35" s="137"/>
+      <c r="J35" s="138"/>
       <c r="K35" s="34" t="s">
         <v>84</v>
       </c>
@@ -32034,18 +32151,18 @@
     </row>
     <row r="36" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B36" s="75"/>
-      <c r="C36" s="145" t="s">
+      <c r="C36" s="160" t="s">
         <v>423</v>
       </c>
-      <c r="D36" s="137"/>
-      <c r="E36" s="137"/>
-      <c r="F36" s="137"/>
-      <c r="G36" s="138"/>
-      <c r="H36" s="136" t="s">
+      <c r="D36" s="149"/>
+      <c r="E36" s="149"/>
+      <c r="F36" s="149"/>
+      <c r="G36" s="150"/>
+      <c r="H36" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="I36" s="137"/>
-      <c r="J36" s="138"/>
+      <c r="I36" s="149"/>
+      <c r="J36" s="150"/>
       <c r="K36" s="81" t="s">
         <v>85</v>
       </c>
@@ -32107,19 +32224,19 @@
       <c r="AF37" s="92"/>
     </row>
     <row r="38" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B38" s="148" t="s">
+      <c r="B38" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C38" s="144"/>
-      <c r="D38" s="144"/>
-      <c r="E38" s="144"/>
-      <c r="F38" s="144"/>
-      <c r="G38" s="149"/>
-      <c r="H38" s="148" t="s">
+      <c r="C38" s="146"/>
+      <c r="D38" s="146"/>
+      <c r="E38" s="146"/>
+      <c r="F38" s="146"/>
+      <c r="G38" s="147"/>
+      <c r="H38" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I38" s="144"/>
-      <c r="J38" s="149"/>
+      <c r="I38" s="146"/>
+      <c r="J38" s="147"/>
       <c r="K38" s="28" t="s">
         <v>68</v>
       </c>
@@ -32147,18 +32264,18 @@
     </row>
     <row r="39" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B39" s="21"/>
-      <c r="C39" s="139" t="s">
+      <c r="C39" s="144" t="s">
         <v>14</v>
       </c>
-      <c r="D39" s="140"/>
-      <c r="E39" s="140"/>
-      <c r="F39" s="140"/>
-      <c r="G39" s="141"/>
-      <c r="H39" s="146" t="s">
+      <c r="D39" s="139"/>
+      <c r="E39" s="139"/>
+      <c r="F39" s="139"/>
+      <c r="G39" s="140"/>
+      <c r="H39" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I39" s="140"/>
-      <c r="J39" s="141"/>
+      <c r="I39" s="139"/>
+      <c r="J39" s="140"/>
       <c r="K39" s="19" t="s">
         <v>86</v>
       </c>
@@ -32178,18 +32295,18 @@
     </row>
     <row r="40" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B40" s="22"/>
-      <c r="C40" s="139" t="s">
+      <c r="C40" s="144" t="s">
         <v>87</v>
       </c>
-      <c r="D40" s="140"/>
-      <c r="E40" s="140"/>
-      <c r="F40" s="140"/>
-      <c r="G40" s="141"/>
-      <c r="H40" s="146" t="s">
+      <c r="D40" s="139"/>
+      <c r="E40" s="139"/>
+      <c r="F40" s="139"/>
+      <c r="G40" s="140"/>
+      <c r="H40" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I40" s="140"/>
-      <c r="J40" s="141"/>
+      <c r="I40" s="139"/>
+      <c r="J40" s="140"/>
       <c r="K40" s="19" t="s">
         <v>88</v>
       </c>
@@ -32209,18 +32326,18 @@
     </row>
     <row r="41" spans="2:32" s="10" customFormat="1">
       <c r="B41" s="22"/>
-      <c r="C41" s="139" t="s">
+      <c r="C41" s="144" t="s">
         <v>16</v>
       </c>
-      <c r="D41" s="140"/>
-      <c r="E41" s="140"/>
-      <c r="F41" s="140"/>
-      <c r="G41" s="141"/>
-      <c r="H41" s="146" t="s">
+      <c r="D41" s="139"/>
+      <c r="E41" s="139"/>
+      <c r="F41" s="139"/>
+      <c r="G41" s="140"/>
+      <c r="H41" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I41" s="140"/>
-      <c r="J41" s="141"/>
+      <c r="I41" s="139"/>
+      <c r="J41" s="140"/>
       <c r="K41" s="19" t="s">
         <v>89</v>
       </c>
@@ -32240,18 +32357,18 @@
     </row>
     <row r="42" spans="2:32" s="10" customFormat="1">
       <c r="B42" s="22"/>
-      <c r="C42" s="139" t="s">
+      <c r="C42" s="144" t="s">
         <v>90</v>
       </c>
-      <c r="D42" s="140"/>
-      <c r="E42" s="140"/>
-      <c r="F42" s="140"/>
-      <c r="G42" s="141"/>
-      <c r="H42" s="146" t="s">
+      <c r="D42" s="139"/>
+      <c r="E42" s="139"/>
+      <c r="F42" s="139"/>
+      <c r="G42" s="140"/>
+      <c r="H42" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I42" s="140"/>
-      <c r="J42" s="141"/>
+      <c r="I42" s="139"/>
+      <c r="J42" s="140"/>
       <c r="K42" s="19" t="s">
         <v>91</v>
       </c>
@@ -32271,18 +32388,18 @@
     </row>
     <row r="43" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B43" s="75"/>
-      <c r="C43" s="142" t="s">
+      <c r="C43" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="D43" s="137"/>
-      <c r="E43" s="137"/>
-      <c r="F43" s="137"/>
-      <c r="G43" s="138"/>
-      <c r="H43" s="136" t="s">
+      <c r="D43" s="149"/>
+      <c r="E43" s="149"/>
+      <c r="F43" s="149"/>
+      <c r="G43" s="150"/>
+      <c r="H43" s="148" t="s">
         <v>73</v>
       </c>
-      <c r="I43" s="137"/>
-      <c r="J43" s="138"/>
+      <c r="I43" s="149"/>
+      <c r="J43" s="150"/>
       <c r="K43" s="81" t="s">
         <v>92</v>
       </c>
@@ -32344,19 +32461,19 @@
       <c r="AF44" s="27"/>
     </row>
     <row r="45" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B45" s="148" t="s">
+      <c r="B45" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C45" s="144"/>
-      <c r="D45" s="144"/>
-      <c r="E45" s="144"/>
-      <c r="F45" s="144"/>
-      <c r="G45" s="149"/>
-      <c r="H45" s="159" t="s">
+      <c r="C45" s="146"/>
+      <c r="D45" s="146"/>
+      <c r="E45" s="146"/>
+      <c r="F45" s="146"/>
+      <c r="G45" s="147"/>
+      <c r="H45" s="153" t="s">
         <v>67</v>
       </c>
-      <c r="I45" s="160"/>
-      <c r="J45" s="161"/>
+      <c r="I45" s="154"/>
+      <c r="J45" s="155"/>
       <c r="K45" s="83" t="s">
         <v>68</v>
       </c>
@@ -32384,18 +32501,18 @@
     </row>
     <row r="46" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B46" s="21"/>
-      <c r="C46" s="139" t="s">
+      <c r="C46" s="144" t="s">
         <v>15</v>
       </c>
-      <c r="D46" s="140"/>
-      <c r="E46" s="140"/>
-      <c r="F46" s="140"/>
-      <c r="G46" s="141"/>
-      <c r="H46" s="150" t="s">
+      <c r="D46" s="139"/>
+      <c r="E46" s="139"/>
+      <c r="F46" s="139"/>
+      <c r="G46" s="140"/>
+      <c r="H46" s="142" t="s">
         <v>73</v>
       </c>
-      <c r="I46" s="151"/>
-      <c r="J46" s="152"/>
+      <c r="I46" s="137"/>
+      <c r="J46" s="138"/>
       <c r="K46" s="19" t="s">
         <v>93</v>
       </c>
@@ -32415,18 +32532,18 @@
     </row>
     <row r="47" spans="2:32" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B47" s="22"/>
-      <c r="C47" s="139" t="s">
+      <c r="C47" s="144" t="s">
         <v>94</v>
       </c>
-      <c r="D47" s="140"/>
-      <c r="E47" s="140"/>
-      <c r="F47" s="140"/>
-      <c r="G47" s="141"/>
-      <c r="H47" s="146" t="s">
+      <c r="D47" s="139"/>
+      <c r="E47" s="139"/>
+      <c r="F47" s="139"/>
+      <c r="G47" s="140"/>
+      <c r="H47" s="141" t="s">
         <v>81</v>
       </c>
-      <c r="I47" s="140"/>
-      <c r="J47" s="141"/>
+      <c r="I47" s="139"/>
+      <c r="J47" s="140"/>
       <c r="K47" s="19" t="s">
         <v>95</v>
       </c>
@@ -32446,14 +32563,14 @@
     </row>
     <row r="48" spans="2:32" s="10" customFormat="1">
       <c r="B48" s="22"/>
-      <c r="C48" s="140"/>
-      <c r="D48" s="140"/>
-      <c r="E48" s="140"/>
-      <c r="F48" s="140"/>
-      <c r="G48" s="141"/>
-      <c r="H48" s="158"/>
-      <c r="I48" s="140"/>
-      <c r="J48" s="141"/>
+      <c r="C48" s="139"/>
+      <c r="D48" s="139"/>
+      <c r="E48" s="139"/>
+      <c r="F48" s="139"/>
+      <c r="G48" s="140"/>
+      <c r="H48" s="143"/>
+      <c r="I48" s="139"/>
+      <c r="J48" s="140"/>
       <c r="K48" s="19" t="s">
         <v>49</v>
       </c>
@@ -32475,14 +32592,14 @@
     </row>
     <row r="49" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B49" s="22"/>
-      <c r="C49" s="140"/>
-      <c r="D49" s="140"/>
-      <c r="E49" s="140"/>
-      <c r="F49" s="140"/>
-      <c r="G49" s="141"/>
-      <c r="H49" s="158"/>
-      <c r="I49" s="140"/>
-      <c r="J49" s="141"/>
+      <c r="C49" s="139"/>
+      <c r="D49" s="139"/>
+      <c r="E49" s="139"/>
+      <c r="F49" s="139"/>
+      <c r="G49" s="140"/>
+      <c r="H49" s="143"/>
+      <c r="I49" s="139"/>
+      <c r="J49" s="140"/>
       <c r="K49" s="19" t="s">
         <v>49</v>
       </c>
@@ -32539,19 +32656,19 @@
       <c r="AG50" s="92"/>
     </row>
     <row r="51" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B51" s="148" t="s">
+      <c r="B51" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C51" s="144"/>
-      <c r="D51" s="144"/>
-      <c r="E51" s="144"/>
-      <c r="F51" s="144"/>
-      <c r="G51" s="149"/>
-      <c r="H51" s="148" t="s">
+      <c r="C51" s="146"/>
+      <c r="D51" s="146"/>
+      <c r="E51" s="146"/>
+      <c r="F51" s="146"/>
+      <c r="G51" s="147"/>
+      <c r="H51" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I51" s="144"/>
-      <c r="J51" s="149"/>
+      <c r="I51" s="146"/>
+      <c r="J51" s="147"/>
       <c r="K51" s="28" t="s">
         <v>68</v>
       </c>
@@ -32580,18 +32697,18 @@
     </row>
     <row r="52" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B52" s="21"/>
-      <c r="C52" s="139" t="s">
+      <c r="C52" s="144" t="s">
         <v>23</v>
       </c>
-      <c r="D52" s="140"/>
-      <c r="E52" s="140"/>
-      <c r="F52" s="140"/>
-      <c r="G52" s="141"/>
-      <c r="H52" s="146" t="s">
+      <c r="D52" s="139"/>
+      <c r="E52" s="139"/>
+      <c r="F52" s="139"/>
+      <c r="G52" s="140"/>
+      <c r="H52" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I52" s="140"/>
-      <c r="J52" s="141"/>
+      <c r="I52" s="139"/>
+      <c r="J52" s="140"/>
       <c r="K52" s="19" t="s">
         <v>99</v>
       </c>
@@ -32611,18 +32728,18 @@
     </row>
     <row r="53" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B53" s="22"/>
-      <c r="C53" s="139" t="s">
+      <c r="C53" s="144" t="s">
         <v>100</v>
       </c>
-      <c r="D53" s="140"/>
-      <c r="E53" s="140"/>
-      <c r="F53" s="140"/>
-      <c r="G53" s="141"/>
-      <c r="H53" s="146" t="s">
+      <c r="D53" s="139"/>
+      <c r="E53" s="139"/>
+      <c r="F53" s="139"/>
+      <c r="G53" s="140"/>
+      <c r="H53" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I53" s="140"/>
-      <c r="J53" s="141"/>
+      <c r="I53" s="139"/>
+      <c r="J53" s="140"/>
       <c r="K53" s="19" t="s">
         <v>101</v>
       </c>
@@ -32642,18 +32759,18 @@
     </row>
     <row r="54" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B54" s="75"/>
-      <c r="C54" s="142" t="s">
+      <c r="C54" s="152" t="s">
         <v>102</v>
       </c>
-      <c r="D54" s="137"/>
-      <c r="E54" s="137"/>
-      <c r="F54" s="137"/>
-      <c r="G54" s="138"/>
-      <c r="H54" s="136" t="s">
+      <c r="D54" s="149"/>
+      <c r="E54" s="149"/>
+      <c r="F54" s="149"/>
+      <c r="G54" s="150"/>
+      <c r="H54" s="148" t="s">
         <v>73</v>
       </c>
-      <c r="I54" s="137"/>
-      <c r="J54" s="138"/>
+      <c r="I54" s="149"/>
+      <c r="J54" s="150"/>
       <c r="K54" s="81" t="s">
         <v>103</v>
       </c>
@@ -32717,19 +32834,19 @@
       <c r="AG55" s="92"/>
     </row>
     <row r="56" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B56" s="148" t="s">
+      <c r="B56" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C56" s="144"/>
-      <c r="D56" s="144"/>
-      <c r="E56" s="144"/>
-      <c r="F56" s="144"/>
-      <c r="G56" s="149"/>
-      <c r="H56" s="148" t="s">
+      <c r="C56" s="146"/>
+      <c r="D56" s="146"/>
+      <c r="E56" s="146"/>
+      <c r="F56" s="146"/>
+      <c r="G56" s="147"/>
+      <c r="H56" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I56" s="144"/>
-      <c r="J56" s="149"/>
+      <c r="I56" s="146"/>
+      <c r="J56" s="147"/>
       <c r="K56" s="28" t="s">
         <v>68</v>
       </c>
@@ -32758,18 +32875,18 @@
     </row>
     <row r="57" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B57" s="21"/>
-      <c r="C57" s="139" t="s">
+      <c r="C57" s="144" t="s">
         <v>6</v>
       </c>
-      <c r="D57" s="140"/>
-      <c r="E57" s="140"/>
-      <c r="F57" s="140"/>
-      <c r="G57" s="141"/>
-      <c r="H57" s="146" t="s">
+      <c r="D57" s="139"/>
+      <c r="E57" s="139"/>
+      <c r="F57" s="139"/>
+      <c r="G57" s="140"/>
+      <c r="H57" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I57" s="140"/>
-      <c r="J57" s="141"/>
+      <c r="I57" s="139"/>
+      <c r="J57" s="140"/>
       <c r="K57" s="19" t="s">
         <v>104</v>
       </c>
@@ -32789,18 +32906,18 @@
     </row>
     <row r="58" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B58" s="22"/>
-      <c r="C58" s="139" t="s">
+      <c r="C58" s="144" t="s">
         <v>105</v>
       </c>
-      <c r="D58" s="140"/>
-      <c r="E58" s="140"/>
-      <c r="F58" s="140"/>
-      <c r="G58" s="141"/>
-      <c r="H58" s="146" t="s">
+      <c r="D58" s="139"/>
+      <c r="E58" s="139"/>
+      <c r="F58" s="139"/>
+      <c r="G58" s="140"/>
+      <c r="H58" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I58" s="140"/>
-      <c r="J58" s="141"/>
+      <c r="I58" s="139"/>
+      <c r="J58" s="140"/>
       <c r="K58" s="19" t="s">
         <v>106</v>
       </c>
@@ -32820,18 +32937,18 @@
     </row>
     <row r="59" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1">
       <c r="B59" s="22"/>
-      <c r="C59" s="139" t="s">
+      <c r="C59" s="144" t="s">
         <v>9</v>
       </c>
-      <c r="D59" s="140"/>
-      <c r="E59" s="140"/>
-      <c r="F59" s="140"/>
-      <c r="G59" s="141"/>
-      <c r="H59" s="146" t="s">
+      <c r="D59" s="139"/>
+      <c r="E59" s="139"/>
+      <c r="F59" s="139"/>
+      <c r="G59" s="140"/>
+      <c r="H59" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I59" s="140"/>
-      <c r="J59" s="141"/>
+      <c r="I59" s="139"/>
+      <c r="J59" s="140"/>
       <c r="K59" s="19" t="s">
         <v>107</v>
       </c>
@@ -32851,18 +32968,18 @@
     </row>
     <row r="60" spans="2:33" s="10" customFormat="1">
       <c r="B60" s="22"/>
-      <c r="C60" s="139" t="s">
+      <c r="C60" s="144" t="s">
         <v>108</v>
       </c>
-      <c r="D60" s="140"/>
-      <c r="E60" s="140"/>
-      <c r="F60" s="140"/>
-      <c r="G60" s="141"/>
-      <c r="H60" s="146" t="s">
+      <c r="D60" s="139"/>
+      <c r="E60" s="139"/>
+      <c r="F60" s="139"/>
+      <c r="G60" s="140"/>
+      <c r="H60" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I60" s="140"/>
-      <c r="J60" s="141"/>
+      <c r="I60" s="139"/>
+      <c r="J60" s="140"/>
       <c r="K60" s="19" t="s">
         <v>109</v>
       </c>
@@ -32882,18 +32999,18 @@
     </row>
     <row r="61" spans="2:33" s="10" customFormat="1">
       <c r="B61" s="22"/>
-      <c r="C61" s="139" t="s">
+      <c r="C61" s="144" t="s">
         <v>110</v>
       </c>
-      <c r="D61" s="140"/>
-      <c r="E61" s="140"/>
-      <c r="F61" s="140"/>
-      <c r="G61" s="141"/>
-      <c r="H61" s="146" t="s">
+      <c r="D61" s="139"/>
+      <c r="E61" s="139"/>
+      <c r="F61" s="139"/>
+      <c r="G61" s="140"/>
+      <c r="H61" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I61" s="140"/>
-      <c r="J61" s="141"/>
+      <c r="I61" s="139"/>
+      <c r="J61" s="140"/>
       <c r="K61" s="19" t="s">
         <v>111</v>
       </c>
@@ -32913,18 +33030,18 @@
     </row>
     <row r="62" spans="2:33" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="B62" s="75"/>
-      <c r="C62" s="142" t="s">
+      <c r="C62" s="152" t="s">
         <v>112</v>
       </c>
-      <c r="D62" s="137"/>
-      <c r="E62" s="137"/>
-      <c r="F62" s="137"/>
-      <c r="G62" s="138"/>
-      <c r="H62" s="136" t="s">
+      <c r="D62" s="149"/>
+      <c r="E62" s="149"/>
+      <c r="F62" s="149"/>
+      <c r="G62" s="150"/>
+      <c r="H62" s="148" t="s">
         <v>81</v>
       </c>
-      <c r="I62" s="137"/>
-      <c r="J62" s="138"/>
+      <c r="I62" s="149"/>
+      <c r="J62" s="150"/>
       <c r="K62" s="81" t="s">
         <v>113</v>
       </c>
@@ -32988,19 +33105,19 @@
       <c r="AG63" s="92"/>
     </row>
     <row r="64" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B64" s="148" t="s">
+      <c r="B64" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C64" s="144"/>
-      <c r="D64" s="144"/>
-      <c r="E64" s="144"/>
-      <c r="F64" s="144"/>
-      <c r="G64" s="149"/>
-      <c r="H64" s="148" t="s">
+      <c r="C64" s="146"/>
+      <c r="D64" s="146"/>
+      <c r="E64" s="146"/>
+      <c r="F64" s="146"/>
+      <c r="G64" s="147"/>
+      <c r="H64" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I64" s="144"/>
-      <c r="J64" s="149"/>
+      <c r="I64" s="146"/>
+      <c r="J64" s="147"/>
       <c r="K64" s="83" t="s">
         <v>68</v>
       </c>
@@ -33029,18 +33146,18 @@
     </row>
     <row r="65" spans="2:33">
       <c r="B65" s="21"/>
-      <c r="C65" s="139" t="s">
+      <c r="C65" s="144" t="s">
         <v>114</v>
       </c>
-      <c r="D65" s="147"/>
-      <c r="E65" s="147"/>
-      <c r="F65" s="147"/>
-      <c r="G65" s="141"/>
-      <c r="H65" s="150" t="s">
+      <c r="D65" s="151"/>
+      <c r="E65" s="151"/>
+      <c r="F65" s="151"/>
+      <c r="G65" s="140"/>
+      <c r="H65" s="142" t="s">
         <v>69</v>
       </c>
-      <c r="I65" s="151"/>
-      <c r="J65" s="152"/>
+      <c r="I65" s="137"/>
+      <c r="J65" s="138"/>
       <c r="K65" s="19" t="s">
         <v>115</v>
       </c>
@@ -33060,18 +33177,18 @@
     </row>
     <row r="66" spans="2:33">
       <c r="B66" s="22"/>
-      <c r="C66" s="139" t="s">
+      <c r="C66" s="144" t="s">
         <v>116</v>
       </c>
-      <c r="D66" s="147"/>
-      <c r="E66" s="147"/>
-      <c r="F66" s="147"/>
-      <c r="G66" s="141"/>
-      <c r="H66" s="146" t="s">
+      <c r="D66" s="151"/>
+      <c r="E66" s="151"/>
+      <c r="F66" s="151"/>
+      <c r="G66" s="140"/>
+      <c r="H66" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I66" s="147"/>
-      <c r="J66" s="141"/>
+      <c r="I66" s="151"/>
+      <c r="J66" s="140"/>
       <c r="K66" s="19" t="s">
         <v>117</v>
       </c>
@@ -33091,18 +33208,18 @@
     </row>
     <row r="67" spans="2:33">
       <c r="B67" s="22"/>
-      <c r="C67" s="139" t="s">
+      <c r="C67" s="144" t="s">
         <v>9</v>
       </c>
-      <c r="D67" s="147"/>
-      <c r="E67" s="147"/>
-      <c r="F67" s="147"/>
-      <c r="G67" s="141"/>
-      <c r="H67" s="146" t="s">
+      <c r="D67" s="151"/>
+      <c r="E67" s="151"/>
+      <c r="F67" s="151"/>
+      <c r="G67" s="140"/>
+      <c r="H67" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I67" s="147"/>
-      <c r="J67" s="141"/>
+      <c r="I67" s="151"/>
+      <c r="J67" s="140"/>
       <c r="K67" s="19" t="s">
         <v>118</v>
       </c>
@@ -33122,18 +33239,18 @@
     </row>
     <row r="68" spans="2:33">
       <c r="B68" s="22"/>
-      <c r="C68" s="139" t="s">
+      <c r="C68" s="144" t="s">
         <v>119</v>
       </c>
-      <c r="D68" s="147"/>
-      <c r="E68" s="147"/>
-      <c r="F68" s="147"/>
-      <c r="G68" s="141"/>
-      <c r="H68" s="146" t="s">
+      <c r="D68" s="151"/>
+      <c r="E68" s="151"/>
+      <c r="F68" s="151"/>
+      <c r="G68" s="140"/>
+      <c r="H68" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I68" s="147"/>
-      <c r="J68" s="141"/>
+      <c r="I68" s="151"/>
+      <c r="J68" s="140"/>
       <c r="K68" s="19" t="s">
         <v>120</v>
       </c>
@@ -33153,18 +33270,18 @@
     </row>
     <row r="69" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
       <c r="B69" s="75"/>
-      <c r="C69" s="142" t="s">
+      <c r="C69" s="152" t="s">
         <v>121</v>
       </c>
-      <c r="D69" s="137"/>
-      <c r="E69" s="137"/>
-      <c r="F69" s="137"/>
-      <c r="G69" s="138"/>
-      <c r="H69" s="136" t="s">
+      <c r="D69" s="149"/>
+      <c r="E69" s="149"/>
+      <c r="F69" s="149"/>
+      <c r="G69" s="150"/>
+      <c r="H69" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="I69" s="137"/>
-      <c r="J69" s="138"/>
+      <c r="I69" s="149"/>
+      <c r="J69" s="150"/>
       <c r="K69" s="81" t="s">
         <v>122</v>
       </c>
@@ -33228,19 +33345,19 @@
       <c r="AG70" s="94"/>
     </row>
     <row r="71" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B71" s="148" t="s">
+      <c r="B71" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C71" s="144"/>
-      <c r="D71" s="144"/>
-      <c r="E71" s="144"/>
-      <c r="F71" s="144"/>
-      <c r="G71" s="149"/>
-      <c r="H71" s="148" t="s">
+      <c r="C71" s="146"/>
+      <c r="D71" s="146"/>
+      <c r="E71" s="146"/>
+      <c r="F71" s="146"/>
+      <c r="G71" s="147"/>
+      <c r="H71" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I71" s="144"/>
-      <c r="J71" s="149"/>
+      <c r="I71" s="146"/>
+      <c r="J71" s="147"/>
       <c r="K71" s="83" t="s">
         <v>68</v>
       </c>
@@ -33269,18 +33386,18 @@
     </row>
     <row r="72" spans="2:33">
       <c r="B72" s="21"/>
-      <c r="C72" s="139" t="s">
+      <c r="C72" s="144" t="s">
         <v>21</v>
       </c>
-      <c r="D72" s="147"/>
-      <c r="E72" s="147"/>
-      <c r="F72" s="147"/>
-      <c r="G72" s="141"/>
-      <c r="H72" s="150" t="s">
+      <c r="D72" s="151"/>
+      <c r="E72" s="151"/>
+      <c r="F72" s="151"/>
+      <c r="G72" s="140"/>
+      <c r="H72" s="142" t="s">
         <v>69</v>
       </c>
-      <c r="I72" s="151"/>
-      <c r="J72" s="152"/>
+      <c r="I72" s="137"/>
+      <c r="J72" s="138"/>
       <c r="K72" s="19" t="s">
         <v>123</v>
       </c>
@@ -33300,18 +33417,18 @@
     </row>
     <row r="73" spans="2:33">
       <c r="B73" s="22"/>
-      <c r="C73" s="139" t="s">
+      <c r="C73" s="144" t="s">
         <v>9</v>
       </c>
-      <c r="D73" s="147"/>
-      <c r="E73" s="147"/>
-      <c r="F73" s="147"/>
-      <c r="G73" s="141"/>
-      <c r="H73" s="146" t="s">
+      <c r="D73" s="151"/>
+      <c r="E73" s="151"/>
+      <c r="F73" s="151"/>
+      <c r="G73" s="140"/>
+      <c r="H73" s="141" t="s">
         <v>69</v>
       </c>
-      <c r="I73" s="147"/>
-      <c r="J73" s="141"/>
+      <c r="I73" s="151"/>
+      <c r="J73" s="140"/>
       <c r="K73" s="19" t="s">
         <v>124</v>
       </c>
@@ -33331,18 +33448,18 @@
     </row>
     <row r="74" spans="2:33">
       <c r="B74" s="22"/>
-      <c r="C74" s="139" t="s">
+      <c r="C74" s="144" t="s">
         <v>125</v>
       </c>
-      <c r="D74" s="147"/>
-      <c r="E74" s="147"/>
-      <c r="F74" s="147"/>
-      <c r="G74" s="141"/>
-      <c r="H74" s="146" t="s">
+      <c r="D74" s="151"/>
+      <c r="E74" s="151"/>
+      <c r="F74" s="151"/>
+      <c r="G74" s="140"/>
+      <c r="H74" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="I74" s="147"/>
-      <c r="J74" s="141"/>
+      <c r="I74" s="151"/>
+      <c r="J74" s="140"/>
       <c r="K74" s="19" t="s">
         <v>126</v>
       </c>
@@ -33362,18 +33479,18 @@
     </row>
     <row r="75" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
       <c r="B75" s="75"/>
-      <c r="C75" s="142" t="s">
+      <c r="C75" s="152" t="s">
         <v>127</v>
       </c>
-      <c r="D75" s="137"/>
-      <c r="E75" s="137"/>
-      <c r="F75" s="137"/>
-      <c r="G75" s="138"/>
-      <c r="H75" s="136" t="s">
+      <c r="D75" s="149"/>
+      <c r="E75" s="149"/>
+      <c r="F75" s="149"/>
+      <c r="G75" s="150"/>
+      <c r="H75" s="148" t="s">
         <v>73</v>
       </c>
-      <c r="I75" s="137"/>
-      <c r="J75" s="138"/>
+      <c r="I75" s="149"/>
+      <c r="J75" s="150"/>
       <c r="K75" s="81" t="s">
         <v>128</v>
       </c>
@@ -33437,19 +33554,19 @@
       <c r="AG76" s="94"/>
     </row>
     <row r="77" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
-      <c r="B77" s="148" t="s">
+      <c r="B77" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C77" s="144"/>
-      <c r="D77" s="144"/>
-      <c r="E77" s="144"/>
-      <c r="F77" s="144"/>
-      <c r="G77" s="149"/>
-      <c r="H77" s="148" t="s">
+      <c r="C77" s="146"/>
+      <c r="D77" s="146"/>
+      <c r="E77" s="146"/>
+      <c r="F77" s="146"/>
+      <c r="G77" s="147"/>
+      <c r="H77" s="145" t="s">
         <v>67</v>
       </c>
-      <c r="I77" s="144"/>
-      <c r="J77" s="149"/>
+      <c r="I77" s="146"/>
+      <c r="J77" s="147"/>
       <c r="K77" s="83" t="s">
         <v>68</v>
       </c>
@@ -33478,18 +33595,18 @@
     </row>
     <row r="78" spans="2:33">
       <c r="B78" s="21"/>
-      <c r="C78" s="139" t="s">
+      <c r="C78" s="144" t="s">
         <v>19</v>
       </c>
-      <c r="D78" s="147"/>
-      <c r="E78" s="147"/>
-      <c r="F78" s="147"/>
-      <c r="G78" s="141"/>
-      <c r="H78" s="150" t="s">
+      <c r="D78" s="151"/>
+      <c r="E78" s="151"/>
+      <c r="F78" s="151"/>
+      <c r="G78" s="140"/>
+      <c r="H78" s="142" t="s">
         <v>73</v>
       </c>
-      <c r="I78" s="151"/>
-      <c r="J78" s="152"/>
+      <c r="I78" s="137"/>
+      <c r="J78" s="138"/>
       <c r="K78" s="19" t="s">
         <v>129</v>
       </c>
@@ -33509,18 +33626,18 @@
     </row>
     <row r="79" spans="2:33">
       <c r="B79" s="22"/>
-      <c r="C79" s="139" t="s">
+      <c r="C79" s="144" t="s">
         <v>130</v>
       </c>
-      <c r="D79" s="147"/>
-      <c r="E79" s="147"/>
-      <c r="F79" s="147"/>
-      <c r="G79" s="141"/>
-      <c r="H79" s="146" t="s">
+      <c r="D79" s="151"/>
+      <c r="E79" s="151"/>
+      <c r="F79" s="151"/>
+      <c r="G79" s="140"/>
+      <c r="H79" s="141" t="s">
         <v>131</v>
       </c>
-      <c r="I79" s="147"/>
-      <c r="J79" s="141"/>
+      <c r="I79" s="151"/>
+      <c r="J79" s="140"/>
       <c r="K79" s="19" t="s">
         <v>132</v>
       </c>
@@ -33540,18 +33657,18 @@
     </row>
     <row r="80" spans="2:33" ht="18.75" customHeight="1" thickBot="1">
       <c r="B80" s="75"/>
-      <c r="C80" s="142" t="s">
+      <c r="C80" s="152" t="s">
         <v>133</v>
       </c>
-      <c r="D80" s="137"/>
-      <c r="E80" s="137"/>
-      <c r="F80" s="137"/>
-      <c r="G80" s="138"/>
-      <c r="H80" s="136" t="s">
+      <c r="D80" s="149"/>
+      <c r="E80" s="149"/>
+      <c r="F80" s="149"/>
+      <c r="G80" s="150"/>
+      <c r="H80" s="148" t="s">
         <v>73</v>
       </c>
-      <c r="I80" s="137"/>
-      <c r="J80" s="138"/>
+      <c r="I80" s="149"/>
+      <c r="J80" s="150"/>
       <c r="K80" s="81" t="s">
         <v>134</v>
       </c>
@@ -33662,12 +33779,81 @@
     </row>
   </sheetData>
   <mergeCells count="97">
-    <mergeCell ref="C24:G25"/>
-    <mergeCell ref="H30:J30"/>
-    <mergeCell ref="H24:J25"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="H80:J80"/>
+    <mergeCell ref="C41:G41"/>
+    <mergeCell ref="H62:J62"/>
+    <mergeCell ref="C43:G43"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="H43:J43"/>
+    <mergeCell ref="H54:J54"/>
+    <mergeCell ref="H41:J41"/>
+    <mergeCell ref="C66:G66"/>
+    <mergeCell ref="C53:G53"/>
+    <mergeCell ref="B56:G56"/>
+    <mergeCell ref="H74:J74"/>
+    <mergeCell ref="H56:J56"/>
+    <mergeCell ref="H68:J68"/>
+    <mergeCell ref="H35:J35"/>
+    <mergeCell ref="C78:G78"/>
+    <mergeCell ref="H79:J79"/>
+    <mergeCell ref="H61:J61"/>
+    <mergeCell ref="C74:G74"/>
+    <mergeCell ref="C67:G67"/>
+    <mergeCell ref="C72:G72"/>
+    <mergeCell ref="H78:J78"/>
+    <mergeCell ref="H73:J73"/>
+    <mergeCell ref="H65:J65"/>
+    <mergeCell ref="H71:J71"/>
+    <mergeCell ref="H75:J75"/>
+    <mergeCell ref="C75:G75"/>
+    <mergeCell ref="B64:G64"/>
+    <mergeCell ref="H53:J53"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="C80:G80"/>
+    <mergeCell ref="H77:J77"/>
+    <mergeCell ref="B51:G51"/>
+    <mergeCell ref="C59:G59"/>
+    <mergeCell ref="H42:J42"/>
+    <mergeCell ref="C46:G46"/>
+    <mergeCell ref="C61:G61"/>
+    <mergeCell ref="H67:J67"/>
+    <mergeCell ref="H59:J59"/>
+    <mergeCell ref="B77:G77"/>
+    <mergeCell ref="H46:J46"/>
+    <mergeCell ref="H52:J52"/>
+    <mergeCell ref="C79:G79"/>
+    <mergeCell ref="C73:G73"/>
+    <mergeCell ref="H72:J72"/>
+    <mergeCell ref="C54:G54"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="C47:G49"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="C60:G60"/>
+    <mergeCell ref="C57:G57"/>
+    <mergeCell ref="C42:G42"/>
+    <mergeCell ref="C39:G39"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="B71:G71"/>
+    <mergeCell ref="B2:V2"/>
+    <mergeCell ref="B11:V11"/>
+    <mergeCell ref="C58:G58"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B5:V5"/>
+    <mergeCell ref="H47:J49"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="H34:J34"/>
+    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="H28:J28"/>
+    <mergeCell ref="H29:J29"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="H31:J31"/>
+    <mergeCell ref="H58:J58"/>
+    <mergeCell ref="H40:J40"/>
     <mergeCell ref="H51:J51"/>
     <mergeCell ref="H69:J69"/>
     <mergeCell ref="C29:G29"/>
@@ -33684,81 +33870,12 @@
     <mergeCell ref="C62:G62"/>
     <mergeCell ref="H32:J32"/>
     <mergeCell ref="B34:G34"/>
-    <mergeCell ref="B71:G71"/>
-    <mergeCell ref="B2:V2"/>
-    <mergeCell ref="B11:V11"/>
-    <mergeCell ref="C58:G58"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="B5:V5"/>
-    <mergeCell ref="H47:J49"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="H34:J34"/>
-    <mergeCell ref="H39:J39"/>
-    <mergeCell ref="H28:J28"/>
-    <mergeCell ref="H29:J29"/>
-    <mergeCell ref="H38:J38"/>
-    <mergeCell ref="H31:J31"/>
-    <mergeCell ref="H58:J58"/>
-    <mergeCell ref="H40:J40"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="C40:G40"/>
-    <mergeCell ref="C47:G49"/>
-    <mergeCell ref="B45:G45"/>
-    <mergeCell ref="C60:G60"/>
-    <mergeCell ref="C57:G57"/>
-    <mergeCell ref="C42:G42"/>
-    <mergeCell ref="C39:G39"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="C80:G80"/>
-    <mergeCell ref="H77:J77"/>
-    <mergeCell ref="B51:G51"/>
-    <mergeCell ref="C59:G59"/>
-    <mergeCell ref="H42:J42"/>
-    <mergeCell ref="C46:G46"/>
-    <mergeCell ref="C61:G61"/>
-    <mergeCell ref="H67:J67"/>
-    <mergeCell ref="H59:J59"/>
-    <mergeCell ref="B77:G77"/>
-    <mergeCell ref="H46:J46"/>
-    <mergeCell ref="H52:J52"/>
-    <mergeCell ref="C79:G79"/>
-    <mergeCell ref="C73:G73"/>
-    <mergeCell ref="H72:J72"/>
-    <mergeCell ref="C54:G54"/>
-    <mergeCell ref="H35:J35"/>
-    <mergeCell ref="C78:G78"/>
-    <mergeCell ref="H79:J79"/>
-    <mergeCell ref="H61:J61"/>
-    <mergeCell ref="C74:G74"/>
-    <mergeCell ref="C67:G67"/>
-    <mergeCell ref="C72:G72"/>
-    <mergeCell ref="H78:J78"/>
-    <mergeCell ref="H73:J73"/>
-    <mergeCell ref="H65:J65"/>
-    <mergeCell ref="H71:J71"/>
-    <mergeCell ref="H75:J75"/>
-    <mergeCell ref="C75:G75"/>
-    <mergeCell ref="B64:G64"/>
-    <mergeCell ref="H53:J53"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="H80:J80"/>
-    <mergeCell ref="C41:G41"/>
-    <mergeCell ref="H62:J62"/>
-    <mergeCell ref="C43:G43"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="H43:J43"/>
-    <mergeCell ref="H54:J54"/>
-    <mergeCell ref="H41:J41"/>
-    <mergeCell ref="C66:G66"/>
-    <mergeCell ref="C53:G53"/>
-    <mergeCell ref="B56:G56"/>
-    <mergeCell ref="H74:J74"/>
-    <mergeCell ref="H56:J56"/>
-    <mergeCell ref="H68:J68"/>
+    <mergeCell ref="C24:G25"/>
+    <mergeCell ref="H30:J30"/>
+    <mergeCell ref="H24:J25"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="H26:J26"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -33767,7 +33884,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H1571"/>
+  <dimension ref="A1:H1584"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="2" max="2" width="12.75" style="2" bestFit="1" customWidth="1"/>
@@ -74333,6 +74450,344 @@
       </c>
       <c r="H1571" s="130" t="s">
         <v>7730</v>
+      </c>
+    </row>
+    <row r="1572" spans="1:8">
+      <c r="A1572">
+        <v>901343</v>
+      </c>
+      <c r="B1572" s="2">
+        <v>91343</v>
+      </c>
+      <c r="C1572" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1572" s="130" t="s">
+        <v>8463</v>
+      </c>
+      <c r="E1572" s="130" t="s">
+        <v>8464</v>
+      </c>
+      <c r="F1572" s="130" t="s">
+        <v>8465</v>
+      </c>
+      <c r="G1572" s="130" t="s">
+        <v>8466</v>
+      </c>
+      <c r="H1572" s="130" t="s">
+        <v>8466</v>
+      </c>
+    </row>
+    <row r="1573" spans="1:8">
+      <c r="A1573">
+        <v>901344</v>
+      </c>
+      <c r="B1573" s="2">
+        <v>91344</v>
+      </c>
+      <c r="C1573" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1573" s="130" t="s">
+        <v>8467</v>
+      </c>
+      <c r="E1573" s="130" t="s">
+        <v>8467</v>
+      </c>
+      <c r="F1573" s="130" t="s">
+        <v>8467</v>
+      </c>
+      <c r="G1573" s="130" t="s">
+        <v>8468</v>
+      </c>
+      <c r="H1573" s="130" t="s">
+        <v>8469</v>
+      </c>
+    </row>
+    <row r="1574" spans="1:8">
+      <c r="A1574">
+        <v>901345</v>
+      </c>
+      <c r="B1574" s="2">
+        <v>91345</v>
+      </c>
+      <c r="C1574" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1574" s="130" t="s">
+        <v>8470</v>
+      </c>
+      <c r="E1574" s="130" t="s">
+        <v>8470</v>
+      </c>
+      <c r="F1574" s="130" t="s">
+        <v>8470</v>
+      </c>
+      <c r="G1574" s="130" t="s">
+        <v>8471</v>
+      </c>
+      <c r="H1574" s="130" t="s">
+        <v>8472</v>
+      </c>
+    </row>
+    <row r="1575" spans="1:8">
+      <c r="A1575">
+        <v>901346</v>
+      </c>
+      <c r="B1575" s="2">
+        <v>91346</v>
+      </c>
+      <c r="C1575" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1575" s="130" t="s">
+        <v>8473</v>
+      </c>
+      <c r="E1575" s="130" t="s">
+        <v>8473</v>
+      </c>
+      <c r="F1575" s="130" t="s">
+        <v>8473</v>
+      </c>
+      <c r="G1575" s="130" t="s">
+        <v>8474</v>
+      </c>
+      <c r="H1575" s="130" t="s">
+        <v>8475</v>
+      </c>
+    </row>
+    <row r="1576" spans="1:8">
+      <c r="A1576">
+        <v>901347</v>
+      </c>
+      <c r="B1576" s="2">
+        <v>91347</v>
+      </c>
+      <c r="C1576" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1576" s="130" t="s">
+        <v>8476</v>
+      </c>
+      <c r="E1576" s="130" t="s">
+        <v>8476</v>
+      </c>
+      <c r="F1576" s="130" t="s">
+        <v>8476</v>
+      </c>
+      <c r="G1576" s="130" t="s">
+        <v>8477</v>
+      </c>
+      <c r="H1576" s="130" t="s">
+        <v>8477</v>
+      </c>
+    </row>
+    <row r="1577" spans="1:8">
+      <c r="A1577">
+        <v>901348</v>
+      </c>
+      <c r="B1577" s="2">
+        <v>91348</v>
+      </c>
+      <c r="C1577" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1577" s="130" t="s">
+        <v>8478</v>
+      </c>
+      <c r="E1577" s="130" t="s">
+        <v>8478</v>
+      </c>
+      <c r="F1577" s="130" t="s">
+        <v>8478</v>
+      </c>
+      <c r="G1577" s="130" t="s">
+        <v>8479</v>
+      </c>
+      <c r="H1577" s="130" t="s">
+        <v>8479</v>
+      </c>
+    </row>
+    <row r="1578" spans="1:8">
+      <c r="A1578">
+        <v>901349</v>
+      </c>
+      <c r="B1578" s="2">
+        <v>91349</v>
+      </c>
+      <c r="C1578" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1578" s="130" t="s">
+        <v>8480</v>
+      </c>
+      <c r="E1578" s="130" t="s">
+        <v>8480</v>
+      </c>
+      <c r="F1578" s="130" t="s">
+        <v>8480</v>
+      </c>
+      <c r="G1578" s="130" t="s">
+        <v>8481</v>
+      </c>
+      <c r="H1578" s="130" t="s">
+        <v>8481</v>
+      </c>
+    </row>
+    <row r="1579" spans="1:8">
+      <c r="A1579">
+        <v>901350</v>
+      </c>
+      <c r="B1579" s="2">
+        <v>91350</v>
+      </c>
+      <c r="C1579" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1579" s="130" t="s">
+        <v>8482</v>
+      </c>
+      <c r="E1579" s="130" t="s">
+        <v>8482</v>
+      </c>
+      <c r="F1579" s="130" t="s">
+        <v>8483</v>
+      </c>
+      <c r="G1579" s="130" t="s">
+        <v>8484</v>
+      </c>
+      <c r="H1579" s="130" t="s">
+        <v>8485</v>
+      </c>
+    </row>
+    <row r="1580" spans="1:8">
+      <c r="A1580">
+        <v>901351</v>
+      </c>
+      <c r="B1580" s="2">
+        <v>91351</v>
+      </c>
+      <c r="C1580" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1580" s="130" t="s">
+        <v>8486</v>
+      </c>
+      <c r="E1580" s="130" t="s">
+        <v>8486</v>
+      </c>
+      <c r="F1580" s="130" t="s">
+        <v>8487</v>
+      </c>
+      <c r="G1580" s="130" t="s">
+        <v>8488</v>
+      </c>
+      <c r="H1580" s="130" t="s">
+        <v>8489</v>
+      </c>
+    </row>
+    <row r="1581" spans="1:8">
+      <c r="A1581">
+        <v>901352</v>
+      </c>
+      <c r="B1581" s="2">
+        <v>91352</v>
+      </c>
+      <c r="C1581" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1581" s="130" t="s">
+        <v>8490</v>
+      </c>
+      <c r="E1581" s="130" t="s">
+        <v>8490</v>
+      </c>
+      <c r="F1581" s="130" t="s">
+        <v>8490</v>
+      </c>
+      <c r="G1581" s="130" t="s">
+        <v>8491</v>
+      </c>
+      <c r="H1581" s="130" t="s">
+        <v>8492</v>
+      </c>
+    </row>
+    <row r="1582" spans="1:8">
+      <c r="A1582">
+        <v>901353</v>
+      </c>
+      <c r="B1582" s="2">
+        <v>91353</v>
+      </c>
+      <c r="C1582" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1582" s="130" t="s">
+        <v>8493</v>
+      </c>
+      <c r="E1582" s="130" t="s">
+        <v>8493</v>
+      </c>
+      <c r="F1582" s="130" t="s">
+        <v>8493</v>
+      </c>
+      <c r="G1582" s="130" t="s">
+        <v>8494</v>
+      </c>
+      <c r="H1582" s="130" t="s">
+        <v>8495</v>
+      </c>
+    </row>
+    <row r="1583" spans="1:8">
+      <c r="A1583">
+        <v>901354</v>
+      </c>
+      <c r="B1583" s="2">
+        <v>91354</v>
+      </c>
+      <c r="C1583" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1583" s="130" t="s">
+        <v>8496</v>
+      </c>
+      <c r="E1583" s="130" t="s">
+        <v>8496</v>
+      </c>
+      <c r="F1583" s="130" t="s">
+        <v>8496</v>
+      </c>
+      <c r="G1583" s="130" t="s">
+        <v>8497</v>
+      </c>
+      <c r="H1583" s="130" t="s">
+        <v>8498</v>
+      </c>
+    </row>
+    <row r="1584" spans="1:8">
+      <c r="A1584">
+        <v>901355</v>
+      </c>
+      <c r="B1584" s="2">
+        <v>91355</v>
+      </c>
+      <c r="C1584" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1584" s="130" t="s">
+        <v>8499</v>
+      </c>
+      <c r="E1584" s="130" t="s">
+        <v>8499</v>
+      </c>
+      <c r="F1584" s="130" t="s">
+        <v>8499</v>
+      </c>
+      <c r="G1584" s="130" t="s">
+        <v>8500</v>
+      </c>
+      <c r="H1584" s="130" t="s">
+        <v>8501</v>
       </c>
     </row>
   </sheetData>
@@ -76256,10 +76711,10 @@
       <c r="B2" s="162" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="151"/>
-      <c r="D2" s="151"/>
-      <c r="E2" s="151"/>
-      <c r="F2" s="151"/>
+      <c r="C2" s="137"/>
+      <c r="D2" s="137"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="137"/>
       <c r="G2" s="163"/>
       <c r="H2" s="11"/>
       <c r="I2" s="11"/>
@@ -76269,10 +76724,10 @@
       <c r="M2" s="165" t="s">
         <v>1</v>
       </c>
-      <c r="N2" s="144"/>
-      <c r="O2" s="144"/>
-      <c r="P2" s="144"/>
-      <c r="Q2" s="149"/>
+      <c r="N2" s="146"/>
+      <c r="O2" s="146"/>
+      <c r="P2" s="146"/>
+      <c r="Q2" s="147"/>
       <c r="R2" s="11"/>
       <c r="S2" s="11"/>
       <c r="T2" s="11"/>
@@ -76280,10 +76735,10 @@
       <c r="V2" s="165" t="s">
         <v>2</v>
       </c>
-      <c r="W2" s="144"/>
-      <c r="X2" s="144"/>
-      <c r="Y2" s="144"/>
-      <c r="Z2" s="149"/>
+      <c r="W2" s="146"/>
+      <c r="X2" s="146"/>
+      <c r="Y2" s="146"/>
+      <c r="Z2" s="147"/>
       <c r="AA2" s="11"/>
       <c r="AB2" s="11"/>
       <c r="AC2" s="10"/>
@@ -76402,10 +76857,10 @@
       <c r="V5" s="165" t="s">
         <v>10</v>
       </c>
-      <c r="W5" s="144"/>
-      <c r="X5" s="144"/>
-      <c r="Y5" s="144"/>
-      <c r="Z5" s="149"/>
+      <c r="W5" s="146"/>
+      <c r="X5" s="146"/>
+      <c r="Y5" s="146"/>
+      <c r="Z5" s="147"/>
       <c r="AA5" s="11"/>
       <c r="AB5" s="11"/>
       <c r="AC5" s="10"/>
@@ -76451,10 +76906,10 @@
       <c r="B7" s="165" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="144"/>
-      <c r="D7" s="144"/>
-      <c r="E7" s="144"/>
-      <c r="F7" s="149"/>
+      <c r="C7" s="146"/>
+      <c r="D7" s="146"/>
+      <c r="E7" s="146"/>
+      <c r="F7" s="147"/>
       <c r="G7" s="33"/>
       <c r="H7" s="33"/>
       <c r="I7" s="33"/>
@@ -76463,10 +76918,10 @@
       <c r="L7" s="165" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="144"/>
-      <c r="N7" s="144"/>
-      <c r="O7" s="144"/>
-      <c r="P7" s="149"/>
+      <c r="M7" s="146"/>
+      <c r="N7" s="146"/>
+      <c r="O7" s="146"/>
+      <c r="P7" s="147"/>
       <c r="Q7" s="11"/>
       <c r="R7" s="11"/>
       <c r="S7" s="11"/>
@@ -76675,10 +77130,10 @@
       <c r="AB14" s="164" t="s">
         <v>18</v>
       </c>
-      <c r="AC14" s="144"/>
-      <c r="AD14" s="144"/>
-      <c r="AE14" s="144"/>
-      <c r="AF14" s="149"/>
+      <c r="AC14" s="146"/>
+      <c r="AD14" s="146"/>
+      <c r="AE14" s="146"/>
+      <c r="AF14" s="147"/>
       <c r="AG14" s="100"/>
       <c r="AH14" s="45"/>
       <c r="AI14" s="12"/>
@@ -76752,10 +77207,10 @@
       <c r="AB17" s="164" t="s">
         <v>20</v>
       </c>
-      <c r="AC17" s="144"/>
-      <c r="AD17" s="144"/>
-      <c r="AE17" s="144"/>
-      <c r="AF17" s="149"/>
+      <c r="AC17" s="146"/>
+      <c r="AD17" s="146"/>
+      <c r="AE17" s="146"/>
+      <c r="AF17" s="147"/>
       <c r="AG17" s="102"/>
       <c r="AH17" s="38"/>
       <c r="AI17" s="10"/>
@@ -76873,10 +77328,10 @@
       <c r="AB21" s="164" t="s">
         <v>22</v>
       </c>
-      <c r="AC21" s="144"/>
-      <c r="AD21" s="144"/>
-      <c r="AE21" s="144"/>
-      <c r="AF21" s="149"/>
+      <c r="AC21" s="146"/>
+      <c r="AD21" s="146"/>
+      <c r="AE21" s="146"/>
+      <c r="AF21" s="147"/>
       <c r="AG21" s="116"/>
       <c r="AH21" s="117"/>
     </row>

</xml_diff>

<commit_message>
[MOD] 장식 UI 수정
</commit_message>
<xml_diff>
--- a/Assets/DB/MMM_DB_Ver.05.xlsx
+++ b/Assets/DB/MMM_DB_Ver.05.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\MoreMustMush\Assets\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{628DA6BB-EF71-4E53-9D11-D4472AADDF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{352C0B71-5F8A-4D04-AEF4-BDBED15795B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10677" uniqueCount="8373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10743" uniqueCount="8422">
   <si>
     <t>Upgrade_Table</t>
   </si>
@@ -28997,6 +28997,191 @@
   </si>
   <si>
     <t>빈 칸</t>
+  </si>
+  <si>
+    <t>아름다움 {0}점</t>
+  </si>
+  <si>
+    <t>설치형 {0}/{1}</t>
+  </si>
+  <si>
+    <t>걸이형 {0}/{1}</t>
+  </si>
+  <si>
+    <t>{0}에 놓이는 장식이 없어요</t>
+  </si>
+  <si>
+    <t>걸이형 자리가 꽉 찼어요 · 다른 장식을 빼 주세요</t>
+  </si>
+  <si>
+    <t>설치형 자리가 꽉 찼어요 · 다른 장식을 빼 주세요</t>
+  </si>
+  <si>
+    <t>{0} 세트</t>
+  </si>
+  <si>
+    <t>공방에서 제작</t>
+  </si>
+  <si>
+    <t>빼기</t>
+  </si>
+  <si>
+    <t>놓기</t>
+  </si>
+  <si>
+    <t>강화 재료 {0}</t>
+  </si>
+  <si>
+    <t>Standing {0}/{1}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>置き型 {0}/{1}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Напольное {0}/{1}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Стоячий {0}/{1}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hanging {0}/{1}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>吊り下げ型 {0}/{1}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Подвесное {0}/{1}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Підвісний {0}/{1}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>No decor goes on the {0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{0}に置ける飾りはありません</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Для зоны «{0}» нет украшений</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Для зони «{0}» немає декору</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hanging spots are full · Take one down first</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>吊り下げ型の枠がいっぱいです・ほかの飾りをはずしてください</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Места для подвесных заняты · Сначала уберите одно</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Місця для підвісних зайняті · Спершу зніміть один</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Standing spots are full · Take one down first</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>置き型の枠がいっぱいです・ほかの飾りをはずしてください</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Места для напольных заняты · Сначала уберите одно</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Місця для стоячих зайняті · Спершу зніміть один</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{0} Set</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{0}セット</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Набор: {0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Набір: {0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Craft at the Workshop</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>工房で制作</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Создай в Мастерской</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Створи в Майстерні</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Remove</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Зняти</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Place</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>置く</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Поставить</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Поставити</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Material {0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>強化材料 {0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Материал {0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Матеріал {0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -33121,7 +33306,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H1568"/>
+  <dimension ref="A1:H1579"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="2" max="2" width="12.75" style="2" bestFit="1" customWidth="1"/>
@@ -73597,6 +73782,292 @@
       </c>
       <c r="H1568" s="130" t="s">
         <v>816</v>
+      </c>
+    </row>
+    <row r="1569" spans="1:8">
+      <c r="A1569">
+        <v>901340</v>
+      </c>
+      <c r="B1569" s="2">
+        <v>91340</v>
+      </c>
+      <c r="C1569" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1569" s="130" t="s">
+        <v>8373</v>
+      </c>
+      <c r="E1569" s="130" t="s">
+        <v>6873</v>
+      </c>
+      <c r="F1569" s="130" t="s">
+        <v>7499</v>
+      </c>
+      <c r="G1569" s="130" t="s">
+        <v>7500</v>
+      </c>
+      <c r="H1569" s="130" t="s">
+        <v>7501</v>
+      </c>
+    </row>
+    <row r="1570" spans="1:8">
+      <c r="A1570">
+        <v>901341</v>
+      </c>
+      <c r="B1570" s="2">
+        <v>91341</v>
+      </c>
+      <c r="C1570" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1570" s="130" t="s">
+        <v>8374</v>
+      </c>
+      <c r="E1570" s="130" t="s">
+        <v>8384</v>
+      </c>
+      <c r="F1570" s="130" t="s">
+        <v>8385</v>
+      </c>
+      <c r="G1570" s="130" t="s">
+        <v>8386</v>
+      </c>
+      <c r="H1570" s="130" t="s">
+        <v>8387</v>
+      </c>
+    </row>
+    <row r="1571" spans="1:8">
+      <c r="A1571">
+        <v>901342</v>
+      </c>
+      <c r="B1571" s="2">
+        <v>91342</v>
+      </c>
+      <c r="C1571" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1571" s="130" t="s">
+        <v>8375</v>
+      </c>
+      <c r="E1571" s="130" t="s">
+        <v>8388</v>
+      </c>
+      <c r="F1571" s="130" t="s">
+        <v>8389</v>
+      </c>
+      <c r="G1571" s="130" t="s">
+        <v>8390</v>
+      </c>
+      <c r="H1571" s="130" t="s">
+        <v>8391</v>
+      </c>
+    </row>
+    <row r="1572" spans="1:8">
+      <c r="A1572">
+        <v>901343</v>
+      </c>
+      <c r="B1572" s="2">
+        <v>91343</v>
+      </c>
+      <c r="C1572" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1572" s="130" t="s">
+        <v>8376</v>
+      </c>
+      <c r="E1572" s="130" t="s">
+        <v>8392</v>
+      </c>
+      <c r="F1572" s="130" t="s">
+        <v>8393</v>
+      </c>
+      <c r="G1572" s="130" t="s">
+        <v>8394</v>
+      </c>
+      <c r="H1572" s="130" t="s">
+        <v>8395</v>
+      </c>
+    </row>
+    <row r="1573" spans="1:8">
+      <c r="A1573">
+        <v>901344</v>
+      </c>
+      <c r="B1573" s="2">
+        <v>91344</v>
+      </c>
+      <c r="C1573" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1573" s="130" t="s">
+        <v>8377</v>
+      </c>
+      <c r="E1573" s="130" t="s">
+        <v>8396</v>
+      </c>
+      <c r="F1573" s="130" t="s">
+        <v>8397</v>
+      </c>
+      <c r="G1573" s="130" t="s">
+        <v>8398</v>
+      </c>
+      <c r="H1573" s="130" t="s">
+        <v>8399</v>
+      </c>
+    </row>
+    <row r="1574" spans="1:8">
+      <c r="A1574">
+        <v>901345</v>
+      </c>
+      <c r="B1574" s="2">
+        <v>91345</v>
+      </c>
+      <c r="C1574" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1574" s="130" t="s">
+        <v>8378</v>
+      </c>
+      <c r="E1574" s="130" t="s">
+        <v>8400</v>
+      </c>
+      <c r="F1574" s="130" t="s">
+        <v>8401</v>
+      </c>
+      <c r="G1574" s="130" t="s">
+        <v>8402</v>
+      </c>
+      <c r="H1574" s="130" t="s">
+        <v>8403</v>
+      </c>
+    </row>
+    <row r="1575" spans="1:8">
+      <c r="A1575">
+        <v>901346</v>
+      </c>
+      <c r="B1575" s="2">
+        <v>91346</v>
+      </c>
+      <c r="C1575" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1575" s="130" t="s">
+        <v>8379</v>
+      </c>
+      <c r="E1575" s="130" t="s">
+        <v>8404</v>
+      </c>
+      <c r="F1575" s="130" t="s">
+        <v>8405</v>
+      </c>
+      <c r="G1575" s="130" t="s">
+        <v>8406</v>
+      </c>
+      <c r="H1575" s="130" t="s">
+        <v>8407</v>
+      </c>
+    </row>
+    <row r="1576" spans="1:8">
+      <c r="A1576">
+        <v>901347</v>
+      </c>
+      <c r="B1576" s="2">
+        <v>91347</v>
+      </c>
+      <c r="C1576" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1576" s="130" t="s">
+        <v>8380</v>
+      </c>
+      <c r="E1576" s="130" t="s">
+        <v>8408</v>
+      </c>
+      <c r="F1576" s="130" t="s">
+        <v>8409</v>
+      </c>
+      <c r="G1576" s="130" t="s">
+        <v>8410</v>
+      </c>
+      <c r="H1576" s="130" t="s">
+        <v>8411</v>
+      </c>
+    </row>
+    <row r="1577" spans="1:8">
+      <c r="A1577">
+        <v>901348</v>
+      </c>
+      <c r="B1577" s="2">
+        <v>91348</v>
+      </c>
+      <c r="C1577" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1577" s="130" t="s">
+        <v>8381</v>
+      </c>
+      <c r="E1577" s="130" t="s">
+        <v>8412</v>
+      </c>
+      <c r="F1577" s="130" t="s">
+        <v>7532</v>
+      </c>
+      <c r="G1577" s="130" t="s">
+        <v>7533</v>
+      </c>
+      <c r="H1577" s="130" t="s">
+        <v>8413</v>
+      </c>
+    </row>
+    <row r="1578" spans="1:8">
+      <c r="A1578">
+        <v>901349</v>
+      </c>
+      <c r="B1578" s="2">
+        <v>91349</v>
+      </c>
+      <c r="C1578" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1578" s="130" t="s">
+        <v>8382</v>
+      </c>
+      <c r="E1578" s="130" t="s">
+        <v>8414</v>
+      </c>
+      <c r="F1578" s="130" t="s">
+        <v>8415</v>
+      </c>
+      <c r="G1578" s="130" t="s">
+        <v>8416</v>
+      </c>
+      <c r="H1578" s="130" t="s">
+        <v>8417</v>
+      </c>
+    </row>
+    <row r="1579" spans="1:8">
+      <c r="A1579">
+        <v>901350</v>
+      </c>
+      <c r="B1579" s="2">
+        <v>91350</v>
+      </c>
+      <c r="C1579" t="s">
+        <v>815</v>
+      </c>
+      <c r="D1579" s="130" t="s">
+        <v>8383</v>
+      </c>
+      <c r="E1579" s="130" t="s">
+        <v>8418</v>
+      </c>
+      <c r="F1579" s="130" t="s">
+        <v>8419</v>
+      </c>
+      <c r="G1579" s="130" t="s">
+        <v>8420</v>
+      </c>
+      <c r="H1579" s="130" t="s">
+        <v>8421</v>
       </c>
     </row>
   </sheetData>

</xml_diff>